<commit_message>
new Careers and Procurement
</commit_message>
<xml_diff>
--- a/public/procurement.xlsx
+++ b/public/procurement.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lka\Desktop\ruAstro\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3435767-70AE-44CB-BCDA-F626F79F0427}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEBAEC6B-4348-4F05-8076-6D1296D931C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="140">
   <si>
     <t>№ п/п</t>
   </si>
@@ -45,24 +45,12 @@
     <t>Примечание</t>
   </si>
   <si>
-    <t>УЗНО Термостат MTK-CT0</t>
-  </si>
-  <si>
     <t>шт</t>
   </si>
   <si>
     <t>ЛГУП-6441</t>
   </si>
   <si>
-    <t>Масло индустриальное YMOIL HC-68 (200л)</t>
-  </si>
-  <si>
-    <t>ЛГУП-6488</t>
-  </si>
-  <si>
-    <t>УЗНО Счетчик Тор-50 Ха 2.833.034 1ExdIICT4 X, IP65</t>
-  </si>
-  <si>
     <t>ЛГУП-6489</t>
   </si>
   <si>
@@ -90,105 +78,12 @@
     <t>НТ00-000048</t>
   </si>
   <si>
-    <t>УЗНО Кольцо А18х1,2 ГОСТ 13942-86</t>
-  </si>
-  <si>
     <t>ЛГУП-6531</t>
   </si>
   <si>
-    <t>УЗНО Кольцо А20х1,2 ГОСТ 13940-86</t>
-  </si>
-  <si>
-    <t>УЗНО Кольцо А75 ГОСТ 13943-86 (с пазами)</t>
-  </si>
-  <si>
-    <t>УЗНО Кольцо А75х1,7 ГОСТ 13943-86_УЗНО</t>
-  </si>
-  <si>
-    <t>УЗНО Кольцо уплотнительное НТ.300.000.010.0</t>
-  </si>
-  <si>
-    <t>УЗНО Магнит D4х5 неодимовый</t>
-  </si>
-  <si>
-    <t>УЗНО Магнит МС3 ЦО 14,5/4 ТУ 3498-005-12591667-2014</t>
-  </si>
-  <si>
-    <t>УЗНО Пружина №442 НТ.110.000.007.0</t>
-  </si>
-  <si>
-    <t>УЗНО Пружина №467 НТ.200.000.029.0</t>
-  </si>
-  <si>
-    <t>УЗНО Пружина крышки НТ.200.004.003.0</t>
-  </si>
-  <si>
-    <t>УЗНО Кольцо 018-021-19-2-3 ГОСТ 9833-73</t>
-  </si>
-  <si>
-    <t>УЗНО Кольцо 014-018-25 ГОСТ 9833-73 (фторкаучук)</t>
-  </si>
-  <si>
-    <t>УЗНО 2-х вентильный клапанный блок КБ-2х40.01(M20x1,5Н,M20x1,5B; M14x1,5B)</t>
-  </si>
-  <si>
-    <t>УЗНО Кольцо 200-210-46-1-1 ГОСТ 9833-73</t>
-  </si>
-  <si>
-    <t>УЗНО Кольцо 100-106-36-2-2 ГОСТ 9833-73</t>
-  </si>
-  <si>
-    <t>УЗНО Кольцо 096-102-36-2-3 ГОСТ 9833-73</t>
-  </si>
-  <si>
-    <t>УЗНО Полиамид D70 П-12Б-20 ТУ 6-05-898-73</t>
-  </si>
-  <si>
     <t>кг</t>
   </si>
   <si>
-    <t>УЗНО Полиамид D80 П-12Б-20 ТУ 6-05-988-87</t>
-  </si>
-  <si>
-    <t>УЗНО Кольцо 080-086-36-1-6 ГОСТ 9833-73</t>
-  </si>
-  <si>
-    <t>УЗНО Кольцо 080-085-30-1-6 ГОСТ 9833-73</t>
-  </si>
-  <si>
-    <t>УЗНО Кольцо 070-076-36-2-4 ГОСТ 9833-73</t>
-  </si>
-  <si>
-    <t>УЗНО Кольцо 062-068-36-2-3 ГОСТ 9833-73</t>
-  </si>
-  <si>
-    <t>УЗНО Кольцо 060-065-30-1-6 ГОСТ 9833-73</t>
-  </si>
-  <si>
-    <t>УЗНО Кольцо 055-060-30-1-6 ГОСТ 9833-73</t>
-  </si>
-  <si>
-    <t>УЗНО Кольцо 035-041-36-2-4 ГОСТ 9833-73</t>
-  </si>
-  <si>
-    <t>УЗНО Кольцо 028-032-25-1-6 ГОСТ 9833-73</t>
-  </si>
-  <si>
-    <t>УЗНО Кольцо 020-025-30-2-4 ГОСТ 9833-73</t>
-  </si>
-  <si>
-    <t>УЗНО Паронит ПМБ 2 ГОСТ 481-80</t>
-  </si>
-  <si>
-    <t>УЗНО Паронит ПОН 2,0 ГОСТ 481-80 (кг)</t>
-  </si>
-  <si>
-    <t>УЗНО Полиамид D30 П-15Б-20  ТУ 6-05-988-87</t>
-  </si>
-  <si>
-    <t>УЗНО Полиамид D40 П-15Б-20 ТУ 6-05-988-87</t>
-  </si>
-  <si>
     <t>Кольцо уплотнительное НТ.202.003.004.0</t>
   </si>
   <si>
@@ -198,120 +93,15 @@
     <t>ЛГУП-6533</t>
   </si>
   <si>
-    <t>УЗНО Рычаг НТ.510.000.003.0 (лазер)</t>
-  </si>
-  <si>
     <t>Шибер НТ.530.000.005.0 (лазер)</t>
   </si>
   <si>
-    <t>УЗНО Труба D22х4 09Г2С</t>
-  </si>
-  <si>
-    <t>ЛГУП-6534</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D20х6 09Г2С</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D85х10 Ст.20 ГОСТ 1050-88</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D152х5 09Г2С ГОСТ 8732-78</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D14х2 09Г2С ГОСТ 8733-74</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D133х32 Ст.20 ГОСТ 8372-78</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D133х28 Ст.20 ГОСТ 8732-78</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D133х25 Ст.20 ГОСТ 8732-78</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D108х8 ГОСТ 8732-78/ 09Г2С ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D108х19 ГОСТ 8732-78/ Ст.09Г2С ГОСТ 19281-14</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D1020х16 ст.09Г2С ГОСТ 20295-85</t>
-  </si>
-  <si>
-    <t>УЗНО Труба 108х8 ст.09Г2С ГОСТ 8732-78</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D720х14 Ст.09Г2С-К50 ГОСТ 20295-85</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D89х8 Ст.35 ГОСТ 1050-80</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D89х8 ГОСТ 872-78 В 09Г2С ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D89х6 ГОСТ 8732-78/ 09Г2С ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D83х12 Ст.20 ГОСТ 1050-88</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D57х6 Ст.20 ГОСТ 1050-88</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D159х14 ГОСТ 8732-78/ Ст.09Г2С-3 ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D57х6 ГОСТ 8732-78/ 09Г2С ГОСТ 4543-2016</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D480х16 10Г2 ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D159х25 Ст.20 ГОСТ 8732-78</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D159х8 ГОСТ 8732-78/ 09Г2С ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D219х10 ГОСТ 8732-78/ 09Г2С ГОСТ 30564-98</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D32х4 Ст.09Г2С ГОСТ 8733-74</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D219х4 ГОСТ 8734-75/ Ст.В20 ГОСТ 8733-74</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D25х7 ст.10Г2 ГОСТ 8733-74</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D273х10 ГОСТ 8732-78/ 09Г2С ГОСТ 30564-98</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D273х16 Ст.09Г2С-3 ГОСТ 8731-87</t>
-  </si>
-  <si>
     <t>Клапан предохранительный СППК4р 17с25нж Ду80 Ру40</t>
   </si>
   <si>
     <t>ЛГУП-6535</t>
   </si>
   <si>
-    <t>УЗНО Задвижка ЗКЛ 50-40 ХЛ1 30лс15нж класс герм. А, исп.F ХЛ1 L=216 без КОФ</t>
-  </si>
-  <si>
-    <t>УЗНО Задвижка ЗКС 31лс77нж Ду 15 Ру 40 МПа (соединение муфтовое Rc 1/2)</t>
-  </si>
-  <si>
-    <t>УЗНО Задвижка клиновая литая ЗКЛ 80-40 УХЛ1 30лс15нж, класс герм.А (ряд 2, исп.фл.3)</t>
-  </si>
-  <si>
-    <t>УЗНО Задвижка клиновая стальная ЗКС Ду25 Ру160 УХЛ1, класс герметичности "А"</t>
-  </si>
-  <si>
     <t>ЛГУП-6540</t>
   </si>
   <si>
@@ -384,216 +174,45 @@
     <t>Шланг пескоструйный Диаметр 25х39, 40 метров, байонетное сцепление</t>
   </si>
   <si>
-    <t>УЗНО Лист S=3 Ст.20 ГОСТ 16523-97</t>
-  </si>
-  <si>
-    <t>ЛГУП-6583</t>
-  </si>
-  <si>
-    <t>УЗНО Круг D98 Ст.20 ГОСТ 1050-88</t>
-  </si>
-  <si>
-    <t>ЛГУП-6584</t>
-  </si>
-  <si>
-    <t>УЗНО дверь левая с доводчиком 1900х1000мм(полотно/коробка RAL7042)с рег вент-ми отверстием</t>
-  </si>
-  <si>
-    <t>ЛГУП-6591</t>
-  </si>
-  <si>
-    <t>УЗНО Магнит ПСМНТ.001.021.001</t>
-  </si>
-  <si>
     <t>ЛГУП-6598</t>
   </si>
   <si>
-    <t>УЗНО Мин. вата типа "URSA" П-125</t>
-  </si>
-  <si>
     <t>м3</t>
   </si>
   <si>
     <t>ЛГУП-6599</t>
   </si>
   <si>
-    <t>УЗНО Петля накладная ПН1-70 ГОСТ 5088-2005</t>
-  </si>
-  <si>
-    <t>УЗНО Плита П-А,I,М,Ш,Е1(600х450х19) ГОСТ 10632-89</t>
-  </si>
-  <si>
-    <t>УЗНО Труба профильная 50х25х4 09Г2С ГОСТ 8645-68</t>
-  </si>
-  <si>
-    <t>ЛГУП-6600</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Датчик температуры ТПС 108Exd-100/80-M20x1,5/8-C10-100M-B/-50/50-0,25-F-FECA1I-П</t>
-  </si>
-  <si>
     <t>ЛГУП-6610</t>
   </si>
   <si>
     <t>Преобразователь избыточного давления ТП-ДИП 0 ... 6МПа IP67; Exd 4-20мА+HART М20х1,5</t>
   </si>
   <si>
-    <t>УЗНО Манометр МП4 P=0..6МПа, ХЛ1 ст.защиты корпуса IP54, кл.точн. 1,0. Присоед-е: М20х1,5 - наружн</t>
-  </si>
-  <si>
-    <t>Влагомер сырой нефти ВСН-2 Ду 80, Ру 40 (угловой)</t>
-  </si>
-  <si>
-    <t>УЗНО Датчик изгибающего момента тип 108 длина крыла 64мм</t>
-  </si>
-  <si>
     <t>Термометр показывающий БТ-52.220-100-1,5-( 0...+100С) М20х1,5</t>
   </si>
   <si>
     <t>Расходомер ЭМИС-МАСС 260-Ех-80-Д-Ж-4,0 вых.сигнал частотно-импульсный, RS-485 Modbus RTU</t>
   </si>
   <si>
-    <t>УЗНО Прокладка А-150-40-А ГОСТ 15180-86</t>
-  </si>
-  <si>
-    <t>ЛГУП-6611</t>
-  </si>
-  <si>
-    <t>УЗНО Прокладка Б-80-40-ПМБ ГОСТ 15180-86</t>
-  </si>
-  <si>
-    <t>УЗНО Прокладка Б-50-40-ПМБ ГОСТ 15180-86</t>
-  </si>
-  <si>
-    <t>УЗНО Прокладка Б-450-40-ПМБ-1-2 ГОСТ 15180-86</t>
-  </si>
-  <si>
-    <t>УЗНО Смола ЭД-20 ГОСТ 10587-84</t>
-  </si>
-  <si>
     <t>ЛГУП-6612</t>
   </si>
   <si>
-    <t>УЗНО Скотч защитный термоусадочный Magnapak цвет белый, 5 см</t>
-  </si>
-  <si>
     <t>м</t>
   </si>
   <si>
-    <t>УЗНО Лента ПСУЛ 20х8/40</t>
-  </si>
-  <si>
     <t>пог. м</t>
   </si>
   <si>
-    <t>УЗНО Изолон НПЭ В 4мм несортовой ТУ 2244-020-00203474-2004</t>
-  </si>
-  <si>
-    <t>УЗНО Пленка полиэтиленовая рукав 0,3х3000 ГОСТ 10354-82</t>
-  </si>
-  <si>
-    <t>УЗНО Литол 24 /кг/</t>
-  </si>
-  <si>
-    <t>УЗНО Сетка полутомпаковая 008Н Л80 ГОСТ 6613-86</t>
-  </si>
-  <si>
-    <t>м2</t>
-  </si>
-  <si>
-    <t>УЗНО Отвердитель ПЭПА</t>
-  </si>
-  <si>
-    <t>УЗНО Герметик "Макрофлекс"  силик. универс. белый 290мл</t>
-  </si>
-  <si>
-    <t>УЗНО Герметик силиконовый универс. белый 310мл</t>
-  </si>
-  <si>
-    <t>УЗНО Емкость пластиковая 0,5л (дно плоское, форма емкости - квадрат или прямоугольник)</t>
-  </si>
-  <si>
-    <t>УЗНО Замок навесной 50мм, влагозащищенный, с заглушкой</t>
-  </si>
-  <si>
-    <t>УЗНО Лезвие для ножа профессионального для резки пленки Магнапак</t>
-  </si>
-  <si>
-    <t>УЗНО Пена монтажная "MAKROFLEX " V=1000 мл</t>
-  </si>
-  <si>
-    <t>УЗНО Пленка воздушно-пузырчатая 1500мм*100пог.м 2 сл (рул)</t>
-  </si>
-  <si>
-    <t>УЗНО Скотч 50мм*120м PROFITTO /6/54 прозрачн</t>
-  </si>
-  <si>
-    <t>УЗНО Скотч-малярный</t>
-  </si>
-  <si>
-    <t>УЗНО Стул ЗФ.6.156.005М</t>
-  </si>
-  <si>
-    <t>УЗНО Стяжка нейлон 200мм (упак)</t>
-  </si>
-  <si>
-    <t>УЗНО Хомут 4х300 пластиковый</t>
-  </si>
-  <si>
-    <t>УЗНО Ящик для техновека/нягань (габариты 1500*600*600мм)</t>
-  </si>
-  <si>
-    <t>УЗНО Ящик УОК НКТ НТ.007.094.000</t>
-  </si>
-  <si>
-    <t>УЗНО Пленка термоусадочная Magnapak белая (ширина 9,8 м, толщина 190 мкм)</t>
-  </si>
-  <si>
-    <t>УЗНО Стропа Magnapack</t>
-  </si>
-  <si>
-    <t>УЗНО Маты МБП-20-10000х1000х50</t>
-  </si>
-  <si>
-    <t>УЗНО Упаковка картонная на УРПД-3.1 405(Д)х225(Ш)х80(В) самосборная</t>
-  </si>
-  <si>
-    <t>АХУП-000302</t>
-  </si>
-  <si>
-    <t>УЗНО Заглушка 108х8-09Г2С ГОСТ 17379-2001</t>
-  </si>
-  <si>
-    <t>ЛГУП-6613</t>
-  </si>
-  <si>
-    <t>УЗНО Заглушка 89х8 ст.09Г2С ГОСТ 17379-2001</t>
-  </si>
-  <si>
     <t>Сапоги летние</t>
   </si>
   <si>
     <t>пар</t>
   </si>
   <si>
-    <t>НТ00-000049</t>
-  </si>
-  <si>
     <t>Костюм рабочий</t>
   </si>
   <si>
-    <t>УЗНО Лист профилированный С21-1000-0,7 L=1510мм RAL2008 (оранж)</t>
-  </si>
-  <si>
-    <t>ЛГУП-6618</t>
-  </si>
-  <si>
-    <t>УЗНО Труба D720х12 Ст.09Г2С ГОСТ 20295-85</t>
-  </si>
-  <si>
-    <t>ЛГУП-6620</t>
-  </si>
-  <si>
     <t>Цена</t>
   </si>
   <si>
@@ -604,6 +223,228 @@
   </si>
   <si>
     <t>ЛГУП-6622</t>
+  </si>
+  <si>
+    <t>Ботинки летние 42 р</t>
+  </si>
+  <si>
+    <t>НТУП-017701</t>
+  </si>
+  <si>
+    <t>Костюм летний от загрязнений и противоэнцефалитный</t>
+  </si>
+  <si>
+    <t>Сцепление крабовое для рукава 25-39мм</t>
+  </si>
+  <si>
+    <t>Термостат MTK-CT0</t>
+  </si>
+  <si>
+    <t>Счетчик Тор-50 Ха 2.833.034 1ExdIICT4 X, IP65</t>
+  </si>
+  <si>
+    <t>Кольцо 020-025-30-2-4 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Кольцо 080-085-30-1-6 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Кольцо 096-102-36-2-3 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Кольцо 100-106-36-2-2 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Кольцо А18х1,2 ГОСТ 13942-86</t>
+  </si>
+  <si>
+    <t>Кольцо А20х1,2 ГОСТ 13940-86</t>
+  </si>
+  <si>
+    <t>Кольцо А75 ГОСТ 13943-86 (с пазами)</t>
+  </si>
+  <si>
+    <t>2-х вентильный клапанный блок КБ-2х40.01(M20x1,5Н,M20x1,5B; M14x1,5B)</t>
+  </si>
+  <si>
+    <t>Пружина крышки НТ.200.004.003.0</t>
+  </si>
+  <si>
+    <t>Кольцо 028-032-25-1-6 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Кольцо 018-021-19-2-3 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Кольцо 014-018-25 ГОСТ 9833-73 (фторкаучук)</t>
+  </si>
+  <si>
+    <t>Кольцо 080-086-36-1-6 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Кольцо 035-041-36-2-4 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Кольцо 055-060-30-1-6 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Кольцо 060-065-30-1-6 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Кольцо 062-068-36-2-3 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Кольцо 070-076-36-2-4 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Кольцо уплотнительное НТ.300.000.010.0</t>
+  </si>
+  <si>
+    <t>Магнит D4х5 неодимовый</t>
+  </si>
+  <si>
+    <t>Магнит МС3 ЦО 14,5/4 ТУ 3498-005-12591667-2014</t>
+  </si>
+  <si>
+    <t>Пружина №442 НТ.110.000.007.0</t>
+  </si>
+  <si>
+    <t>Пружина №467 НТ.200.000.029.0</t>
+  </si>
+  <si>
+    <t>Кольцо 200-210-46-1-1 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Паронит ПМБ 2 ГОСТ 481-80</t>
+  </si>
+  <si>
+    <t>Паронит ПОН 2,0 ГОСТ 481-80 (кг)</t>
+  </si>
+  <si>
+    <t>Полиамид D80 П-12Б-20 ТУ 6-05-988-87</t>
+  </si>
+  <si>
+    <t>Полиамид D70 П-12Б-20 ТУ 6-05-898-73</t>
+  </si>
+  <si>
+    <t>Полиамид D40 П-15Б-20 ТУ 6-05-988-87</t>
+  </si>
+  <si>
+    <t>Полиамид D30 П-15Б-20  ТУ 6-05-988-87</t>
+  </si>
+  <si>
+    <t>Рычаг НТ.510.000.003.0 (лазер)</t>
+  </si>
+  <si>
+    <t>Задвижка ЗКЛ 50-40 ХЛ1 30лс15нж класс герм. А, исп.F ХЛ1 L=216 без КОФ</t>
+  </si>
+  <si>
+    <t>Задвижка ЗКС 31лс77нж Ду 15 Ру 40 МПа (соединение муфтовое Rc 1/2)</t>
+  </si>
+  <si>
+    <t>Задвижка клиновая литая ЗКЛ 80-40 УХЛ1 30лс15нж, класс герм.А (ряд 2, исп.фл.3)</t>
+  </si>
+  <si>
+    <t>Задвижка клиновая стальная ЗКС Ду25 Ру160 УХЛ1, класс герметичности "А"</t>
+  </si>
+  <si>
+    <t>Магнит ПСМНТ.001.021.001</t>
+  </si>
+  <si>
+    <t>Петля накладная ПН1-70 ГОСТ 5088-2005</t>
+  </si>
+  <si>
+    <t>Плита П-А,I,М,Ш,Е1(600х450х19) ГОСТ 10632-89</t>
+  </si>
+  <si>
+    <t>Мин. вата типа "URSA" П-125</t>
+  </si>
+  <si>
+    <t>Датчик изгибающего момента тип 108 длина крыла 64мм</t>
+  </si>
+  <si>
+    <t>Манометр МП4 P=0..6МПа, ХЛ1 ст.защиты корпуса IP54, кл.точн. 1,0. Присоед-е: М20х1,5 - наружн</t>
+  </si>
+  <si>
+    <t>Влагомер сырой нефти ВСН-2 Ду 80, Ру 40 (угловой) взрывозащ.1Ex ib IIA T6, IP67</t>
+  </si>
+  <si>
+    <t>Датчик температуры ТПС 108Exd-100/80-M20x1,5/8-C10-100M-B/-50/50-0,25-F-FECA1I-П</t>
+  </si>
+  <si>
+    <t>Изолон НПЭ В 4мм несортовой ТУ 2244-020-00203474-2004</t>
+  </si>
+  <si>
+    <t>Литол 24 /кг/</t>
+  </si>
+  <si>
+    <t>Пленка полиэтиленовая рукав 0,3х3000 ГОСТ 10354-82</t>
+  </si>
+  <si>
+    <t>Отвердитель ПЭПА</t>
+  </si>
+  <si>
+    <t>Лента ПСУЛ 20х8/40</t>
+  </si>
+  <si>
+    <t>Скотч защитный термоусадочный Magnapak цвет белый, 5 см</t>
+  </si>
+  <si>
+    <t>Смола ЭД-20 ГОСТ 10587-84</t>
+  </si>
+  <si>
+    <t>Замок навесной 50мм, влагозащищенный, с заглушкой</t>
+  </si>
+  <si>
+    <t>Лезвие для ножа профессионального для резки пленки Магнапак</t>
+  </si>
+  <si>
+    <t>Стропа Magnapack</t>
+  </si>
+  <si>
+    <t>Ящик УОК НКТ НТ.007.094.000</t>
+  </si>
+  <si>
+    <t>Ящик для техновека/нягань (габариты 1500*600*600мм)</t>
+  </si>
+  <si>
+    <t>Хомут 4х300 пластиковый</t>
+  </si>
+  <si>
+    <t>Стяжка нейлон 200мм (упак)</t>
+  </si>
+  <si>
+    <t>Стул ЗФ.6.156.005М</t>
+  </si>
+  <si>
+    <t>Скотч-малярный</t>
+  </si>
+  <si>
+    <t>Скотч 50мм*120м PROFITTO /6/54 прозрачн</t>
+  </si>
+  <si>
+    <t>Пленка воздушно-пузырчатая 1500мм*100пог.м 2 сл (рул)</t>
+  </si>
+  <si>
+    <t>Пленка термоусадочная Magnapak белая (ширина 9,8 м, толщина 190 мкм)</t>
+  </si>
+  <si>
+    <t>Маты МБП-20-10000х1000х50</t>
+  </si>
+  <si>
+    <t>Пена монтажная "MAKROFLEX " V=1000 мл</t>
+  </si>
+  <si>
+    <t>Емкость пластиковая 0,5л (дно плоское, форма емкости - квадрат или прямоугольник)</t>
+  </si>
+  <si>
+    <t>Герметик силиконовый универс. белый 310мл</t>
+  </si>
+  <si>
+    <t>Герметик "Макрофлекс"  силик. универс. белый 290мл</t>
+  </si>
+  <si>
+    <t>Кольцо А75х1,7 ГОСТ 13943-86</t>
   </si>
 </sst>
 </file>
@@ -1103,13 +944,13 @@
         <v>5</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>189</v>
+        <v>62</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>190</v>
+        <v>63</v>
       </c>
       <c r="I1" s="11" t="s">
-        <v>191</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1118,16 +959,16 @@
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="10" t="s">
-        <v>6</v>
+        <v>70</v>
       </c>
       <c r="D2" s="6">
         <v>5</v>
       </c>
       <c r="E2" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>7</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1136,16 +977,16 @@
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="10" t="s">
-        <v>9</v>
+        <v>71</v>
       </c>
       <c r="D3" s="6">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1154,16 +995,16 @@
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="10" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D4" s="6">
-        <v>8</v>
+        <v>300</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1172,16 +1013,16 @@
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="10" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="D5" s="6">
         <v>300</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1190,16 +1031,16 @@
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="10" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D6" s="6">
         <v>300</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1208,16 +1049,16 @@
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D7" s="6">
         <v>300</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1226,16 +1067,16 @@
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="6">
+        <v>50</v>
+      </c>
+      <c r="E8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="6">
-        <v>300</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>7</v>
-      </c>
       <c r="F8" s="5" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1244,16 +1085,16 @@
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="10" t="s">
-        <v>18</v>
+        <v>72</v>
       </c>
       <c r="D9" s="6">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1262,16 +1103,16 @@
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="10" t="s">
-        <v>29</v>
+        <v>73</v>
       </c>
       <c r="D10" s="6">
         <v>1</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1280,16 +1121,16 @@
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="10" t="s">
-        <v>28</v>
+        <v>84</v>
       </c>
       <c r="D11" s="6">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1298,16 +1139,16 @@
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="10" t="s">
-        <v>27</v>
+        <v>74</v>
       </c>
       <c r="D12" s="6">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1316,16 +1157,16 @@
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="10" t="s">
-        <v>26</v>
+        <v>75</v>
       </c>
       <c r="D13" s="6">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1334,16 +1175,16 @@
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="10" t="s">
-        <v>25</v>
+        <v>76</v>
       </c>
       <c r="D14" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1352,16 +1193,16 @@
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="10" t="s">
-        <v>40</v>
+        <v>77</v>
       </c>
       <c r="D15" s="6">
-        <v>0.3</v>
+        <v>2</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1370,16 +1211,16 @@
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="10" t="s">
-        <v>30</v>
+        <v>78</v>
       </c>
       <c r="D16" s="6">
         <v>1</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1388,16 +1229,16 @@
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="10" t="s">
-        <v>31</v>
+        <v>79</v>
       </c>
       <c r="D17" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1406,16 +1247,16 @@
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="10" t="s">
-        <v>35</v>
+        <v>83</v>
       </c>
       <c r="D18" s="6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1424,16 +1265,16 @@
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="10" t="s">
-        <v>43</v>
+        <v>82</v>
       </c>
       <c r="D19" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1442,16 +1283,16 @@
       </c>
       <c r="B20" s="4"/>
       <c r="C20" s="10" t="s">
-        <v>44</v>
+        <v>81</v>
       </c>
       <c r="D20" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1460,16 +1301,16 @@
       </c>
       <c r="B21" s="4"/>
       <c r="C21" s="10" t="s">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="D21" s="6">
         <v>2</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1478,16 +1319,16 @@
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="10" t="s">
-        <v>46</v>
+        <v>86</v>
       </c>
       <c r="D22" s="6">
         <v>4</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1496,16 +1337,16 @@
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="10" t="s">
-        <v>47</v>
+        <v>87</v>
       </c>
       <c r="D23" s="6">
         <v>2</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1514,16 +1355,16 @@
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="10" t="s">
-        <v>54</v>
+        <v>88</v>
       </c>
       <c r="D24" s="6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1532,16 +1373,16 @@
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="10" t="s">
-        <v>48</v>
+        <v>89</v>
       </c>
       <c r="D25" s="6">
         <v>3</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1550,16 +1391,16 @@
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="10" t="s">
-        <v>53</v>
+        <v>139</v>
       </c>
       <c r="D26" s="6">
-        <v>0.22</v>
+        <v>1</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1568,16 +1409,16 @@
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="10" t="s">
-        <v>52</v>
+        <v>90</v>
       </c>
       <c r="D27" s="6">
-        <v>0.08</v>
+        <v>2</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1586,16 +1427,16 @@
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="10" t="s">
-        <v>51</v>
+        <v>91</v>
       </c>
       <c r="D28" s="6">
-        <v>0.44400000000000001</v>
+        <v>4</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1604,16 +1445,16 @@
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="10" t="s">
-        <v>50</v>
+        <v>92</v>
       </c>
       <c r="D29" s="6">
-        <v>0.17</v>
+        <v>40</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1622,16 +1463,16 @@
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="10" t="s">
-        <v>49</v>
+        <v>93</v>
       </c>
       <c r="D30" s="6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1640,16 +1481,16 @@
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="10" t="s">
-        <v>42</v>
+        <v>94</v>
       </c>
       <c r="D31" s="6">
         <v>1</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1658,16 +1499,16 @@
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="10" t="s">
-        <v>41</v>
+        <v>80</v>
       </c>
       <c r="D32" s="6">
         <v>2</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1676,16 +1517,16 @@
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="10" t="s">
-        <v>37</v>
+        <v>95</v>
       </c>
       <c r="D33" s="6">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1694,16 +1535,16 @@
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="10" t="s">
-        <v>36</v>
+        <v>96</v>
       </c>
       <c r="D34" s="6">
-        <v>6</v>
+        <v>0.17</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1712,16 +1553,16 @@
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="10" t="s">
-        <v>21</v>
+        <v>97</v>
       </c>
       <c r="D35" s="6">
-        <v>2</v>
+        <v>0.44400000000000001</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1730,16 +1571,16 @@
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="10" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D36" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1748,16 +1589,16 @@
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="10" t="s">
-        <v>24</v>
+        <v>98</v>
       </c>
       <c r="D37" s="6">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1766,16 +1607,16 @@
       </c>
       <c r="B38" s="4"/>
       <c r="C38" s="10" t="s">
-        <v>38</v>
+        <v>99</v>
       </c>
       <c r="D38" s="6">
         <v>0.44</v>
       </c>
       <c r="E38" s="7" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1784,16 +1625,16 @@
       </c>
       <c r="B39" s="4"/>
       <c r="C39" s="10" t="s">
-        <v>34</v>
+        <v>100</v>
       </c>
       <c r="D39" s="6">
-        <v>4</v>
+        <v>0.22</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1802,16 +1643,16 @@
       </c>
       <c r="B40" s="4"/>
       <c r="C40" s="10" t="s">
-        <v>33</v>
+        <v>101</v>
       </c>
       <c r="D40" s="6">
-        <v>4</v>
+        <v>0.08</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1820,16 +1661,16 @@
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="10" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="D41" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1838,16 +1679,16 @@
       </c>
       <c r="B42" s="4"/>
       <c r="C42" s="10" t="s">
-        <v>55</v>
+        <v>102</v>
       </c>
       <c r="D42" s="6">
         <v>1</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>56</v>
+        <v>21</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1856,16 +1697,16 @@
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="10" t="s">
-        <v>58</v>
+        <v>22</v>
       </c>
       <c r="D43" s="6">
         <v>1</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>56</v>
+        <v>21</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1874,16 +1715,16 @@
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="10" t="s">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="D44" s="6">
         <v>1</v>
       </c>
       <c r="E44" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>56</v>
+        <v>24</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1892,16 +1733,16 @@
       </c>
       <c r="B45" s="4"/>
       <c r="C45" s="10" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
       <c r="D45" s="6">
-        <v>1.59</v>
+        <v>4</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1910,16 +1751,16 @@
       </c>
       <c r="B46" s="4"/>
       <c r="C46" s="10" t="s">
-        <v>72</v>
+        <v>104</v>
       </c>
       <c r="D46" s="6">
-        <v>617.29999999999995</v>
+        <v>2</v>
       </c>
       <c r="E46" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1928,16 +1769,16 @@
       </c>
       <c r="B47" s="4"/>
       <c r="C47" s="10" t="s">
-        <v>84</v>
+        <v>105</v>
       </c>
       <c r="D47" s="6">
-        <v>7.24</v>
+        <v>7</v>
       </c>
       <c r="E47" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F47" s="5" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1946,16 +1787,16 @@
       </c>
       <c r="B48" s="4"/>
       <c r="C48" s="10" t="s">
-        <v>80</v>
+        <v>106</v>
       </c>
       <c r="D48" s="6">
-        <v>36.6</v>
+        <v>1</v>
       </c>
       <c r="E48" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1964,16 +1805,16 @@
       </c>
       <c r="B49" s="4"/>
       <c r="C49" s="10" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="D49" s="6">
-        <v>39.42</v>
+        <v>3</v>
       </c>
       <c r="E49" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F49" s="5" t="s">
-        <v>60</v>
+        <v>25</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1982,16 +1823,16 @@
       </c>
       <c r="B50" s="4"/>
       <c r="C50" s="10" t="s">
-        <v>85</v>
+        <v>26</v>
       </c>
       <c r="D50" s="6">
-        <v>7.45</v>
+        <v>1</v>
       </c>
       <c r="E50" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F50" s="5" t="s">
-        <v>60</v>
+        <v>27</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2000,16 +1841,16 @@
       </c>
       <c r="B51" s="4"/>
       <c r="C51" s="10" t="s">
-        <v>86</v>
+        <v>31</v>
       </c>
       <c r="D51" s="6">
-        <v>1.36</v>
+        <v>3</v>
       </c>
       <c r="E51" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F51" s="5" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2018,16 +1859,16 @@
       </c>
       <c r="B52" s="4"/>
       <c r="C52" s="10" t="s">
-        <v>66</v>
+        <v>30</v>
       </c>
       <c r="D52" s="6">
-        <v>33.4</v>
+        <v>3</v>
       </c>
       <c r="E52" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F52" s="5" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2036,16 +1877,16 @@
       </c>
       <c r="B53" s="4"/>
       <c r="C53" s="10" t="s">
-        <v>65</v>
+        <v>28</v>
       </c>
       <c r="D53" s="6">
-        <v>18.48</v>
+        <v>3</v>
       </c>
       <c r="E53" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F53" s="5" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2054,16 +1895,16 @@
       </c>
       <c r="B54" s="4"/>
       <c r="C54" s="10" t="s">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="D54" s="6">
-        <v>1.25</v>
+        <v>3</v>
       </c>
       <c r="E54" s="7" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="F54" s="5" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
     </row>
     <row r="55" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2072,16 +1913,16 @@
       </c>
       <c r="B55" s="4"/>
       <c r="C55" s="10" t="s">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="D55" s="8">
-        <v>2.85</v>
+        <v>3</v>
       </c>
       <c r="E55" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F55" s="5" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
     </row>
     <row r="56" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2090,16 +1931,16 @@
       </c>
       <c r="B56" s="4"/>
       <c r="C56" s="10" t="s">
-        <v>78</v>
+        <v>28</v>
       </c>
       <c r="D56" s="6">
-        <v>18.91</v>
+        <v>8</v>
       </c>
       <c r="E56" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F56" s="5" t="s">
-        <v>60</v>
+        <v>35</v>
       </c>
     </row>
     <row r="57" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2108,16 +1949,16 @@
       </c>
       <c r="B57" s="4"/>
       <c r="C57" s="10" t="s">
-        <v>81</v>
+        <v>33</v>
       </c>
       <c r="D57" s="6">
-        <v>13.2</v>
+        <v>8</v>
       </c>
       <c r="E57" s="7" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="F57" s="5" t="s">
-        <v>60</v>
+        <v>35</v>
       </c>
     </row>
     <row r="58" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2126,16 +1967,16 @@
       </c>
       <c r="B58" s="4"/>
       <c r="C58" s="10" t="s">
-        <v>82</v>
+        <v>31</v>
       </c>
       <c r="D58" s="6">
-        <v>3.7</v>
+        <v>8</v>
       </c>
       <c r="E58" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F58" s="5" t="s">
-        <v>60</v>
+        <v>35</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2144,16 +1985,16 @@
       </c>
       <c r="B59" s="4"/>
       <c r="C59" s="10" t="s">
-        <v>79</v>
+        <v>30</v>
       </c>
       <c r="D59" s="6">
-        <v>66.959999999999994</v>
+        <v>16</v>
       </c>
       <c r="E59" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F59" s="5" t="s">
-        <v>60</v>
+        <v>35</v>
       </c>
     </row>
     <row r="60" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2162,16 +2003,16 @@
       </c>
       <c r="B60" s="4"/>
       <c r="C60" s="10" t="s">
-        <v>77</v>
+        <v>32</v>
       </c>
       <c r="D60" s="6">
-        <v>3.9</v>
+        <v>8</v>
       </c>
       <c r="E60" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F60" s="5" t="s">
-        <v>60</v>
+        <v>35</v>
       </c>
     </row>
     <row r="61" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2180,16 +2021,16 @@
       </c>
       <c r="B61" s="4"/>
       <c r="C61" s="10" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="D61" s="6">
-        <v>0.69</v>
+        <v>3</v>
       </c>
       <c r="E61" s="7" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="F61" s="5" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
     </row>
     <row r="62" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2198,16 +2039,16 @@
       </c>
       <c r="B62" s="4"/>
       <c r="C62" s="10" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="D62" s="6">
-        <v>167.75</v>
+        <v>3</v>
       </c>
       <c r="E62" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F62" s="5" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
     </row>
     <row r="63" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2216,16 +2057,16 @@
       </c>
       <c r="B63" s="4"/>
       <c r="C63" s="10" t="s">
-        <v>74</v>
+        <v>30</v>
       </c>
       <c r="D63" s="6">
-        <v>14.38</v>
+        <v>3</v>
       </c>
       <c r="E63" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F63" s="5" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
     </row>
     <row r="64" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2234,16 +2075,16 @@
       </c>
       <c r="B64" s="4"/>
       <c r="C64" s="10" t="s">
-        <v>73</v>
+        <v>31</v>
       </c>
       <c r="D64" s="6">
-        <v>6.45</v>
+        <v>3</v>
       </c>
       <c r="E64" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F64" s="5" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
     </row>
     <row r="65" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2252,16 +2093,16 @@
       </c>
       <c r="B65" s="4"/>
       <c r="C65" s="10" t="s">
-        <v>62</v>
+        <v>38</v>
       </c>
       <c r="D65" s="6">
-        <v>0.56999999999999995</v>
+        <v>3</v>
       </c>
       <c r="E65" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F65" s="5" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
     </row>
     <row r="66" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2270,16 +2111,16 @@
       </c>
       <c r="B66" s="4"/>
       <c r="C66" s="10" t="s">
-        <v>87</v>
+        <v>32</v>
       </c>
       <c r="D66" s="6">
-        <v>12.88</v>
+        <v>3</v>
       </c>
       <c r="E66" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F66" s="5" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
     </row>
     <row r="67" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2288,16 +2129,16 @@
       </c>
       <c r="B67" s="4"/>
       <c r="C67" s="10" t="s">
-        <v>61</v>
+        <v>37</v>
       </c>
       <c r="D67" s="6">
-        <v>0.68</v>
+        <v>3</v>
       </c>
       <c r="E67" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F67" s="5" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
     </row>
     <row r="68" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2306,16 +2147,16 @@
       </c>
       <c r="B68" s="4"/>
       <c r="C68" s="10" t="s">
-        <v>71</v>
+        <v>33</v>
       </c>
       <c r="D68" s="6">
-        <v>32.19</v>
+        <v>1</v>
       </c>
       <c r="E68" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F68" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="F68" s="5" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="69" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2324,16 +2165,16 @@
       </c>
       <c r="B69" s="4"/>
       <c r="C69" s="10" t="s">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="D69" s="6">
-        <v>1144.9100000000001</v>
+        <v>2</v>
       </c>
       <c r="E69" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="F69" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="F69" s="5" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="70" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2342,16 +2183,16 @@
       </c>
       <c r="B70" s="4"/>
       <c r="C70" s="10" t="s">
-        <v>69</v>
+        <v>31</v>
       </c>
       <c r="D70" s="6">
-        <v>3.32</v>
+        <v>1</v>
       </c>
       <c r="E70" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="F70" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="F70" s="5" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="71" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2360,16 +2201,16 @@
       </c>
       <c r="B71" s="4"/>
       <c r="C71" s="10" t="s">
-        <v>68</v>
+        <v>28</v>
       </c>
       <c r="D71" s="6">
-        <v>14.12</v>
+        <v>1</v>
       </c>
       <c r="E71" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="F71" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="F71" s="5" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="72" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2378,16 +2219,16 @@
       </c>
       <c r="B72" s="4"/>
       <c r="C72" s="10" t="s">
-        <v>67</v>
+        <v>32</v>
       </c>
       <c r="D72" s="6">
-        <v>2.9</v>
+        <v>1</v>
       </c>
       <c r="E72" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="F72" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="F72" s="5" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="73" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2396,16 +2237,16 @@
       </c>
       <c r="B73" s="4"/>
       <c r="C73" s="10" t="s">
-        <v>88</v>
+        <v>40</v>
       </c>
       <c r="D73" s="6">
-        <v>44.31</v>
+        <v>2</v>
       </c>
       <c r="E73" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F73" s="5" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
     </row>
     <row r="74" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2414,16 +2255,16 @@
       </c>
       <c r="B74" s="4"/>
       <c r="C74" s="10" t="s">
-        <v>94</v>
+        <v>42</v>
       </c>
       <c r="D74" s="6">
         <v>1</v>
       </c>
       <c r="E74" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F74" s="5" t="s">
-        <v>90</v>
+        <v>41</v>
       </c>
     </row>
     <row r="75" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2432,16 +2273,16 @@
       </c>
       <c r="B75" s="4"/>
       <c r="C75" s="10" t="s">
-        <v>93</v>
+        <v>43</v>
       </c>
       <c r="D75" s="6">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E75" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F75" s="5" t="s">
-        <v>90</v>
+        <v>41</v>
       </c>
     </row>
     <row r="76" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2450,16 +2291,16 @@
       </c>
       <c r="B76" s="4"/>
       <c r="C76" s="10" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="D76" s="6">
         <v>2</v>
       </c>
       <c r="E76" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F76" s="5" t="s">
-        <v>90</v>
+        <v>41</v>
       </c>
     </row>
     <row r="77" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2468,16 +2309,16 @@
       </c>
       <c r="B77" s="4"/>
       <c r="C77" s="10" t="s">
-        <v>89</v>
+        <v>45</v>
       </c>
       <c r="D77" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E77" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F77" s="5" t="s">
-        <v>90</v>
+        <v>41</v>
       </c>
     </row>
     <row r="78" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2486,16 +2327,16 @@
       </c>
       <c r="B78" s="4"/>
       <c r="C78" s="10" t="s">
-        <v>91</v>
+        <v>69</v>
       </c>
       <c r="D78" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E78" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F78" s="5" t="s">
-        <v>90</v>
+        <v>41</v>
       </c>
     </row>
     <row r="79" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2504,16 +2345,16 @@
       </c>
       <c r="B79" s="4"/>
       <c r="C79" s="10" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
       <c r="D79" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E79" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F79" s="5" t="s">
-        <v>95</v>
+        <v>41</v>
       </c>
     </row>
     <row r="80" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2522,16 +2363,16 @@
       </c>
       <c r="B80" s="4"/>
       <c r="C80" s="10" t="s">
-        <v>96</v>
+        <v>47</v>
       </c>
       <c r="D80" s="6">
         <v>1</v>
       </c>
       <c r="E80" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F80" s="5" t="s">
-        <v>97</v>
+        <v>41</v>
       </c>
     </row>
     <row r="81" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2540,16 +2381,16 @@
       </c>
       <c r="B81" s="4"/>
       <c r="C81" s="10" t="s">
-        <v>102</v>
+        <v>46</v>
       </c>
       <c r="D81" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E81" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F81" s="5" t="s">
-        <v>99</v>
+        <v>41</v>
       </c>
     </row>
     <row r="82" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2558,16 +2399,16 @@
       </c>
       <c r="B82" s="4"/>
       <c r="C82" s="10" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="D82" s="6">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E82" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F82" s="5" t="s">
-        <v>99</v>
+        <v>49</v>
       </c>
     </row>
     <row r="83" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2576,16 +2417,16 @@
       </c>
       <c r="B83" s="4"/>
       <c r="C83" s="10" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="D83" s="6">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="E83" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F83" s="5" t="s">
-        <v>99</v>
+        <v>51</v>
       </c>
     </row>
     <row r="84" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2594,16 +2435,16 @@
       </c>
       <c r="B84" s="4"/>
       <c r="C84" s="10" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="D84" s="6">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E84" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F84" s="5" t="s">
-        <v>99</v>
+        <v>51</v>
       </c>
     </row>
     <row r="85" spans="1:6" ht="10.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2612,16 +2453,16 @@
       </c>
       <c r="B85" s="4"/>
       <c r="C85" s="10" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="D85" s="6">
-        <v>3</v>
+        <v>11.52</v>
       </c>
       <c r="E85" s="7" t="s">
-        <v>104</v>
+        <v>50</v>
       </c>
       <c r="F85" s="5" t="s">
-        <v>99</v>
+        <v>51</v>
       </c>
     </row>
     <row r="86" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2630,16 +2471,16 @@
       </c>
       <c r="B86" s="4"/>
       <c r="C86" s="10" t="s">
-        <v>100</v>
+        <v>54</v>
       </c>
       <c r="D86" s="6">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="E86" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F86" s="5" t="s">
-        <v>105</v>
+        <v>52</v>
       </c>
     </row>
     <row r="87" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2648,16 +2489,16 @@
       </c>
       <c r="B87" s="4"/>
       <c r="C87" s="10" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="D87" s="6">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E87" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F87" s="5" t="s">
-        <v>105</v>
+        <v>52</v>
       </c>
     </row>
     <row r="88" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2666,16 +2507,16 @@
       </c>
       <c r="B88" s="4"/>
       <c r="C88" s="10" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="D88" s="6">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E88" s="7" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="F88" s="5" t="s">
-        <v>105</v>
+        <v>52</v>
       </c>
     </row>
     <row r="89" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2684,16 +2525,16 @@
       </c>
       <c r="B89" s="4"/>
       <c r="C89" s="10" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="D89" s="6">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E89" s="7" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="F89" s="5" t="s">
-        <v>105</v>
+        <v>52</v>
       </c>
     </row>
     <row r="90" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2702,16 +2543,16 @@
       </c>
       <c r="B90" s="4"/>
       <c r="C90" s="10" t="s">
-        <v>103</v>
+        <v>55</v>
       </c>
       <c r="D90" s="6">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E90" s="7" t="s">
-        <v>104</v>
+        <v>6</v>
       </c>
       <c r="F90" s="5" t="s">
-        <v>105</v>
+        <v>52</v>
       </c>
     </row>
     <row r="91" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2720,16 +2561,16 @@
       </c>
       <c r="B91" s="4"/>
       <c r="C91" s="10" t="s">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="D91" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E91" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F91" s="5" t="s">
-        <v>106</v>
+        <v>52</v>
       </c>
     </row>
     <row r="92" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2738,16 +2579,16 @@
       </c>
       <c r="B92" s="4"/>
       <c r="C92" s="10" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="D92" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E92" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F92" s="5" t="s">
-        <v>106</v>
+        <v>52</v>
       </c>
     </row>
     <row r="93" spans="1:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -2756,16 +2597,16 @@
       </c>
       <c r="B93" s="4"/>
       <c r="C93" s="10" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="D93" s="6">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="E93" s="7" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="F93" s="5" t="s">
-        <v>106</v>
+        <v>56</v>
       </c>
     </row>
     <row r="94" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2774,16 +2615,16 @@
       </c>
       <c r="B94" s="4"/>
       <c r="C94" s="10" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="D94" s="6">
-        <v>3</v>
+        <v>0.13</v>
       </c>
       <c r="E94" s="7" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="F94" s="5" t="s">
-        <v>106</v>
+        <v>56</v>
       </c>
     </row>
     <row r="95" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2792,16 +2633,16 @@
       </c>
       <c r="B95" s="4"/>
       <c r="C95" s="10" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="D95" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E95" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F95" s="5" t="s">
-        <v>106</v>
+        <v>56</v>
       </c>
     </row>
     <row r="96" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2810,16 +2651,16 @@
       </c>
       <c r="B96" s="4"/>
       <c r="C96" s="10" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="D96" s="6">
-        <v>3</v>
+        <v>2E-3</v>
       </c>
       <c r="E96" s="7" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="F96" s="5" t="s">
-        <v>106</v>
+        <v>56</v>
       </c>
     </row>
     <row r="97" spans="1:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -2828,16 +2669,16 @@
       </c>
       <c r="B97" s="4"/>
       <c r="C97" s="10" t="s">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="D97" s="6">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="E97" s="7" t="s">
-        <v>104</v>
+        <v>58</v>
       </c>
       <c r="F97" s="5" t="s">
-        <v>106</v>
+        <v>56</v>
       </c>
     </row>
     <row r="98" spans="1:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -2846,16 +2687,16 @@
       </c>
       <c r="B98" s="4"/>
       <c r="C98" s="10" t="s">
-        <v>102</v>
+        <v>120</v>
       </c>
       <c r="D98" s="6">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="E98" s="7" t="s">
-        <v>7</v>
+        <v>57</v>
       </c>
       <c r="F98" s="5" t="s">
-        <v>109</v>
+        <v>56</v>
       </c>
     </row>
     <row r="99" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2864,16 +2705,16 @@
       </c>
       <c r="B99" s="4"/>
       <c r="C99" s="10" t="s">
-        <v>101</v>
+        <v>121</v>
       </c>
       <c r="D99" s="6">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="E99" s="7" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="F99" s="5" t="s">
-        <v>109</v>
+        <v>56</v>
       </c>
     </row>
     <row r="100" spans="1:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -2882,16 +2723,16 @@
       </c>
       <c r="B100" s="4"/>
       <c r="C100" s="10" t="s">
-        <v>98</v>
+        <v>122</v>
       </c>
       <c r="D100" s="6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E100" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F100" s="5" t="s">
-        <v>109</v>
+        <v>56</v>
       </c>
     </row>
     <row r="101" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2900,16 +2741,16 @@
       </c>
       <c r="B101" s="4"/>
       <c r="C101" s="10" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="D101" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E101" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F101" s="5" t="s">
-        <v>109</v>
+        <v>56</v>
       </c>
     </row>
     <row r="102" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2918,16 +2759,16 @@
       </c>
       <c r="B102" s="4"/>
       <c r="C102" s="10" t="s">
-        <v>103</v>
+        <v>124</v>
       </c>
       <c r="D102" s="6">
-        <v>1</v>
+        <v>63</v>
       </c>
       <c r="E102" s="7" t="s">
-        <v>104</v>
+        <v>57</v>
       </c>
       <c r="F102" s="5" t="s">
-        <v>109</v>
+        <v>56</v>
       </c>
     </row>
     <row r="103" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2936,34 +2777,34 @@
       </c>
       <c r="B103" s="4"/>
       <c r="C103" s="10" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="D103" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E103" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F103" s="5" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="3">
         <v>103</v>
       </c>
       <c r="B104" s="4"/>
       <c r="C104" s="10" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="D104" s="6">
         <v>1</v>
       </c>
       <c r="E104" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F104" s="5" t="s">
-        <v>111</v>
+        <v>56</v>
       </c>
     </row>
     <row r="105" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2972,16 +2813,16 @@
       </c>
       <c r="B105" s="4"/>
       <c r="C105" s="10" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="D105" s="6">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="E105" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F105" s="5" t="s">
-        <v>111</v>
+        <v>56</v>
       </c>
     </row>
     <row r="106" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2990,16 +2831,16 @@
       </c>
       <c r="B106" s="4"/>
       <c r="C106" s="10" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="D106" s="6">
         <v>2</v>
       </c>
       <c r="E106" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F106" s="5" t="s">
-        <v>111</v>
+        <v>56</v>
       </c>
     </row>
     <row r="107" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3008,16 +2849,16 @@
       </c>
       <c r="B107" s="4"/>
       <c r="C107" s="10" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
       <c r="D107" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E107" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F107" s="5" t="s">
-        <v>111</v>
+        <v>56</v>
       </c>
     </row>
     <row r="108" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3026,16 +2867,16 @@
       </c>
       <c r="B108" s="4"/>
       <c r="C108" s="10" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
       <c r="D108" s="6">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E108" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F108" s="5" t="s">
-        <v>111</v>
+        <v>56</v>
       </c>
     </row>
     <row r="109" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3044,16 +2885,16 @@
       </c>
       <c r="B109" s="4"/>
       <c r="C109" s="10" t="s">
-        <v>112</v>
+        <v>131</v>
       </c>
       <c r="D109" s="6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E109" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F109" s="5" t="s">
-        <v>111</v>
+        <v>56</v>
       </c>
     </row>
     <row r="110" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3062,16 +2903,16 @@
       </c>
       <c r="B110" s="4"/>
       <c r="C110" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D110" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E110" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F110" s="5" t="s">
-        <v>111</v>
+        <v>56</v>
       </c>
     </row>
     <row r="111" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3080,16 +2921,16 @@
       </c>
       <c r="B111" s="4"/>
       <c r="C111" s="10" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="D111" s="6">
-        <v>1.71</v>
+        <v>1</v>
       </c>
       <c r="E111" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F111" s="5" t="s">
-        <v>120</v>
+        <v>56</v>
       </c>
     </row>
     <row r="112" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.2">
@@ -3098,16 +2939,16 @@
       </c>
       <c r="B112" s="4"/>
       <c r="C112" s="10" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="D112" s="6">
-        <v>11.6</v>
+        <v>2</v>
       </c>
       <c r="E112" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F112" s="5" t="s">
-        <v>122</v>
+        <v>56</v>
       </c>
     </row>
     <row r="113" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3116,16 +2957,16 @@
       </c>
       <c r="B113" s="4"/>
       <c r="C113" s="10" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="D113" s="6">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E113" s="7" t="s">
-        <v>7</v>
+        <v>57</v>
       </c>
       <c r="F113" s="5" t="s">
-        <v>124</v>
+        <v>56</v>
       </c>
     </row>
     <row r="114" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3134,16 +2975,16 @@
       </c>
       <c r="B114" s="4"/>
       <c r="C114" s="10" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="D114" s="6">
-        <v>8</v>
+        <v>4.0199999999999996</v>
       </c>
       <c r="E114" s="7" t="s">
-        <v>7</v>
+        <v>50</v>
       </c>
       <c r="F114" s="5" t="s">
-        <v>126</v>
+        <v>56</v>
       </c>
     </row>
     <row r="115" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3152,16 +2993,16 @@
       </c>
       <c r="B115" s="4"/>
       <c r="C115" s="10" t="s">
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="D115" s="6">
-        <v>16</v>
+        <v>1.44</v>
       </c>
       <c r="E115" s="7" t="s">
-        <v>7</v>
+        <v>50</v>
       </c>
       <c r="F115" s="5" t="s">
-        <v>129</v>
+        <v>56</v>
       </c>
     </row>
     <row r="116" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3170,16 +3011,16 @@
       </c>
       <c r="B116" s="4"/>
       <c r="C116" s="10" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="D116" s="6">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E116" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F116" s="5" t="s">
-        <v>129</v>
+        <v>56</v>
       </c>
     </row>
     <row r="117" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3188,16 +3029,16 @@
       </c>
       <c r="B117" s="4"/>
       <c r="C117" s="10" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="D117" s="6">
-        <v>11.52</v>
+        <v>1</v>
       </c>
       <c r="E117" s="7" t="s">
-        <v>128</v>
+        <v>6</v>
       </c>
       <c r="F117" s="5" t="s">
-        <v>129</v>
+        <v>56</v>
       </c>
     </row>
     <row r="118" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3206,16 +3047,16 @@
       </c>
       <c r="B118" s="4"/>
       <c r="C118" s="10" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="D118" s="6">
-        <v>235.28</v>
+        <v>1</v>
       </c>
       <c r="E118" s="7" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="F118" s="5" t="s">
-        <v>133</v>
+        <v>56</v>
       </c>
     </row>
     <row r="119" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3227,13 +3068,13 @@
         <v>138</v>
       </c>
       <c r="D119" s="6">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E119" s="7" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="F119" s="5" t="s">
-        <v>135</v>
+        <v>56</v>
       </c>
     </row>
     <row r="120" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3242,16 +3083,16 @@
       </c>
       <c r="B120" s="4"/>
       <c r="C120" s="10" t="s">
-        <v>137</v>
+        <v>61</v>
       </c>
       <c r="D120" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E120" s="7" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F120" s="5" t="s">
-        <v>135</v>
+        <v>65</v>
       </c>
     </row>
     <row r="121" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3260,16 +3101,16 @@
       </c>
       <c r="B121" s="4"/>
       <c r="C121" s="10" t="s">
-        <v>141</v>
+        <v>59</v>
       </c>
       <c r="D121" s="6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E121" s="7" t="s">
-        <v>7</v>
+        <v>60</v>
       </c>
       <c r="F121" s="5" t="s">
-        <v>135</v>
+        <v>65</v>
       </c>
     </row>
     <row r="122" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3278,16 +3119,16 @@
       </c>
       <c r="B122" s="4"/>
       <c r="C122" s="10" t="s">
-        <v>136</v>
+        <v>66</v>
       </c>
       <c r="D122" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E122" s="7" t="s">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="F122" s="5" t="s">
-        <v>135</v>
+        <v>67</v>
       </c>
     </row>
     <row r="123" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3296,16 +3137,16 @@
       </c>
       <c r="B123" s="4"/>
       <c r="C123" s="10" t="s">
-        <v>134</v>
+        <v>66</v>
       </c>
       <c r="D123" s="6">
         <v>1</v>
       </c>
       <c r="E123" s="7" t="s">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="F123" s="5" t="s">
-        <v>135</v>
+        <v>67</v>
       </c>
     </row>
     <row r="124" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3314,16 +3155,16 @@
       </c>
       <c r="B124" s="4"/>
       <c r="C124" s="10" t="s">
-        <v>140</v>
+        <v>68</v>
       </c>
       <c r="D124" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E124" s="7" t="s">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="F124" s="5" t="s">
-        <v>135</v>
+        <v>67</v>
       </c>
     </row>
     <row r="125" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3332,827 +3173,377 @@
       </c>
       <c r="B125" s="4"/>
       <c r="C125" s="10" t="s">
-        <v>139</v>
+        <v>68</v>
       </c>
       <c r="D125" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E125" s="7" t="s">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="F125" s="5" t="s">
-        <v>135</v>
+        <v>67</v>
       </c>
     </row>
     <row r="126" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A126" s="3">
-        <v>125</v>
-      </c>
+      <c r="A126" s="3"/>
       <c r="B126" s="4"/>
-      <c r="C126" s="10" t="s">
-        <v>146</v>
-      </c>
-      <c r="D126" s="6">
-        <v>3</v>
-      </c>
-      <c r="E126" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F126" s="5" t="s">
-        <v>143</v>
-      </c>
+      <c r="C126" s="10"/>
+      <c r="D126" s="6"/>
+      <c r="E126" s="7"/>
+      <c r="F126" s="5"/>
     </row>
     <row r="127" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A127" s="3">
-        <v>126</v>
-      </c>
+      <c r="A127" s="3"/>
       <c r="B127" s="4"/>
-      <c r="C127" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="D127" s="6">
-        <v>1</v>
-      </c>
-      <c r="E127" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F127" s="5" t="s">
-        <v>143</v>
-      </c>
+      <c r="C127" s="10"/>
+      <c r="D127" s="6"/>
+      <c r="E127" s="7"/>
+      <c r="F127" s="5"/>
     </row>
     <row r="128" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A128" s="3">
-        <v>127</v>
-      </c>
+      <c r="A128" s="3"/>
       <c r="B128" s="4"/>
-      <c r="C128" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="D128" s="6">
-        <v>17</v>
-      </c>
-      <c r="E128" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F128" s="5" t="s">
-        <v>143</v>
-      </c>
+      <c r="C128" s="10"/>
+      <c r="D128" s="6"/>
+      <c r="E128" s="7"/>
+      <c r="F128" s="5"/>
     </row>
     <row r="129" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A129" s="3">
-        <v>128</v>
-      </c>
+      <c r="A129" s="3"/>
       <c r="B129" s="4"/>
-      <c r="C129" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="D129" s="6">
-        <v>22</v>
-      </c>
-      <c r="E129" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F129" s="5" t="s">
-        <v>143</v>
-      </c>
+      <c r="C129" s="10"/>
+      <c r="D129" s="6"/>
+      <c r="E129" s="7"/>
+      <c r="F129" s="5"/>
     </row>
     <row r="130" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A130" s="3">
-        <v>129</v>
-      </c>
+      <c r="A130" s="3"/>
       <c r="B130" s="4"/>
-      <c r="C130" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="D130" s="6">
-        <v>1</v>
-      </c>
-      <c r="E130" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F130" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C130" s="10"/>
+      <c r="D130" s="6"/>
+      <c r="E130" s="7"/>
+      <c r="F130" s="5"/>
     </row>
     <row r="131" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A131" s="3">
-        <v>130</v>
-      </c>
+      <c r="A131" s="3"/>
       <c r="B131" s="4"/>
-      <c r="C131" s="10" t="s">
-        <v>156</v>
-      </c>
-      <c r="D131" s="6">
-        <v>2.1999999999999999E-2</v>
-      </c>
-      <c r="E131" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="F131" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C131" s="10"/>
+      <c r="D131" s="6"/>
+      <c r="E131" s="7"/>
+      <c r="F131" s="5"/>
     </row>
     <row r="132" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A132" s="3">
-        <v>131</v>
-      </c>
+      <c r="A132" s="3"/>
       <c r="B132" s="4"/>
-      <c r="C132" s="10" t="s">
-        <v>160</v>
-      </c>
-      <c r="D132" s="6">
-        <v>1</v>
-      </c>
-      <c r="E132" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F132" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C132" s="10"/>
+      <c r="D132" s="6"/>
+      <c r="E132" s="7"/>
+      <c r="F132" s="5"/>
     </row>
     <row r="133" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A133" s="3">
-        <v>132</v>
-      </c>
+      <c r="A133" s="3"/>
       <c r="B133" s="4"/>
-      <c r="C133" s="10" t="s">
-        <v>159</v>
-      </c>
-      <c r="D133" s="6">
-        <v>6</v>
-      </c>
-      <c r="E133" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F133" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C133" s="10"/>
+      <c r="D133" s="6"/>
+      <c r="E133" s="7"/>
+      <c r="F133" s="5"/>
     </row>
     <row r="134" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A134" s="3">
-        <v>133</v>
-      </c>
+      <c r="A134" s="3"/>
       <c r="B134" s="4"/>
-      <c r="C134" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="D134" s="6">
-        <v>1</v>
-      </c>
-      <c r="E134" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F134" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C134" s="10"/>
+      <c r="D134" s="6"/>
+      <c r="E134" s="7"/>
+      <c r="F134" s="5"/>
     </row>
     <row r="135" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A135" s="3">
-        <v>134</v>
-      </c>
+      <c r="A135" s="3"/>
       <c r="B135" s="4"/>
-      <c r="C135" s="10" t="s">
-        <v>153</v>
-      </c>
-      <c r="D135" s="6">
-        <v>3.5</v>
-      </c>
-      <c r="E135" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F135" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C135" s="10"/>
+      <c r="D135" s="6"/>
+      <c r="E135" s="7"/>
+      <c r="F135" s="5"/>
     </row>
     <row r="136" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A136" s="3">
-        <v>135</v>
-      </c>
+      <c r="A136" s="3"/>
       <c r="B136" s="4"/>
-      <c r="C136" s="10" t="s">
-        <v>155</v>
-      </c>
-      <c r="D136" s="6">
-        <v>0.13</v>
-      </c>
-      <c r="E136" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F136" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C136" s="10"/>
+      <c r="D136" s="6"/>
+      <c r="E136" s="7"/>
+      <c r="F136" s="5"/>
     </row>
     <row r="137" spans="1:6" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A137" s="3">
-        <v>136</v>
-      </c>
+      <c r="A137" s="3"/>
       <c r="B137" s="4"/>
-      <c r="C137" s="10" t="s">
-        <v>151</v>
-      </c>
-      <c r="D137" s="6">
-        <v>36</v>
-      </c>
-      <c r="E137" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="F137" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C137" s="10"/>
+      <c r="D137" s="6"/>
+      <c r="E137" s="7"/>
+      <c r="F137" s="5"/>
     </row>
     <row r="138" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A138" s="3">
-        <v>137</v>
-      </c>
+      <c r="A138" s="3"/>
       <c r="B138" s="4"/>
-      <c r="C138" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="D138" s="6">
-        <v>38</v>
-      </c>
-      <c r="E138" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="F138" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C138" s="10"/>
+      <c r="D138" s="6"/>
+      <c r="E138" s="7"/>
+      <c r="F138" s="5"/>
     </row>
     <row r="139" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A139" s="3">
-        <v>138</v>
-      </c>
+      <c r="A139" s="3"/>
       <c r="B139" s="4"/>
-      <c r="C139" s="10" t="s">
-        <v>158</v>
-      </c>
-      <c r="D139" s="6">
-        <v>2E-3</v>
-      </c>
-      <c r="E139" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F139" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C139" s="10"/>
+      <c r="D139" s="6"/>
+      <c r="E139" s="7"/>
+      <c r="F139" s="5"/>
     </row>
     <row r="140" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A140" s="3">
-        <v>139</v>
-      </c>
+      <c r="A140" s="3"/>
       <c r="B140" s="4"/>
-      <c r="C140" s="10" t="s">
-        <v>147</v>
-      </c>
-      <c r="D140" s="6">
-        <v>0.01</v>
-      </c>
-      <c r="E140" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F140" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C140" s="10"/>
+      <c r="D140" s="6"/>
+      <c r="E140" s="7"/>
+      <c r="F140" s="5"/>
     </row>
     <row r="141" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A141" s="3">
-        <v>140</v>
-      </c>
+      <c r="A141" s="3"/>
       <c r="B141" s="4"/>
-      <c r="C141" s="10" t="s">
-        <v>162</v>
-      </c>
-      <c r="D141" s="6">
-        <v>3</v>
-      </c>
-      <c r="E141" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F141" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C141" s="10"/>
+      <c r="D141" s="6"/>
+      <c r="E141" s="7"/>
+      <c r="F141" s="5"/>
     </row>
     <row r="142" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A142" s="3">
-        <v>141</v>
-      </c>
+      <c r="A142" s="3"/>
       <c r="B142" s="4"/>
-      <c r="C142" s="10" t="s">
-        <v>163</v>
-      </c>
-      <c r="D142" s="6">
-        <v>1</v>
-      </c>
-      <c r="E142" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F142" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C142" s="10"/>
+      <c r="D142" s="6"/>
+      <c r="E142" s="7"/>
+      <c r="F142" s="5"/>
     </row>
     <row r="143" spans="1:6" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A143" s="3">
-        <v>142</v>
-      </c>
+      <c r="A143" s="3"/>
       <c r="B143" s="4"/>
-      <c r="C143" s="10" t="s">
-        <v>174</v>
-      </c>
-      <c r="D143" s="6">
-        <v>63</v>
-      </c>
-      <c r="E143" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="F143" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C143" s="10"/>
+      <c r="D143" s="6"/>
+      <c r="E143" s="7"/>
+      <c r="F143" s="5"/>
     </row>
     <row r="144" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A144" s="3">
-        <v>143</v>
-      </c>
+      <c r="A144" s="3"/>
       <c r="B144" s="4"/>
-      <c r="C144" s="10" t="s">
-        <v>173</v>
-      </c>
-      <c r="D144" s="6">
-        <v>22</v>
-      </c>
-      <c r="E144" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="F144" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C144" s="10"/>
+      <c r="D144" s="6"/>
+      <c r="E144" s="7"/>
+      <c r="F144" s="5"/>
     </row>
     <row r="145" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A145" s="3">
-        <v>144</v>
-      </c>
+      <c r="A145" s="3"/>
       <c r="B145" s="4"/>
-      <c r="C145" s="10" t="s">
-        <v>175</v>
-      </c>
-      <c r="D145" s="6">
-        <v>4.0199999999999996</v>
-      </c>
-      <c r="E145" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="F145" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C145" s="10"/>
+      <c r="D145" s="6"/>
+      <c r="E145" s="7"/>
+      <c r="F145" s="5"/>
     </row>
     <row r="146" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A146" s="3">
-        <v>145</v>
-      </c>
+      <c r="A146" s="3"/>
       <c r="B146" s="4"/>
-      <c r="C146" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="D146" s="6">
-        <v>1.44</v>
-      </c>
-      <c r="E146" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="F146" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C146" s="10"/>
+      <c r="D146" s="6"/>
+      <c r="E146" s="7"/>
+      <c r="F146" s="5"/>
     </row>
     <row r="147" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A147" s="3">
-        <v>146</v>
-      </c>
+      <c r="A147" s="3"/>
       <c r="B147" s="4"/>
-      <c r="C147" s="10" t="s">
-        <v>172</v>
-      </c>
-      <c r="D147" s="6">
-        <v>3</v>
-      </c>
-      <c r="E147" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F147" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C147" s="10"/>
+      <c r="D147" s="6"/>
+      <c r="E147" s="7"/>
+      <c r="F147" s="5"/>
     </row>
     <row r="148" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A148" s="3">
-        <v>147</v>
-      </c>
+      <c r="A148" s="3"/>
       <c r="B148" s="4"/>
-      <c r="C148" s="10" t="s">
-        <v>171</v>
-      </c>
-      <c r="D148" s="6">
-        <v>1</v>
-      </c>
-      <c r="E148" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F148" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C148" s="10"/>
+      <c r="D148" s="6"/>
+      <c r="E148" s="7"/>
+      <c r="F148" s="5"/>
     </row>
     <row r="149" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A149" s="3">
-        <v>148</v>
-      </c>
+      <c r="A149" s="3"/>
       <c r="B149" s="4"/>
-      <c r="C149" s="10" t="s">
-        <v>170</v>
-      </c>
-      <c r="D149" s="6">
-        <v>32</v>
-      </c>
-      <c r="E149" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F149" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C149" s="10"/>
+      <c r="D149" s="6"/>
+      <c r="E149" s="7"/>
+      <c r="F149" s="5"/>
     </row>
     <row r="150" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A150" s="3">
-        <v>149</v>
-      </c>
+      <c r="A150" s="3"/>
       <c r="B150" s="4"/>
-      <c r="C150" s="10" t="s">
-        <v>169</v>
-      </c>
-      <c r="D150" s="6">
-        <v>2</v>
-      </c>
-      <c r="E150" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F150" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C150" s="10"/>
+      <c r="D150" s="6"/>
+      <c r="E150" s="7"/>
+      <c r="F150" s="5"/>
     </row>
     <row r="151" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A151" s="3">
-        <v>150</v>
-      </c>
+      <c r="A151" s="3"/>
       <c r="B151" s="4"/>
-      <c r="C151" s="10" t="s">
-        <v>168</v>
-      </c>
-      <c r="D151" s="6">
-        <v>1</v>
-      </c>
-      <c r="E151" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F151" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C151" s="10"/>
+      <c r="D151" s="6"/>
+      <c r="E151" s="7"/>
+      <c r="F151" s="5"/>
     </row>
     <row r="152" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A152" s="3">
-        <v>151</v>
-      </c>
+      <c r="A152" s="3"/>
       <c r="B152" s="4"/>
-      <c r="C152" s="10" t="s">
-        <v>167</v>
-      </c>
-      <c r="D152" s="6">
-        <v>10</v>
-      </c>
-      <c r="E152" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F152" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C152" s="10"/>
+      <c r="D152" s="6"/>
+      <c r="E152" s="7"/>
+      <c r="F152" s="5"/>
     </row>
     <row r="153" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A153" s="3">
-        <v>152</v>
-      </c>
+      <c r="A153" s="3"/>
       <c r="B153" s="4"/>
-      <c r="C153" s="10" t="s">
-        <v>166</v>
-      </c>
-      <c r="D153" s="6">
-        <v>4</v>
-      </c>
-      <c r="E153" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F153" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C153" s="10"/>
+      <c r="D153" s="6"/>
+      <c r="E153" s="7"/>
+      <c r="F153" s="5"/>
     </row>
     <row r="154" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A154" s="3">
-        <v>153</v>
-      </c>
+      <c r="A154" s="3"/>
       <c r="B154" s="4"/>
-      <c r="C154" s="10" t="s">
-        <v>131</v>
-      </c>
-      <c r="D154" s="6">
-        <v>1</v>
-      </c>
-      <c r="E154" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F154" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C154" s="10"/>
+      <c r="D154" s="6"/>
+      <c r="E154" s="7"/>
+      <c r="F154" s="5"/>
     </row>
     <row r="155" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A155" s="3">
-        <v>154</v>
-      </c>
+      <c r="A155" s="3"/>
       <c r="B155" s="4"/>
-      <c r="C155" s="10" t="s">
-        <v>165</v>
-      </c>
-      <c r="D155" s="6">
-        <v>1</v>
-      </c>
-      <c r="E155" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F155" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C155" s="10"/>
+      <c r="D155" s="6"/>
+      <c r="E155" s="7"/>
+      <c r="F155" s="5"/>
     </row>
     <row r="156" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A156" s="3">
-        <v>155</v>
-      </c>
+      <c r="A156" s="3"/>
       <c r="B156" s="4"/>
-      <c r="C156" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="D156" s="6">
-        <v>2</v>
-      </c>
-      <c r="E156" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F156" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C156" s="10"/>
+      <c r="D156" s="6"/>
+      <c r="E156" s="7"/>
+      <c r="F156" s="5"/>
     </row>
     <row r="157" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A157" s="3">
-        <v>156</v>
-      </c>
+      <c r="A157" s="3"/>
       <c r="B157" s="4"/>
-      <c r="C157" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="D157" s="6">
-        <v>5</v>
-      </c>
-      <c r="E157" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F157" s="5" t="s">
-        <v>148</v>
-      </c>
+      <c r="C157" s="10"/>
+      <c r="D157" s="6"/>
+      <c r="E157" s="7"/>
+      <c r="F157" s="5"/>
     </row>
     <row r="158" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A158" s="3">
-        <v>157</v>
-      </c>
+      <c r="A158" s="3"/>
       <c r="B158" s="4"/>
-      <c r="C158" s="10" t="s">
-        <v>176</v>
-      </c>
-      <c r="D158" s="6">
-        <v>1</v>
-      </c>
-      <c r="E158" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F158" s="5" t="s">
-        <v>177</v>
-      </c>
+      <c r="C158" s="10"/>
+      <c r="D158" s="6"/>
+      <c r="E158" s="7"/>
+      <c r="F158" s="5"/>
     </row>
     <row r="159" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A159" s="3">
-        <v>158</v>
-      </c>
+      <c r="A159" s="3"/>
       <c r="B159" s="4"/>
-      <c r="C159" s="10" t="s">
-        <v>180</v>
-      </c>
-      <c r="D159" s="6">
-        <v>1</v>
-      </c>
-      <c r="E159" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F159" s="5" t="s">
-        <v>179</v>
-      </c>
+      <c r="C159" s="10"/>
+      <c r="D159" s="6"/>
+      <c r="E159" s="7"/>
+      <c r="F159" s="5"/>
     </row>
     <row r="160" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A160" s="3">
-        <v>159</v>
-      </c>
+      <c r="A160" s="3"/>
       <c r="B160" s="4"/>
-      <c r="C160" s="10" t="s">
-        <v>178</v>
-      </c>
-      <c r="D160" s="6">
-        <v>1</v>
-      </c>
-      <c r="E160" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F160" s="5" t="s">
-        <v>179</v>
-      </c>
+      <c r="C160" s="10"/>
+      <c r="D160" s="6"/>
+      <c r="E160" s="7"/>
+      <c r="F160" s="5"/>
     </row>
     <row r="161" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A161" s="3">
-        <v>160</v>
-      </c>
+      <c r="A161" s="3"/>
       <c r="B161" s="4"/>
-      <c r="C161" s="10" t="s">
-        <v>184</v>
-      </c>
-      <c r="D161" s="6">
-        <v>2</v>
-      </c>
-      <c r="E161" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F161" s="5" t="s">
-        <v>183</v>
-      </c>
+      <c r="C161" s="10"/>
+      <c r="D161" s="6"/>
+      <c r="E161" s="7"/>
+      <c r="F161" s="5"/>
     </row>
     <row r="162" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A162" s="3">
-        <v>161</v>
-      </c>
+      <c r="A162" s="3"/>
       <c r="B162" s="4"/>
-      <c r="C162" s="10" t="s">
-        <v>181</v>
-      </c>
-      <c r="D162" s="6">
-        <v>2</v>
-      </c>
-      <c r="E162" s="7" t="s">
-        <v>182</v>
-      </c>
-      <c r="F162" s="5" t="s">
-        <v>183</v>
-      </c>
+      <c r="C162" s="10"/>
+      <c r="D162" s="6"/>
+      <c r="E162" s="7"/>
+      <c r="F162" s="5"/>
     </row>
     <row r="163" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A163" s="3">
-        <v>162</v>
-      </c>
+      <c r="A163" s="3"/>
       <c r="B163" s="4"/>
-      <c r="C163" s="10" t="s">
-        <v>185</v>
-      </c>
-      <c r="D163" s="6">
-        <v>12</v>
-      </c>
-      <c r="E163" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F163" s="5" t="s">
-        <v>186</v>
-      </c>
+      <c r="C163" s="10"/>
+      <c r="D163" s="6"/>
+      <c r="E163" s="7"/>
+      <c r="F163" s="5"/>
     </row>
     <row r="164" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A164" s="3">
-        <v>163</v>
-      </c>
+      <c r="A164" s="3"/>
       <c r="B164" s="4"/>
-      <c r="C164" s="10" t="s">
-        <v>187</v>
-      </c>
-      <c r="D164" s="6">
-        <v>1248.52</v>
-      </c>
-      <c r="E164" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F164" s="5" t="s">
-        <v>188</v>
-      </c>
+      <c r="C164" s="10"/>
+      <c r="D164" s="6"/>
+      <c r="E164" s="7"/>
+      <c r="F164" s="5"/>
     </row>
     <row r="165" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A165" s="3">
-        <v>164</v>
-      </c>
+      <c r="A165" s="3"/>
       <c r="B165" s="4"/>
-      <c r="C165" s="10" t="s">
-        <v>187</v>
-      </c>
-      <c r="D165" s="6">
-        <v>1248.52</v>
-      </c>
-      <c r="E165" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F165" s="5" t="s">
-        <v>188</v>
-      </c>
+      <c r="C165" s="10"/>
+      <c r="D165" s="6"/>
+      <c r="E165" s="7"/>
+      <c r="F165" s="5"/>
     </row>
     <row r="166" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A166" s="3">
-        <v>165</v>
-      </c>
+      <c r="A166" s="3"/>
       <c r="B166" s="4"/>
-      <c r="C166" s="10" t="s">
-        <v>187</v>
-      </c>
-      <c r="D166" s="6">
-        <v>312.13</v>
-      </c>
-      <c r="E166" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F166" s="5" t="s">
-        <v>188</v>
-      </c>
+      <c r="C166" s="10"/>
+      <c r="D166" s="6"/>
+      <c r="E166" s="7"/>
+      <c r="F166" s="5"/>
     </row>
     <row r="167" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A167" s="3">
-        <v>166</v>
-      </c>
+      <c r="A167" s="3"/>
       <c r="B167" s="4"/>
-      <c r="C167" s="10" t="s">
-        <v>187</v>
-      </c>
-      <c r="D167" s="6">
-        <v>312.13</v>
-      </c>
-      <c r="E167" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F167" s="5" t="s">
-        <v>188</v>
-      </c>
+      <c r="C167" s="10"/>
+      <c r="D167" s="6"/>
+      <c r="E167" s="7"/>
+      <c r="F167" s="5"/>
     </row>
     <row r="168" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A168" s="3">
-        <v>167</v>
-      </c>
+      <c r="A168" s="3"/>
       <c r="B168" s="4"/>
-      <c r="C168" s="10" t="s">
-        <v>187</v>
-      </c>
-      <c r="D168" s="6">
-        <v>312.13</v>
-      </c>
-      <c r="E168" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F168" s="5" t="s">
-        <v>188</v>
-      </c>
+      <c r="C168" s="10"/>
+      <c r="D168" s="6"/>
+      <c r="E168" s="7"/>
+      <c r="F168" s="5"/>
     </row>
     <row r="169" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A169" s="3">
-        <v>168</v>
-      </c>
+      <c r="A169" s="3"/>
       <c r="B169" s="4"/>
-      <c r="C169" s="10" t="s">
-        <v>181</v>
-      </c>
-      <c r="D169" s="6">
-        <v>5</v>
-      </c>
-      <c r="E169" s="7" t="s">
-        <v>182</v>
-      </c>
-      <c r="F169" s="5" t="s">
-        <v>192</v>
-      </c>
+      <c r="C169" s="10"/>
+      <c r="D169" s="6"/>
+      <c r="E169" s="7"/>
+      <c r="F169" s="5"/>
     </row>
     <row r="170" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A170" s="3">
-        <v>169</v>
-      </c>
+      <c r="A170" s="3"/>
       <c r="B170" s="4"/>
-      <c r="C170" s="10" t="s">
-        <v>184</v>
-      </c>
-      <c r="D170" s="6">
-        <v>5</v>
-      </c>
-      <c r="E170" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F170" s="5" t="s">
-        <v>192</v>
-      </c>
+      <c r="C170" s="10"/>
+      <c r="D170" s="6"/>
+      <c r="E170" s="7"/>
+      <c r="F170" s="5"/>
     </row>
     <row r="171" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A171" s="3"/>

</xml_diff>

<commit_message>
new home, news and Layout
</commit_message>
<xml_diff>
--- a/public/procurement.xlsx
+++ b/public/procurement.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lka\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{141D86CA-40BA-49E4-AB5C-5D264E776348}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7475053D-1628-47ED-96A9-1CD5DA872060}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4755" yWindow="3270" windowWidth="23730" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="148">
   <si>
     <t>№ п/п</t>
   </si>
@@ -54,237 +54,219 @@
     <t>Труба D89х12 Ст.09Г2 ГОСТ 19281-89</t>
   </si>
   <si>
-    <t>АС 30, Гидравл. тележка 3000 кг, 1150х550 мм, полиурет.колесо, двойные полиурет.ролики, цвет красный</t>
+    <t>не исп. Труба D89х6 ГОСТ 8732-78/ Ст.20 ГОСТ 8731-87</t>
+  </si>
+  <si>
+    <t>ЛГУП-7315</t>
   </si>
   <si>
     <t>шт</t>
   </si>
   <si>
-    <t>ЛГУП-7313</t>
-  </si>
-  <si>
-    <t>ЛГУП-7315</t>
-  </si>
-  <si>
-    <t>не исп. Труба D89х6 ГОСТ 8732-78/ Ст.20 ГОСТ 8731-87</t>
-  </si>
-  <si>
-    <t>Лист 3 ст 35</t>
-  </si>
-  <si>
-    <t>ЛГУП-7319</t>
+    <t>ЛГУП-7331</t>
+  </si>
+  <si>
+    <t>Каска строительная оранжевая Исток</t>
+  </si>
+  <si>
+    <t>шт.</t>
+  </si>
+  <si>
+    <t>Маркер по металлу черный тонкий</t>
+  </si>
+  <si>
+    <t>Ветошь</t>
+  </si>
+  <si>
+    <t>Маркер белый</t>
+  </si>
+  <si>
+    <t>Каска строительная белая</t>
+  </si>
+  <si>
+    <t>Маркер по металлу белый</t>
+  </si>
+  <si>
+    <t>Огнетушитель ОП-8</t>
+  </si>
+  <si>
+    <t>Перчатки с латесным покрытием</t>
+  </si>
+  <si>
+    <t>пар</t>
+  </si>
+  <si>
+    <t>Перчатки х/б трикотажные 5 нитей 10 класс с ПВХ -Камаз 426</t>
+  </si>
+  <si>
+    <t>пара</t>
   </si>
   <si>
     <t>Маркер  краска красный по металлу</t>
   </si>
   <si>
-    <t>шт.</t>
-  </si>
-  <si>
-    <t>ЛГУП-7331</t>
-  </si>
-  <si>
-    <t>Перчатки х/б трикотажные 5 нитей 10 класс с ПВХ -Камаз 426</t>
-  </si>
-  <si>
-    <t>пара</t>
-  </si>
-  <si>
-    <t>Перчатки с латесным покрытием</t>
-  </si>
-  <si>
-    <t>пар</t>
-  </si>
-  <si>
-    <t>Ветошь</t>
-  </si>
-  <si>
-    <t>Маркер белый</t>
-  </si>
-  <si>
-    <t>Каска строительная белая</t>
-  </si>
-  <si>
-    <t>Каска строительная оранжевая Исток</t>
-  </si>
-  <si>
-    <t>Маркер по металлу черный тонкий</t>
-  </si>
-  <si>
-    <t>Маркер по металлу белый</t>
-  </si>
-  <si>
-    <t>Огнетушитель ОП-8</t>
+    <t>Гайковерт</t>
+  </si>
+  <si>
+    <t>ЛГУП-7332</t>
+  </si>
+  <si>
+    <t>Ключ комбинированные омедненные 41</t>
+  </si>
+  <si>
+    <t>Ключ комбинированные омедненные 36</t>
+  </si>
+  <si>
+    <t>Ключ комбинированные омедненные 30</t>
+  </si>
+  <si>
+    <t>Ключ комбинированные омедненные 24</t>
+  </si>
+  <si>
+    <t>Трещетка ключ 1/2</t>
+  </si>
+  <si>
+    <t>Ножницы по металлу</t>
+  </si>
+  <si>
+    <t>Ключи обмедненные</t>
+  </si>
+  <si>
+    <t>набор</t>
+  </si>
+  <si>
+    <t>Кувалда 1 кг.</t>
   </si>
   <si>
     <t>Резак</t>
   </si>
   <si>
-    <t>ЛГУП-7332</t>
-  </si>
-  <si>
-    <t>Ножницы по металлу</t>
-  </si>
-  <si>
-    <t>Трещетка ключ 1/2</t>
-  </si>
-  <si>
-    <t>Ключ комбинированные омедненные 24</t>
-  </si>
-  <si>
-    <t>Ключ комбинированные омедненные 30</t>
-  </si>
-  <si>
-    <t>Ключ комбинированные омедненные 36</t>
-  </si>
-  <si>
-    <t>Ключ комбинированные омедненные 41</t>
-  </si>
-  <si>
-    <t>Гайковерт</t>
-  </si>
-  <si>
-    <t>Кувалда 1 кг.</t>
-  </si>
-  <si>
-    <t>Ключи обмедненные</t>
-  </si>
-  <si>
-    <t>набор</t>
-  </si>
-  <si>
-    <t>ЛГУП-7333</t>
-  </si>
-  <si>
-    <t>отвод 89х8, 09Г2С ГОСТ 17375-2001</t>
-  </si>
-  <si>
-    <t>Отвод 76х8, ст09г2с ГОСТ 17375-2001</t>
-  </si>
-  <si>
-    <t>Отвод 57х6, 09Г2С ГОСТ 17375-2001</t>
+    <t>Эмаль ПФ-115 желтая (22кг)</t>
+  </si>
+  <si>
+    <t>ЛГУП-7334</t>
+  </si>
+  <si>
+    <t>Эмаль ПФ 115 красная 1,8кг STATUS /6</t>
+  </si>
+  <si>
+    <t>Растворитель 646 (5л)</t>
   </si>
   <si>
     <t>Эмаль ПФ-115 коричневая (25 кг), шт</t>
   </si>
   <si>
-    <t>ЛГУП-7334</t>
-  </si>
-  <si>
-    <t>Эмаль ПФ-115 серая 5,5 кг</t>
-  </si>
-  <si>
-    <t>Эмаль ПФ 115 красная 1,8кг STATUS /6</t>
-  </si>
-  <si>
-    <t>Эмаль ПФ-115 желтая (22кг)</t>
-  </si>
-  <si>
-    <t>Эмаль ПФ 115 черная 1,8кг STATUS /6</t>
-  </si>
-  <si>
-    <t>Паронит 3 мм</t>
-  </si>
-  <si>
-    <t>лист</t>
-  </si>
-  <si>
-    <t>Растворитель 646 (5л)</t>
-  </si>
-  <si>
-    <t>Паронит 2мм</t>
-  </si>
-  <si>
     <t>Растворитель Р-4 /кг/</t>
   </si>
   <si>
-    <t>Уголок 50х50х3 ГОСТ 8509-93/ст.20 ГОСТ 19281-2014</t>
-  </si>
-  <si>
-    <t>ЛГУП-7336</t>
-  </si>
-  <si>
-    <t>Опресовочный насос (ручной) на 60кг (6МПа)</t>
-  </si>
-  <si>
-    <t>Салфетки влажные SMART ЭКОНОМ для всей семьи 70шт</t>
-  </si>
-  <si>
-    <t>НТУП-017966</t>
-  </si>
-  <si>
-    <t>Грифель для карандаша механического 0,5мм, НВ</t>
-  </si>
-  <si>
-    <t>Грифель для карандаша механического 0,7мм, НВ</t>
-  </si>
-  <si>
-    <t>Папка-регистратор 50 мм</t>
-  </si>
-  <si>
-    <t>Папка-регистратор 75 мм</t>
-  </si>
-  <si>
-    <t>Мыло жидкое</t>
-  </si>
-  <si>
-    <t>Разделитель цветной картонный 240-105мм</t>
-  </si>
-  <si>
-    <t>Белизна-гель 3 в 1</t>
-  </si>
-  <si>
-    <t>Конверты А5, комплект 500шт</t>
-  </si>
-  <si>
-    <t>Скобы №10</t>
-  </si>
-  <si>
-    <t>Ручка шариковая синяя</t>
-  </si>
-  <si>
-    <t>Скобы №24/6</t>
-  </si>
-  <si>
-    <t>Бумага А4 500л.</t>
-  </si>
-  <si>
-    <t>Туалетная бумага</t>
-  </si>
-  <si>
-    <t>Мешки для мусора 30 л синие в рулоне 30шт. прочные,ПНД 10мкм 50*60 см, LAIMA</t>
-  </si>
-  <si>
-    <t>Батарейки GP Super, AA (LR6,15А), алкалиновые, пальч., КОМПЛЕКТ 10 шт., в пленке, 15A-2CRB10_АМК</t>
-  </si>
-  <si>
-    <t>компл</t>
-  </si>
-  <si>
-    <t>Закладки клейкие неоновые STAFF "СТРЕЛКИ" 45х8 мм, 100шт (5 цв. х 20 л.) на пласт.основании, 111355</t>
-  </si>
-  <si>
-    <t>00УП-000005</t>
+    <t>Дробемет для швеллера с конвейерной сеткой</t>
+  </si>
+  <si>
+    <t>ЛГУП-7338</t>
+  </si>
+  <si>
+    <t>Маркировка фланца</t>
+  </si>
+  <si>
+    <t>ЛГУП-7339</t>
+  </si>
+  <si>
+    <t>Шина</t>
+  </si>
+  <si>
+    <t>НТУП-017968</t>
+  </si>
+  <si>
+    <t>Строительство фундамента лестничной клетки(без учета материала)</t>
+  </si>
+  <si>
+    <t>ЛГУП-7342</t>
+  </si>
+  <si>
+    <t>Строительство Промышленного пола(без учета материала)</t>
+  </si>
+  <si>
+    <t>Строительство Отмоски и цоколя(без учета материала)</t>
+  </si>
+  <si>
+    <t>ЛГУП-7346</t>
+  </si>
+  <si>
+    <t>м</t>
+  </si>
+  <si>
+    <t>ЛГУП-7347</t>
+  </si>
+  <si>
+    <t>ЛГУП-7348</t>
+  </si>
+  <si>
+    <t>ЛГУП-7349</t>
+  </si>
+  <si>
+    <t>ЛГУП-7351</t>
+  </si>
+  <si>
+    <t>ЛГУП-7352</t>
+  </si>
+  <si>
+    <t>ЛГУП-7353</t>
+  </si>
+  <si>
+    <t>ЛГУП-7355</t>
+  </si>
+  <si>
+    <t>Фланец 25-40-11-1-E-09Г2С-IV ГОСТ 33259-2015</t>
+  </si>
+  <si>
+    <t>ЛГУП-7356</t>
+  </si>
+  <si>
+    <t>ЛГУП-7357</t>
+  </si>
+  <si>
+    <t>Услуги по договору номер 7</t>
+  </si>
+  <si>
+    <t>АХУП-000649</t>
+  </si>
+  <si>
+    <t>ЛГУП-7365</t>
+  </si>
+  <si>
+    <t>ЛГУП-7366</t>
+  </si>
+  <si>
+    <t>л (дм3)</t>
+  </si>
+  <si>
+    <t>ЛГУП-7367</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Труба D25х7 ст.10Г2 ГОСТ 8733-74</t>
+  </si>
+  <si>
+    <t>Уголок 40х40х3 ГОСТ 8509-93/ Ст3пс ГОСТ 535-88</t>
+  </si>
+  <si>
+    <t>Труба D377х12 ст.09Г2С-К50 ГОСТ 8731-78</t>
+  </si>
+  <si>
+    <t>Труба D720х12 Ст.09Г2С-К50 ГОСТ 20295-85</t>
+  </si>
+  <si>
+    <t>Труба D159х10 ГОСТ 8732-78/ 09Г2С ГОСТ 8731-74</t>
+  </si>
+  <si>
+    <t>Труба D219х18 Ст.09ГС ГОСТ 8731-74</t>
   </si>
   <si>
     <t>Труба D219х4 ГОСТ 8734-75/ Ст.В20 ГОСТ 8733-74</t>
   </si>
   <si>
-    <t>Труба D219х18 Ст.09ГС ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>Труба D159х10 ГОСТ 8732-78/ 09Г2С ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>Труба D720х12 Ст.09Г2С-К50 ГОСТ 20295-85</t>
-  </si>
-  <si>
-    <t>Труба D377х12 ст.09Г2С-К50 ГОСТ 8731-78</t>
-  </si>
-  <si>
-    <t>Уголок 40х40х3 ГОСТ 8509-93/ Ст3пс ГОСТ 535-88</t>
-  </si>
-  <si>
     <t>Труба D89х8 ГОСТ 872-78 В 09Г2С ГОСТ 8731-74</t>
   </si>
   <si>
@@ -303,106 +285,190 @@
     <t>Труба D273х10 ГОСТ 8732-78/ 09Г2С ГОСТ 30564-98</t>
   </si>
   <si>
-    <t>Труба D25х7 ст.10Г2 ГОСТ 8733-74</t>
+    <t>Труба D57х4 ГОСТ 8732-78/ 09Г2С ГОСТ 8731-74</t>
   </si>
   <si>
     <t>Труба D480х16 10Г2 ГОСТ 8731-74</t>
   </si>
   <si>
+    <t>Труба D57х5 ГОСТ 8732-78/09Г2С ГОСТ 8731-74</t>
+  </si>
+  <si>
+    <t>Труба D110х16 ГОСТ 8734-75/ Ст.20 ГОСТ 8733-74</t>
+  </si>
+  <si>
+    <t>Труба D73х9 Ст20 ГОСТ 8731-74</t>
+  </si>
+  <si>
+    <t>не исп. Труба D83х10 Ст20 ГОСТ 8731-74</t>
+  </si>
+  <si>
+    <t>Труба D42х10 Ст.09Г2С ГОСТ 19281-89</t>
+  </si>
+  <si>
+    <t>Труба D140х25 Ст.20 ГОСТ 8732-78</t>
+  </si>
+  <si>
+    <t>Труба D159х18 Ст.20 ГОСТ 8732-78</t>
+  </si>
+  <si>
+    <t>Труба D83*10 Ст.12Х18Н10Т ГОСТ 5949-72</t>
+  </si>
+  <si>
     <t>Труба D89х8 Ст.35 ГОСТ 1050-80</t>
   </si>
   <si>
-    <t>Труба D42х10 Ст.09Г2С ГОСТ 19281-89</t>
-  </si>
-  <si>
-    <t>Труба D83*10 Ст.12Х18Н10Т ГОСТ 5949-72</t>
-  </si>
-  <si>
-    <t>Труба D159х18 Ст.20 ГОСТ 8732-78</t>
-  </si>
-  <si>
-    <t>Труба D140х25 Ст.20 ГОСТ 8732-78</t>
+    <t>Труба 25х3,2 ГОСТ 3262-75 (D33,5)</t>
+  </si>
+  <si>
+    <t>Труба D83х9 Ст.40Х ГОСТ 8731-87</t>
+  </si>
+  <si>
+    <t>Труба D219х5 Ст.20 ГОСТ 1050-88</t>
   </si>
   <si>
     <t>Труба D146х22 Ст.20 ГОСТ 8732-78</t>
   </si>
   <si>
+    <t>Труба D108х11 Ст. 20Х13 ГОСТ 5632-72</t>
+  </si>
+  <si>
     <t>Труба D121х6 ГОСТ 8732-78 /Ст. 20 ГОСТ 8731-74</t>
   </si>
   <si>
+    <t>Труба D14х2 09Г2С ГОСТ 8733-74</t>
+  </si>
+  <si>
     <t>Труба D180х25 ГОСТ 8732-78 / 09Г2С ГОСТ 19281-89</t>
   </si>
   <si>
+    <t>Труба D65х14 Ст.20 ГОСТ 8731-74</t>
+  </si>
+  <si>
+    <t>Труба D194х14 В20 ГОСТ 8732-78</t>
+  </si>
+  <si>
     <t>Труба D83*9 Ст.20 ГОСТ 1050-88</t>
   </si>
   <si>
-    <t>Труба D194х14 В20 ГОСТ 8732-78</t>
-  </si>
-  <si>
-    <t>не исп. Труба D83х10 Ст20 ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>Труба D73х9 Ст20 ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>Труба D110х16 ГОСТ 8734-75/ Ст.20 ГОСТ 8733-74</t>
-  </si>
-  <si>
-    <t>Труба D57х5 ГОСТ 8732-78/09Г2С ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>Труба D57х4 ГОСТ 8732-78/ 09Г2С ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>Труба D65х14 Ст.20 ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>Труба D14х2 09Г2С ГОСТ 8733-74</t>
-  </si>
-  <si>
-    <t>Труба D108х11 Ст. 20Х13 ГОСТ 5632-72</t>
-  </si>
-  <si>
-    <t>Труба D219х5 Ст.20 ГОСТ 1050-88</t>
-  </si>
-  <si>
-    <t>Труба D83х9 Ст.40Х ГОСТ 8731-87</t>
-  </si>
-  <si>
-    <t>Труба 25х3,2 ГОСТ 3262-75 (D33,5)</t>
-  </si>
-  <si>
     <t>Маркер черный</t>
   </si>
   <si>
     <t>Фумлента</t>
   </si>
   <si>
-    <t>Переход 114х8-89х8 Ст.09Г2С ГОСТ 17378-01</t>
-  </si>
-  <si>
-    <t>Переход 89х8-76х8 ст. 09Г2С ГОСТ 17378-01</t>
-  </si>
-  <si>
-    <t>Переход 159х8-108х8 ст.09Г2С ГОСТ 17378-01</t>
-  </si>
-  <si>
-    <t>Лист S=4 09Г2С</t>
-  </si>
-  <si>
-    <t>Швеллер №20У ГОСТ 8240-97/ 325-09Г2С ГОСТ 19281-2014</t>
-  </si>
-  <si>
-    <t>Швеллер №5П ГОСТ 8240-97/ Ст.09Г2С ГОСТ 535-2005</t>
-  </si>
-  <si>
-    <t>Уголок 50х50х5 ГОСТ 8509-93/ Ст.09Г2С ГОСТ 19281-2014</t>
-  </si>
-  <si>
-    <t>Лист чечевица В-К-ПУ-3,0 Ст.09Г2С ГОСТ 8568-77</t>
-  </si>
-  <si>
-    <t>Лист S=3,0 ГОСТ 19903-74/09Г2С ГОСТ 19281-89</t>
+    <t>Гайка М30х1,5-6Н.09Г2С.019 ГОСТ 5915-70</t>
+  </si>
+  <si>
+    <t>Болт 1.2 М30х1000</t>
+  </si>
+  <si>
+    <t>Кабель ВВГнг(А)-LS-ХЛ 4x1,5 d10,2мм</t>
+  </si>
+  <si>
+    <t>Гайка М16-6Н.09Г2С (оцинк.) ГОСТ 9064-75</t>
+  </si>
+  <si>
+    <t>Круг ДКРН D48 НД БрАЖ9-4 ГОСТ 1628-78</t>
+  </si>
+  <si>
+    <t>Круг D165 09Г2С-8-ТО ГОСТ 19281-89</t>
+  </si>
+  <si>
+    <t>Круг D450 Ст.09Г2С ГОСТ 2590-2006</t>
+  </si>
+  <si>
+    <t>Лист S=1 ст.09Г2С ГОСТ16523-89</t>
+  </si>
+  <si>
+    <t>Полоса 30х30 Ст.20Л</t>
+  </si>
+  <si>
+    <t>Шестигранник S=17 Ст.20 ГОСТ 1050-88</t>
+  </si>
+  <si>
+    <t>Шестигранник S=24 Ст.20 ГОСТ 1050-88</t>
+  </si>
+  <si>
+    <t>Шестигранник S=27 Ст.35 ГОСТ 1050-88</t>
+  </si>
+  <si>
+    <t>Шестигранник S=30 Ст.20 ГОСТ 1050-88</t>
+  </si>
+  <si>
+    <t>Шестигранник S=30 Ст.45 ГОСТ 535-88</t>
+  </si>
+  <si>
+    <t>Шестигранник S=46 Ст.09Г2С ГОСТ 535-88</t>
+  </si>
+  <si>
+    <t>Шестигранник S=46 Ст.45 ГОСТ 535-88</t>
+  </si>
+  <si>
+    <t>Отвод 45-89х8-09Г2С ГОСТ 17375-2001</t>
+  </si>
+  <si>
+    <t>Тройник 20х3-09Г2С ГОСТ 17376-2001</t>
+  </si>
+  <si>
+    <t>Светильник взрывозащищенный ДБП 09-15-001 УХЛ1 ExdllBT6G IP65</t>
+  </si>
+  <si>
+    <t>Труба D14х3 ГОСТ 8732-78/ 09Г2С ГОСТ 8731-74</t>
+  </si>
+  <si>
+    <t>Труба D20х3 ГОСТ 8732-78/ 09Г2С  ГОСТ 8731-74</t>
+  </si>
+  <si>
+    <t>Фланец 1-250-40 09Г2С ГОСТ 12821-80</t>
+  </si>
+  <si>
+    <t>Фланец 2-50-40 09Г2С ГОСТ 12821-80</t>
+  </si>
+  <si>
+    <t>Болт М20-6gх30.58 (S30) ГОСТ 7798-70</t>
+  </si>
+  <si>
+    <t>Заклепка 4х8.31 ГОСТ 10299-80</t>
+  </si>
+  <si>
+    <t>Шпилька АМ30-6gх180.60.35.III.4.019 ГОСТ 9066-75</t>
+  </si>
+  <si>
+    <t>Шпилька АМ16-6gx80 ГОСТ 9066-75</t>
+  </si>
+  <si>
+    <t>Шайба 8.01.019 ГОСТ 11371-78</t>
+  </si>
+  <si>
+    <t>Шайба 8 65Г 019 ГОСТ 6402-70</t>
+  </si>
+  <si>
+    <t>Шайба 30.Ст3сп3.II.4.019 ГОСТ 9065-75</t>
+  </si>
+  <si>
+    <t>Шайба 16 ГОСТ 6958-78</t>
+  </si>
+  <si>
+    <t>Фланец х-300-40 (заготовка-поковка Ст.08Х18Н10 гр.IV КП195 ГОСТ 8479-70)</t>
+  </si>
+  <si>
+    <t>Растворитель Р-4 ГОСТ 7827-74</t>
+  </si>
+  <si>
+    <t>Грунт-эмаль Дюропокс ДТМ 70 цвет серый (наружка)</t>
+  </si>
+  <si>
+    <t>Краска-спрей SABOTAGE (желтая)</t>
+  </si>
+  <si>
+    <t>Разбавитель Procore Universal Thinner</t>
+  </si>
+  <si>
+    <t>Прокладка Б-50-40-ПМБ ГОСТ 15180-86</t>
+  </si>
+  <si>
+    <t>Краска-спрей SABOTAGE 39(черный)</t>
   </si>
 </sst>
 </file>
@@ -839,13 +905,13 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F116"/>
+  <dimension ref="A1:F139"/>
   <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="11.45" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.1640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="46.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="74.83203125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="14.1640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="63.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" style="1" customWidth="1"/>
     <col min="5" max="5" width="13" style="1" customWidth="1"/>
     <col min="6" max="6" width="14.5" style="1" customWidth="1"/>
   </cols>
@@ -876,10 +942,10 @@
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="8" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="D2" s="5">
-        <v>95.25</v>
+        <v>20.399999999999999</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>6</v>
@@ -894,10 +960,10 @@
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="8" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="D3" s="5">
-        <v>291.60000000000002</v>
+        <v>48.6</v>
       </c>
       <c r="E3" s="6" t="s">
         <v>6</v>
@@ -912,10 +978,10 @@
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="D4" s="5">
-        <v>233.85</v>
+        <v>75</v>
+      </c>
+      <c r="D4" s="7">
+        <v>2000</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>6</v>
@@ -930,10 +996,10 @@
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="5">
-        <v>47.85</v>
+        <v>76</v>
+      </c>
+      <c r="D5" s="7">
+        <v>4500</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>6</v>
@@ -948,10 +1014,10 @@
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="D6" s="7">
-        <v>4500</v>
+        <v>8</v>
+      </c>
+      <c r="D6" s="5">
+        <v>47.85</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>6</v>
@@ -966,10 +1032,10 @@
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="D7" s="7">
-        <v>2000</v>
+        <v>77</v>
+      </c>
+      <c r="D7" s="5">
+        <v>233.85</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>6</v>
@@ -984,10 +1050,10 @@
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="8" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="D8" s="5">
-        <v>48.6</v>
+        <v>291.60000000000002</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>6</v>
@@ -1002,10 +1068,10 @@
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="8" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="D9" s="5">
-        <v>97.8</v>
+        <v>95.25</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>6</v>
@@ -1020,10 +1086,10 @@
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="8" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="D10" s="5">
-        <v>57.15</v>
+        <v>97.8</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>6</v>
@@ -1038,10 +1104,10 @@
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="8" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="D11" s="5">
-        <v>33.75</v>
+        <v>57.15</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>6</v>
@@ -1056,10 +1122,10 @@
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="8" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="D12" s="5">
-        <v>16.5</v>
+        <v>33.75</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>6</v>
@@ -1074,10 +1140,10 @@
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="8" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="D13" s="5">
-        <v>7.05</v>
+        <v>16.5</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>6</v>
@@ -1092,10 +1158,10 @@
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="8" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="D14" s="5">
-        <v>193.2</v>
+        <v>7.05</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>6</v>
@@ -1110,10 +1176,10 @@
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="8" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="D15" s="5">
-        <v>20.399999999999999</v>
+        <v>193.2</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>6</v>
@@ -1122,7 +1188,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -1131,13 +1197,13 @@
         <v>9</v>
       </c>
       <c r="D16" s="5">
-        <v>2</v>
+        <v>26.52</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1146,16 +1212,16 @@
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="8" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="D17" s="5">
-        <v>36.6</v>
+        <v>0.84</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1164,16 +1230,16 @@
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="8" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="D18" s="5">
-        <v>6.45</v>
+        <v>51.52</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1182,16 +1248,16 @@
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="8" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="D19" s="5">
-        <v>5.16</v>
+        <v>146.4</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1200,16 +1266,16 @@
       </c>
       <c r="B20" s="4"/>
       <c r="C20" s="8" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="D20" s="5">
-        <v>0.43</v>
+        <v>1.52</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1218,16 +1284,16 @@
       </c>
       <c r="B21" s="4"/>
       <c r="C21" s="8" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="D21" s="5">
-        <v>2.2400000000000002</v>
+        <v>11.2</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1236,16 +1302,16 @@
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="8" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="D22" s="5">
-        <v>6.06</v>
+        <v>5.68</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1254,16 +1320,16 @@
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="8" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="D23" s="5">
-        <v>2.87</v>
+        <v>2.52</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1272,16 +1338,16 @@
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="8" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="D24" s="5">
-        <v>2.7</v>
+        <v>13.76</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1290,16 +1356,16 @@
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="8" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="D25" s="5">
-        <v>5.35</v>
+        <v>19.440000000000001</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1308,16 +1374,16 @@
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="8" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="D26" s="5">
-        <v>19.440000000000001</v>
+        <v>6.06</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1326,16 +1392,16 @@
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="8" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="D27" s="5">
-        <v>2.04</v>
+        <v>2.2400000000000002</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1344,16 +1410,16 @@
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="8" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="D28" s="5">
-        <v>77.760000000000005</v>
+        <v>0.43</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1362,16 +1428,16 @@
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="8" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="D29" s="5">
-        <v>43.48</v>
+        <v>5.16</v>
       </c>
       <c r="E29" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1380,16 +1446,16 @@
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="8" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="D30" s="5">
-        <v>2.52</v>
+        <v>6.45</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1398,16 +1464,16 @@
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="8" t="s">
-        <v>105</v>
+        <v>87</v>
       </c>
       <c r="D31" s="5">
-        <v>5.68</v>
+        <v>36.6</v>
       </c>
       <c r="E31" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1416,16 +1482,16 @@
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="8" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="D32" s="5">
-        <v>11.2</v>
+        <v>1.1950000000000001</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1434,16 +1500,16 @@
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="8" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="D33" s="5">
-        <v>1.52</v>
+        <v>3.97</v>
       </c>
       <c r="E33" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1452,16 +1518,16 @@
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="8" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D34" s="5">
-        <v>146.4</v>
+        <v>17.84</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1470,16 +1536,16 @@
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="8" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D35" s="5">
-        <v>51.52</v>
+        <v>8.9600000000000009</v>
       </c>
       <c r="E35" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1488,16 +1554,16 @@
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="8" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="D36" s="5">
-        <v>0.84</v>
+        <v>1.72</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1506,16 +1572,16 @@
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="8" t="s">
-        <v>13</v>
+        <v>93</v>
       </c>
       <c r="D37" s="5">
-        <v>26.52</v>
+        <v>24.24</v>
       </c>
       <c r="E37" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1524,16 +1590,16 @@
       </c>
       <c r="B38" s="4"/>
       <c r="C38" s="8" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="D38" s="5">
-        <v>13.76</v>
+        <v>15.24</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1542,16 +1608,16 @@
       </c>
       <c r="B39" s="4"/>
       <c r="C39" s="8" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="D39" s="5">
-        <v>8.8000000000000007</v>
+        <v>11.48</v>
       </c>
       <c r="E39" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1560,16 +1626,16 @@
       </c>
       <c r="B40" s="4"/>
       <c r="C40" s="8" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="D40" s="5">
-        <v>6.64</v>
+        <v>3.56</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1578,16 +1644,16 @@
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="8" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D41" s="5">
-        <v>21.4</v>
+        <v>10.8</v>
       </c>
       <c r="E41" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1596,7 +1662,7 @@
       </c>
       <c r="B42" s="4"/>
       <c r="C42" s="8" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="D42" s="5">
         <v>4</v>
@@ -1605,7 +1671,7 @@
         <v>6</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1614,16 +1680,16 @@
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="8" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D43" s="5">
-        <v>10.8</v>
+        <v>21.4</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1632,16 +1698,16 @@
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="8" t="s">
-        <v>111</v>
+        <v>83</v>
       </c>
       <c r="D44" s="5">
-        <v>3.56</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1650,16 +1716,16 @@
       </c>
       <c r="B45" s="4"/>
       <c r="C45" s="8" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D45" s="5">
-        <v>11.48</v>
+        <v>6.64</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1668,16 +1734,16 @@
       </c>
       <c r="B46" s="4"/>
       <c r="C46" s="8" t="s">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="D46" s="5">
-        <v>15.24</v>
+        <v>2.87</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1686,16 +1752,16 @@
       </c>
       <c r="B47" s="4"/>
       <c r="C47" s="8" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D47" s="5">
-        <v>24.24</v>
+        <v>2.7</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1704,16 +1770,16 @@
       </c>
       <c r="B48" s="4"/>
       <c r="C48" s="8" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="D48" s="5">
-        <v>1.72</v>
+        <v>5.35</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1722,16 +1788,16 @@
       </c>
       <c r="B49" s="4"/>
       <c r="C49" s="8" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="D49" s="5">
-        <v>8.9600000000000009</v>
+        <v>43.48</v>
       </c>
       <c r="E49" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1740,16 +1806,16 @@
       </c>
       <c r="B50" s="4"/>
       <c r="C50" s="8" t="s">
-        <v>112</v>
+        <v>73</v>
       </c>
       <c r="D50" s="5">
-        <v>17.84</v>
+        <v>7.72</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1758,16 +1824,16 @@
       </c>
       <c r="B51" s="4"/>
       <c r="C51" s="8" t="s">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="D51" s="5">
-        <v>7.72</v>
+        <v>2.04</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1776,31 +1842,31 @@
       </c>
       <c r="B52" s="4"/>
       <c r="C52" s="8" t="s">
-        <v>113</v>
+        <v>78</v>
       </c>
       <c r="D52" s="5">
-        <v>3.97</v>
+        <v>77.760000000000005</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="3">
         <v>52</v>
       </c>
       <c r="B53" s="4"/>
       <c r="C53" s="8" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="D53" s="5">
-        <v>1.1950000000000001</v>
+        <v>40</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="F53" s="4" t="s">
         <v>12</v>
@@ -1812,16 +1878,16 @@
       </c>
       <c r="B54" s="4"/>
       <c r="C54" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D54" s="5">
+        <v>10</v>
+      </c>
+      <c r="E54" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D54" s="7">
-        <v>1000</v>
-      </c>
-      <c r="E54" s="6" t="s">
-        <v>6</v>
-      </c>
       <c r="F54" s="4" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="55" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1830,16 +1896,16 @@
       </c>
       <c r="B55" s="4"/>
       <c r="C55" s="8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D55" s="5">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="56" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1848,16 +1914,16 @@
       </c>
       <c r="B56" s="4"/>
       <c r="C56" s="8" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D56" s="5">
-        <v>500</v>
+        <v>10</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="57" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1866,16 +1932,16 @@
       </c>
       <c r="B57" s="4"/>
       <c r="C57" s="8" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D57" s="5">
-        <v>800</v>
+        <v>40</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="58" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1884,16 +1950,16 @@
       </c>
       <c r="B58" s="4"/>
       <c r="C58" s="8" t="s">
-        <v>23</v>
+        <v>109</v>
       </c>
       <c r="D58" s="5">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1902,16 +1968,16 @@
       </c>
       <c r="B59" s="4"/>
       <c r="C59" s="8" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="D59" s="5">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="60" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1920,16 +1986,16 @@
       </c>
       <c r="B60" s="4"/>
       <c r="C60" s="8" t="s">
-        <v>115</v>
+        <v>19</v>
       </c>
       <c r="D60" s="5">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="61" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1938,16 +2004,16 @@
       </c>
       <c r="B61" s="4"/>
       <c r="C61" s="8" t="s">
-        <v>116</v>
+        <v>20</v>
       </c>
       <c r="D61" s="5">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="62" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1956,16 +2022,16 @@
       </c>
       <c r="B62" s="4"/>
       <c r="C62" s="8" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D62" s="5">
-        <v>5</v>
+        <v>800</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="63" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1974,16 +2040,16 @@
       </c>
       <c r="B63" s="4"/>
       <c r="C63" s="8" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D63" s="5">
-        <v>10</v>
+        <v>500</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="64" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1992,16 +2058,16 @@
       </c>
       <c r="B64" s="4"/>
       <c r="C64" s="8" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D64" s="5">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="65" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2010,16 +2076,16 @@
       </c>
       <c r="B65" s="4"/>
       <c r="C65" s="8" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D65" s="5">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
     </row>
     <row r="66" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2028,16 +2094,16 @@
       </c>
       <c r="B66" s="4"/>
       <c r="C66" s="8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D66" s="5">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
     </row>
     <row r="67" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2046,16 +2112,16 @@
       </c>
       <c r="B67" s="4"/>
       <c r="C67" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D67" s="5">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="68" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2064,16 +2130,16 @@
       </c>
       <c r="B68" s="4"/>
       <c r="C68" s="8" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D68" s="5">
         <v>10</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="69" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2082,16 +2148,16 @@
       </c>
       <c r="B69" s="4"/>
       <c r="C69" s="8" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D69" s="5">
         <v>10</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="70" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2100,16 +2166,16 @@
       </c>
       <c r="B70" s="4"/>
       <c r="C70" s="8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D70" s="5">
         <v>10</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="71" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2118,16 +2184,16 @@
       </c>
       <c r="B71" s="4"/>
       <c r="C71" s="8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D71" s="5">
         <v>10</v>
       </c>
       <c r="E71" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="72" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2136,16 +2202,16 @@
       </c>
       <c r="B72" s="4"/>
       <c r="C72" s="8" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D72" s="5">
         <v>10</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="73" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2154,16 +2220,16 @@
       </c>
       <c r="B73" s="4"/>
       <c r="C73" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D73" s="5">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E73" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="74" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2172,37 +2238,37 @@
       </c>
       <c r="B74" s="4"/>
       <c r="C74" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D74" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="3">
         <v>74</v>
       </c>
       <c r="B75" s="4"/>
       <c r="C75" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D75" s="5">
+        <v>1</v>
+      </c>
+      <c r="E75" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F75" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D75" s="5">
-        <v>6</v>
-      </c>
-      <c r="E75" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="F75" s="4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="76" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="3">
         <v>75</v>
       </c>
@@ -2211,229 +2277,229 @@
         <v>40</v>
       </c>
       <c r="D76" s="5">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="3">
         <v>76</v>
       </c>
       <c r="B77" s="4"/>
       <c r="C77" s="8" t="s">
-        <v>117</v>
+        <v>41</v>
       </c>
       <c r="D77" s="5">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E77" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="3">
         <v>77</v>
       </c>
       <c r="B78" s="4"/>
       <c r="C78" s="8" t="s">
-        <v>118</v>
+        <v>42</v>
       </c>
       <c r="D78" s="5">
-        <v>200</v>
+        <v>4</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F78" s="4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="3">
         <v>78</v>
       </c>
       <c r="B79" s="4"/>
       <c r="C79" s="8" t="s">
-        <v>119</v>
+        <v>43</v>
       </c>
       <c r="D79" s="5">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E79" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F79" s="4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="3">
         <v>79</v>
       </c>
       <c r="B80" s="4"/>
       <c r="C80" s="8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D80" s="5">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="3">
         <v>80</v>
       </c>
       <c r="B81" s="4"/>
       <c r="C81" s="8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D81" s="5">
-        <v>20</v>
+        <v>400</v>
       </c>
       <c r="E81" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="3">
         <v>81</v>
       </c>
       <c r="B82" s="4"/>
       <c r="C82" s="8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D82" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="3">
         <v>82</v>
       </c>
       <c r="B83" s="4"/>
       <c r="C83" s="8" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D83" s="5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E83" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F83" s="4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="3">
         <v>83</v>
       </c>
       <c r="B84" s="4"/>
       <c r="C84" s="8" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="D84" s="5">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="3">
         <v>84</v>
       </c>
       <c r="B85" s="4"/>
       <c r="C85" s="8" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D85" s="5">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E85" s="6" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F85" s="4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="3">
         <v>85</v>
       </c>
       <c r="B86" s="4"/>
       <c r="C86" s="8" t="s">
-        <v>50</v>
+        <v>110</v>
       </c>
       <c r="D86" s="5">
-        <v>1</v>
+        <v>256</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="3">
         <v>86</v>
       </c>
       <c r="B87" s="4"/>
       <c r="C87" s="8" t="s">
-        <v>51</v>
+        <v>111</v>
       </c>
       <c r="D87" s="5">
-        <v>17</v>
+        <v>128</v>
       </c>
       <c r="E87" s="6" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="3">
         <v>87</v>
       </c>
       <c r="B88" s="4"/>
       <c r="C88" s="8" t="s">
-        <v>52</v>
+        <v>112</v>
       </c>
       <c r="D88" s="5">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
     </row>
     <row r="89" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2442,16 +2508,16 @@
       </c>
       <c r="B89" s="4"/>
       <c r="C89" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="D89" s="5">
-        <v>10</v>
+        <v>113</v>
+      </c>
+      <c r="D89" s="7">
+        <v>13486</v>
       </c>
       <c r="E89" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
     </row>
     <row r="90" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2460,16 +2526,16 @@
       </c>
       <c r="B90" s="4"/>
       <c r="C90" s="8" t="s">
-        <v>55</v>
+        <v>114</v>
       </c>
       <c r="D90" s="5">
-        <v>30</v>
+        <v>4.1399999999999997</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>53</v>
+        <v>6</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
     </row>
     <row r="91" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2478,28 +2544,28 @@
       </c>
       <c r="B91" s="4"/>
       <c r="C91" s="8" t="s">
-        <v>56</v>
+        <v>115</v>
       </c>
       <c r="D91" s="5">
-        <v>20</v>
+        <v>27.51</v>
       </c>
       <c r="E91" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="92" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="3">
         <v>91</v>
       </c>
       <c r="B92" s="4"/>
       <c r="C92" s="8" t="s">
-        <v>57</v>
+        <v>116</v>
       </c>
       <c r="D92" s="5">
-        <v>20</v>
+        <v>167.4</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>6</v>
@@ -2508,16 +2574,16 @@
         <v>58</v>
       </c>
     </row>
-    <row r="93" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="3">
         <v>92</v>
       </c>
       <c r="B93" s="4"/>
       <c r="C93" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="D93" s="7">
-        <v>1000</v>
+        <v>117</v>
+      </c>
+      <c r="D93" s="5">
+        <v>0.03</v>
       </c>
       <c r="E93" s="6" t="s">
         <v>6</v>
@@ -2526,184 +2592,184 @@
         <v>58</v>
       </c>
     </row>
-    <row r="94" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="3">
         <v>93</v>
       </c>
       <c r="B94" s="4"/>
       <c r="C94" s="8" t="s">
-        <v>59</v>
+        <v>118</v>
       </c>
       <c r="D94" s="5">
-        <v>1</v>
+        <v>1.59</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="F94" s="4" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="95" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="3">
         <v>94</v>
       </c>
       <c r="B95" s="4"/>
       <c r="C95" s="8" t="s">
-        <v>60</v>
+        <v>119</v>
       </c>
       <c r="D95" s="5">
-        <v>5</v>
+        <v>0.21</v>
       </c>
       <c r="E95" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F95" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="3">
         <v>95</v>
       </c>
       <c r="B96" s="4"/>
       <c r="C96" s="8" t="s">
-        <v>62</v>
+        <v>120</v>
       </c>
       <c r="D96" s="5">
-        <v>5</v>
+        <v>0.42</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F96" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="3">
         <v>96</v>
       </c>
       <c r="B97" s="4"/>
       <c r="C97" s="8" t="s">
-        <v>63</v>
+        <v>121</v>
       </c>
       <c r="D97" s="5">
-        <v>5</v>
+        <v>0.33</v>
       </c>
       <c r="E97" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="98" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="3">
         <v>97</v>
       </c>
       <c r="B98" s="4"/>
       <c r="C98" s="8" t="s">
-        <v>64</v>
+        <v>122</v>
       </c>
       <c r="D98" s="5">
-        <v>10</v>
+        <v>0.72</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="3">
         <v>98</v>
       </c>
       <c r="B99" s="4"/>
       <c r="C99" s="8" t="s">
-        <v>65</v>
+        <v>123</v>
       </c>
       <c r="D99" s="5">
-        <v>10</v>
+        <v>1.62</v>
       </c>
       <c r="E99" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="100" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="3">
         <v>99</v>
       </c>
       <c r="B100" s="4"/>
       <c r="C100" s="8" t="s">
-        <v>66</v>
+        <v>124</v>
       </c>
       <c r="D100" s="5">
-        <v>1</v>
+        <v>3.6</v>
       </c>
       <c r="E100" s="6" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="F100" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="101" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="3">
         <v>100</v>
       </c>
       <c r="B101" s="4"/>
       <c r="C101" s="8" t="s">
-        <v>67</v>
+        <v>125</v>
       </c>
       <c r="D101" s="5">
-        <v>1</v>
+        <v>4.32</v>
       </c>
       <c r="E101" s="6" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="F101" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="102" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="3">
         <v>101</v>
       </c>
       <c r="B102" s="4"/>
       <c r="C102" s="8" t="s">
-        <v>68</v>
+        <v>126</v>
       </c>
       <c r="D102" s="5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F102" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="3">
         <v>102</v>
       </c>
       <c r="B103" s="4"/>
       <c r="C103" s="8" t="s">
-        <v>69</v>
+        <v>127</v>
       </c>
       <c r="D103" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E103" s="6" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F103" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="104" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2712,232 +2778,561 @@
       </c>
       <c r="B104" s="4"/>
       <c r="C104" s="8" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="D104" s="5">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="E104" s="6" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F104" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="105" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="3">
         <v>104</v>
       </c>
       <c r="B105" s="4"/>
       <c r="C105" s="8" t="s">
-        <v>71</v>
+        <v>129</v>
       </c>
       <c r="D105" s="5">
-        <v>12</v>
+        <v>1.62</v>
       </c>
       <c r="E105" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F105" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="106" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="3">
         <v>105</v>
       </c>
       <c r="B106" s="4"/>
       <c r="C106" s="8" t="s">
-        <v>72</v>
+        <v>130</v>
       </c>
       <c r="D106" s="5">
-        <v>40</v>
+        <v>2.5</v>
       </c>
       <c r="E106" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F106" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="107" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="3">
         <v>106</v>
       </c>
       <c r="B107" s="4"/>
       <c r="C107" s="8" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="D107" s="5">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E107" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F107" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="3">
         <v>107</v>
       </c>
       <c r="B108" s="4"/>
       <c r="C108" s="8" t="s">
-        <v>74</v>
+        <v>131</v>
       </c>
       <c r="D108" s="5">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E108" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F108" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="3">
         <v>108</v>
       </c>
       <c r="B109" s="4"/>
       <c r="C109" s="8" t="s">
-        <v>75</v>
+        <v>132</v>
       </c>
       <c r="D109" s="5">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E109" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F109" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="3">
         <v>109</v>
       </c>
       <c r="B110" s="4"/>
       <c r="C110" s="8" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D110" s="5">
-        <v>6</v>
+        <v>9.7200000000000006</v>
       </c>
       <c r="E110" s="6" t="s">
-        <v>77</v>
+        <v>6</v>
       </c>
       <c r="F110" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="111" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="3">
         <v>110</v>
       </c>
       <c r="B111" s="4"/>
       <c r="C111" s="8" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D111" s="5">
-        <v>10</v>
+        <v>19.559999999999999</v>
       </c>
       <c r="E111" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F111" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="112" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="3">
         <v>111</v>
       </c>
       <c r="B112" s="4"/>
       <c r="C112" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="D112" s="7">
-        <v>3757</v>
+        <v>81</v>
+      </c>
+      <c r="D112" s="5">
+        <v>11.43</v>
       </c>
       <c r="E112" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F112" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="3">
         <v>112</v>
       </c>
       <c r="B113" s="4"/>
       <c r="C113" s="8" t="s">
-        <v>122</v>
+        <v>82</v>
       </c>
       <c r="D113" s="5">
-        <v>372.6</v>
+        <v>18</v>
       </c>
       <c r="E113" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F113" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="114" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="3">
         <v>113</v>
       </c>
       <c r="B114" s="4"/>
       <c r="C114" s="8" t="s">
-        <v>123</v>
+        <v>83</v>
       </c>
       <c r="D114" s="5">
-        <v>745.5</v>
+        <v>3.3</v>
       </c>
       <c r="E114" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F114" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="115" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="3">
         <v>114</v>
       </c>
       <c r="B115" s="4"/>
       <c r="C115" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="D115" s="7">
-        <v>1712</v>
+        <v>84</v>
+      </c>
+      <c r="D115" s="5">
+        <v>1.41</v>
       </c>
       <c r="E115" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F115" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="116" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="3">
         <v>115</v>
       </c>
       <c r="B116" s="4"/>
       <c r="C116" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="D116" s="5">
+        <v>38.64</v>
+      </c>
+      <c r="E116" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F116" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A117" s="3">
+        <v>116</v>
+      </c>
+      <c r="B117" s="4"/>
+      <c r="C117" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="D117" s="5">
+        <v>4.08</v>
+      </c>
+      <c r="E117" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F117" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A118" s="3">
+        <v>117</v>
+      </c>
+      <c r="B118" s="4"/>
+      <c r="C118" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="D118" s="5">
+        <v>58.32</v>
+      </c>
+      <c r="E118" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F118" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A119" s="3">
+        <v>118</v>
+      </c>
+      <c r="B119" s="4"/>
+      <c r="C119" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="D119" s="5">
+        <v>5</v>
+      </c>
+      <c r="E119" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F119" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A120" s="3">
+        <v>119</v>
+      </c>
+      <c r="B120" s="4"/>
+      <c r="C120" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="D120" s="5">
+        <v>6</v>
+      </c>
+      <c r="E120" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F120" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A121" s="3">
+        <v>120</v>
+      </c>
+      <c r="B121" s="4"/>
+      <c r="C121" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="D121" s="5">
+        <v>12</v>
+      </c>
+      <c r="E121" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F121" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A122" s="3">
+        <v>121</v>
+      </c>
+      <c r="B122" s="4"/>
+      <c r="C122" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="D122" s="5">
+        <v>36</v>
+      </c>
+      <c r="E122" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F122" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A123" s="3">
+        <v>122</v>
+      </c>
+      <c r="B123" s="4"/>
+      <c r="C123" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="D123" s="5">
+        <v>12</v>
+      </c>
+      <c r="E123" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F123" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A124" s="3">
+        <v>123</v>
+      </c>
+      <c r="B124" s="4"/>
+      <c r="C124" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="D124" s="5">
+        <v>6</v>
+      </c>
+      <c r="E124" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F124" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A125" s="3">
+        <v>124</v>
+      </c>
+      <c r="B125" s="4"/>
+      <c r="C125" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="D125" s="5">
+        <v>3</v>
+      </c>
+      <c r="E125" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F125" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A126" s="3">
         <v>125</v>
       </c>
-      <c r="D116" s="7">
-        <v>1250.96</v>
-      </c>
-      <c r="E116" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="F116" s="4" t="s">
-        <v>79</v>
+      <c r="B126" s="4"/>
+      <c r="C126" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="D126" s="5">
+        <v>72</v>
+      </c>
+      <c r="E126" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F126" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A127" s="3">
+        <v>126</v>
+      </c>
+      <c r="B127" s="4"/>
+      <c r="C127" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="D127" s="5">
+        <v>3</v>
+      </c>
+      <c r="E127" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F127" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A128" s="3">
+        <v>127</v>
+      </c>
+      <c r="B128" s="4"/>
+      <c r="C128" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="D128" s="5">
+        <v>4</v>
+      </c>
+      <c r="E128" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F128" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A129" s="3">
+        <v>128</v>
+      </c>
+      <c r="B129" s="4"/>
+      <c r="C129" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="D129" s="5">
+        <v>5</v>
+      </c>
+      <c r="E129" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F129" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A130" s="3">
+        <v>129</v>
+      </c>
+      <c r="B130" s="4"/>
+      <c r="C130" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="D130" s="5">
+        <v>9.9</v>
+      </c>
+      <c r="E130" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F130" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A131" s="3">
+        <v>130</v>
+      </c>
+      <c r="B131" s="4"/>
+      <c r="C131" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="D131" s="5">
+        <v>1</v>
+      </c>
+      <c r="E131" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F131" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A132" s="3">
+        <v>131</v>
+      </c>
+      <c r="B132" s="4"/>
+      <c r="C132" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="D132" s="5">
+        <v>3</v>
+      </c>
+      <c r="E132" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F132" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A133" s="3">
+        <v>132</v>
+      </c>
+      <c r="B133" s="4"/>
+      <c r="C133" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="D133" s="5">
+        <v>3</v>
+      </c>
+      <c r="E133" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F133" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A134" s="3">
+        <v>133</v>
+      </c>
+      <c r="B134" s="4"/>
+      <c r="C134" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="D134" s="5">
+        <v>1</v>
+      </c>
+      <c r="E134" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F134" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" ht="11.45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C139" s="1" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new menu and About
</commit_message>
<xml_diff>
--- a/public/procurement.xlsx
+++ b/public/procurement.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lka\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7475053D-1628-47ED-96A9-1CD5DA872060}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE7ADDF4-5CE3-44B5-817A-59A9D04ACD1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4755" yWindow="3270" windowWidth="23730" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="170">
   <si>
     <t>№ п/п</t>
   </si>
@@ -54,9 +54,6 @@
     <t>Труба D89х12 Ст.09Г2 ГОСТ 19281-89</t>
   </si>
   <si>
-    <t>не исп. Труба D89х6 ГОСТ 8732-78/ Ст.20 ГОСТ 8731-87</t>
-  </si>
-  <si>
     <t>ЛГУП-7315</t>
   </si>
   <si>
@@ -66,24 +63,24 @@
     <t>ЛГУП-7331</t>
   </si>
   <si>
+    <t>Каска строительная белая</t>
+  </si>
+  <si>
+    <t>шт.</t>
+  </si>
+  <si>
     <t>Каска строительная оранжевая Исток</t>
   </si>
   <si>
-    <t>шт.</t>
+    <t>Ветошь</t>
+  </si>
+  <si>
+    <t>Маркер белый</t>
   </si>
   <si>
     <t>Маркер по металлу черный тонкий</t>
   </si>
   <si>
-    <t>Ветошь</t>
-  </si>
-  <si>
-    <t>Маркер белый</t>
-  </si>
-  <si>
-    <t>Каска строительная белая</t>
-  </si>
-  <si>
     <t>Маркер по металлу белый</t>
   </si>
   <si>
@@ -105,30 +102,33 @@
     <t>Маркер  краска красный по металлу</t>
   </si>
   <si>
+    <t>Ключ комбинированные омедненные 41</t>
+  </si>
+  <si>
+    <t>ЛГУП-7332</t>
+  </si>
+  <si>
+    <t>Ключ комбинированные омедненные 36</t>
+  </si>
+  <si>
+    <t>Ключ комбинированные омедненные 30</t>
+  </si>
+  <si>
+    <t>Ключ комбинированные омедненные 24</t>
+  </si>
+  <si>
+    <t>Трещетка ключ 1/2</t>
+  </si>
+  <si>
     <t>Гайковерт</t>
   </si>
   <si>
-    <t>ЛГУП-7332</t>
-  </si>
-  <si>
-    <t>Ключ комбинированные омедненные 41</t>
-  </si>
-  <si>
-    <t>Ключ комбинированные омедненные 36</t>
-  </si>
-  <si>
-    <t>Ключ комбинированные омедненные 30</t>
-  </si>
-  <si>
-    <t>Ключ комбинированные омедненные 24</t>
-  </si>
-  <si>
-    <t>Трещетка ключ 1/2</t>
-  </si>
-  <si>
     <t>Ножницы по металлу</t>
   </si>
   <si>
+    <t>Резак</t>
+  </si>
+  <si>
     <t>Ключи обмедненные</t>
   </si>
   <si>
@@ -138,9 +138,6 @@
     <t>Кувалда 1 кг.</t>
   </si>
   <si>
-    <t>Резак</t>
-  </si>
-  <si>
     <t>Эмаль ПФ-115 желтая (22кг)</t>
   </si>
   <si>
@@ -150,12 +147,12 @@
     <t>Эмаль ПФ 115 красная 1,8кг STATUS /6</t>
   </si>
   <si>
+    <t>Эмаль ПФ-115 коричневая (25 кг), шт</t>
+  </si>
+  <si>
     <t>Растворитель 646 (5л)</t>
   </si>
   <si>
-    <t>Эмаль ПФ-115 коричневая (25 кг), шт</t>
-  </si>
-  <si>
     <t>Растворитель Р-4 /кг/</t>
   </si>
   <si>
@@ -177,73 +174,109 @@
     <t>НТУП-017968</t>
   </si>
   <si>
+    <t>Строительство Отмоски и цоколя(без учета материала)</t>
+  </si>
+  <si>
+    <t>ЛГУП-7342</t>
+  </si>
+  <si>
+    <t>Строительство Промышленного пола(без учета материала)</t>
+  </si>
+  <si>
     <t>Строительство фундамента лестничной клетки(без учета материала)</t>
   </si>
   <si>
-    <t>ЛГУП-7342</t>
-  </si>
-  <si>
-    <t>Строительство Промышленного пола(без учета материала)</t>
-  </si>
-  <si>
-    <t>Строительство Отмоски и цоколя(без учета материала)</t>
-  </si>
-  <si>
-    <t>ЛГУП-7346</t>
-  </si>
-  <si>
     <t>м</t>
   </si>
   <si>
     <t>ЛГУП-7347</t>
   </si>
   <si>
-    <t>ЛГУП-7348</t>
-  </si>
-  <si>
     <t>ЛГУП-7349</t>
   </si>
   <si>
-    <t>ЛГУП-7351</t>
-  </si>
-  <si>
-    <t>ЛГУП-7352</t>
-  </si>
-  <si>
-    <t>ЛГУП-7353</t>
-  </si>
-  <si>
-    <t>ЛГУП-7355</t>
+    <t>ЛГУП-7356</t>
   </si>
   <si>
     <t>Фланец 25-40-11-1-E-09Г2С-IV ГОСТ 33259-2015</t>
   </si>
   <si>
-    <t>ЛГУП-7356</t>
-  </si>
-  <si>
     <t>ЛГУП-7357</t>
   </si>
   <si>
-    <t>Услуги по договору номер 7</t>
-  </si>
-  <si>
-    <t>АХУП-000649</t>
-  </si>
-  <si>
     <t>ЛГУП-7365</t>
   </si>
   <si>
-    <t>ЛГУП-7366</t>
+    <t>ЛГУП-7367</t>
   </si>
   <si>
     <t>л (дм3)</t>
   </si>
   <si>
-    <t>ЛГУП-7367</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
+    <t>ЛГУП-7374</t>
+  </si>
+  <si>
+    <t>ЛГУП-7375</t>
+  </si>
+  <si>
+    <t>ЛГУП-7378</t>
+  </si>
+  <si>
+    <t>Окно 1100х900 мм /шт/ (ПВХ-профили морозостойкого исп) рал9016 белый</t>
+  </si>
+  <si>
+    <t>Бордюры тротуарные</t>
+  </si>
+  <si>
+    <t>ЛГУП-7380</t>
+  </si>
+  <si>
+    <t>Бетон М-250</t>
+  </si>
+  <si>
+    <t>м3</t>
+  </si>
+  <si>
+    <t>Туя Смарагд высота 1,5 м</t>
+  </si>
+  <si>
+    <t>ЛГУП-7381</t>
+  </si>
+  <si>
+    <t>Укладка бордюрного камня 340 м</t>
+  </si>
+  <si>
+    <t>ед</t>
+  </si>
+  <si>
+    <t>ЛГУП-7382</t>
+  </si>
+  <si>
+    <t>Наконечник НКИ 6,0-6</t>
+  </si>
+  <si>
+    <t>ЛГУП-7384</t>
+  </si>
+  <si>
+    <t>Труба 377х10, 09Г2с / тн</t>
+  </si>
+  <si>
+    <t>т</t>
+  </si>
+  <si>
+    <t>НТУП-017990</t>
+  </si>
+  <si>
+    <t>Труба 720х12 ст.09Г2С/кг</t>
+  </si>
+  <si>
+    <t>Костюм москитный</t>
+  </si>
+  <si>
+    <t>ЛГУП-7386</t>
+  </si>
+  <si>
+    <t>Спрей от комаров "Москитол"</t>
   </si>
   <si>
     <t>Труба D25х7 ст.10Г2 ГОСТ 8733-74</t>
@@ -285,90 +318,45 @@
     <t>Труба D273х10 ГОСТ 8732-78/ 09Г2С ГОСТ 30564-98</t>
   </si>
   <si>
-    <t>Труба D57х4 ГОСТ 8732-78/ 09Г2С ГОСТ 8731-74</t>
+    <t>Труба D219х5 Ст.20 ГОСТ 1050-88</t>
+  </si>
+  <si>
+    <t>Труба D140х25 Ст.20 ГОСТ 8732-78</t>
+  </si>
+  <si>
+    <t>Труба D146х22 Ст.20 ГОСТ 8732-78</t>
+  </si>
+  <si>
+    <t>Труба D57х5 ГОСТ 8732-78/09Г2С ГОСТ 8731-74</t>
   </si>
   <si>
     <t>Труба D480х16 10Г2 ГОСТ 8731-74</t>
   </si>
   <si>
-    <t>Труба D57х5 ГОСТ 8732-78/09Г2С ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>Труба D110х16 ГОСТ 8734-75/ Ст.20 ГОСТ 8733-74</t>
-  </si>
-  <si>
-    <t>Труба D73х9 Ст20 ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>не исп. Труба D83х10 Ст20 ГОСТ 8731-74</t>
-  </si>
-  <si>
     <t>Труба D42х10 Ст.09Г2С ГОСТ 19281-89</t>
   </si>
   <si>
-    <t>Труба D140х25 Ст.20 ГОСТ 8732-78</t>
-  </si>
-  <si>
-    <t>Труба D159х18 Ст.20 ГОСТ 8732-78</t>
+    <t>Труба D108х11 Ст. 20Х13 ГОСТ 5632-72</t>
   </si>
   <si>
     <t>Труба D83*10 Ст.12Х18Н10Т ГОСТ 5949-72</t>
   </si>
   <si>
-    <t>Труба D89х8 Ст.35 ГОСТ 1050-80</t>
-  </si>
-  <si>
-    <t>Труба 25х3,2 ГОСТ 3262-75 (D33,5)</t>
+    <t>Труба D65х14 Ст.20 ГОСТ 8731-74</t>
   </si>
   <si>
     <t>Труба D83х9 Ст.40Х ГОСТ 8731-87</t>
   </si>
   <si>
-    <t>Труба D219х5 Ст.20 ГОСТ 1050-88</t>
-  </si>
-  <si>
-    <t>Труба D146х22 Ст.20 ГОСТ 8732-78</t>
-  </si>
-  <si>
-    <t>Труба D108х11 Ст. 20Х13 ГОСТ 5632-72</t>
-  </si>
-  <si>
-    <t>Труба D121х6 ГОСТ 8732-78 /Ст. 20 ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>Труба D14х2 09Г2С ГОСТ 8733-74</t>
-  </si>
-  <si>
-    <t>Труба D180х25 ГОСТ 8732-78 / 09Г2С ГОСТ 19281-89</t>
-  </si>
-  <si>
-    <t>Труба D65х14 Ст.20 ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>Труба D194х14 В20 ГОСТ 8732-78</t>
-  </si>
-  <si>
-    <t>Труба D83*9 Ст.20 ГОСТ 1050-88</t>
-  </si>
-  <si>
     <t>Маркер черный</t>
   </si>
   <si>
     <t>Фумлента</t>
   </si>
   <si>
-    <t>Гайка М30х1,5-6Н.09Г2С.019 ГОСТ 5915-70</t>
-  </si>
-  <si>
-    <t>Болт 1.2 М30х1000</t>
-  </si>
-  <si>
     <t>Кабель ВВГнг(А)-LS-ХЛ 4x1,5 d10,2мм</t>
   </si>
   <si>
-    <t>Гайка М16-6Н.09Г2С (оцинк.) ГОСТ 9064-75</t>
-  </si>
-  <si>
     <t>Круг ДКРН D48 НД БрАЖ9-4 ГОСТ 1628-78</t>
   </si>
   <si>
@@ -405,70 +393,148 @@
     <t>Шестигранник S=46 Ст.45 ГОСТ 535-88</t>
   </si>
   <si>
-    <t>Отвод 45-89х8-09Г2С ГОСТ 17375-2001</t>
-  </si>
-  <si>
-    <t>Тройник 20х3-09Г2С ГОСТ 17376-2001</t>
-  </si>
-  <si>
-    <t>Светильник взрывозащищенный ДБП 09-15-001 УХЛ1 ExdllBT6G IP65</t>
-  </si>
-  <si>
-    <t>Труба D14х3 ГОСТ 8732-78/ 09Г2С ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>Труба D20х3 ГОСТ 8732-78/ 09Г2С  ГОСТ 8731-74</t>
-  </si>
-  <si>
     <t>Фланец 1-250-40 09Г2С ГОСТ 12821-80</t>
   </si>
   <si>
     <t>Фланец 2-50-40 09Г2С ГОСТ 12821-80</t>
   </si>
   <si>
+    <t>Шпилька АМ16-6gx80 ГОСТ 9066-75</t>
+  </si>
+  <si>
     <t>Болт М20-6gх30.58 (S30) ГОСТ 7798-70</t>
   </si>
   <si>
+    <t>Шайба 8 65Г 019 ГОСТ 6402-70</t>
+  </si>
+  <si>
+    <t>Шпилька АМ30-6gх180.60.35.III.4.019 ГОСТ 9066-75</t>
+  </si>
+  <si>
+    <t>Шайба 8.01.019 ГОСТ 11371-78</t>
+  </si>
+  <si>
     <t>Заклепка 4х8.31 ГОСТ 10299-80</t>
   </si>
   <si>
-    <t>Шпилька АМ30-6gх180.60.35.III.4.019 ГОСТ 9066-75</t>
-  </si>
-  <si>
-    <t>Шпилька АМ16-6gx80 ГОСТ 9066-75</t>
-  </si>
-  <si>
-    <t>Шайба 8.01.019 ГОСТ 11371-78</t>
-  </si>
-  <si>
-    <t>Шайба 8 65Г 019 ГОСТ 6402-70</t>
+    <t>Шайба 16 ГОСТ 6958-78</t>
   </si>
   <si>
     <t>Шайба 30.Ст3сп3.II.4.019 ГОСТ 9065-75</t>
   </si>
   <si>
-    <t>Шайба 16 ГОСТ 6958-78</t>
-  </si>
-  <si>
-    <t>Фланец х-300-40 (заготовка-поковка Ст.08Х18Н10 гр.IV КП195 ГОСТ 8479-70)</t>
+    <t>Краска-спрей SABOTAGE (желтая)</t>
+  </si>
+  <si>
+    <t>Краска-спрей SABOTAGE 39(черный)</t>
+  </si>
+  <si>
+    <t>Прокладка Б-50-40-ПМБ ГОСТ 15180-86</t>
+  </si>
+  <si>
+    <t>Разбавитель Procore Universal Thinner</t>
+  </si>
+  <si>
+    <t>Грунт-эмаль Дюропокс ДТМ 70 цвет серый (наружка)</t>
   </si>
   <si>
     <t>Растворитель Р-4 ГОСТ 7827-74</t>
   </si>
   <si>
-    <t>Грунт-эмаль Дюропокс ДТМ 70 цвет серый (наружка)</t>
-  </si>
-  <si>
-    <t>Краска-спрей SABOTAGE (желтая)</t>
-  </si>
-  <si>
-    <t>Разбавитель Procore Universal Thinner</t>
-  </si>
-  <si>
-    <t>Прокладка Б-50-40-ПМБ ГОСТ 15180-86</t>
-  </si>
-  <si>
-    <t>Краска-спрей SABOTAGE 39(черный)</t>
+    <t>Шпилька резьбовая оцинкованная M12 DIN 975</t>
+  </si>
+  <si>
+    <t>Заклепка 4,8х10</t>
+  </si>
+  <si>
+    <t>Заклепка 4,8х8 оцинкованная</t>
+  </si>
+  <si>
+    <t>Саморез для сэндвич панелей 5,5х25</t>
+  </si>
+  <si>
+    <t>Болт М20х50 ГОСТ15591-70</t>
+  </si>
+  <si>
+    <t>Гайка М10.5 019 ГОСТ 5927-70</t>
+  </si>
+  <si>
+    <t>Гайка М20-6Н ГОСТ 5915-70</t>
+  </si>
+  <si>
+    <t>Саморез кровельный 5,5х19 RAL9016 (белый)</t>
+  </si>
+  <si>
+    <t>Саморез кровельный 5,5х25 RAL 2007(оранж)</t>
+  </si>
+  <si>
+    <t>Саморез кровельный 5,5х25 RAL9016 (белый)</t>
+  </si>
+  <si>
+    <t>Саморез кровельный 6,3*70</t>
+  </si>
+  <si>
+    <t>Саморез металл/металл 4,2х19</t>
+  </si>
+  <si>
+    <t>Шпилька 2М16х1,5-6gx120.109.40Х.26 ГОСТ 22034-76</t>
+  </si>
+  <si>
+    <t>Шпилька М16-6gх260.58.35Х.026 ГОСТ 22042-76</t>
+  </si>
+  <si>
+    <t>Труба профильная 50х25х3 Ст.3сп5 ГОСТ 8645-68</t>
+  </si>
+  <si>
+    <t>Труба профильная 50х25х4 09Г2С ГОСТ 8645-68</t>
+  </si>
+  <si>
+    <t>Труба профильная 60х60х5 ГОСТ 8639-82/09Г2С ГОСТ 19281-2014</t>
+  </si>
+  <si>
+    <t>Профиль 50х25х3 ст.09Г2С ГОСТ 30245-2012</t>
+  </si>
+  <si>
+    <t>Труба D89х6 ГОСТ 8732-78/ 09Г2С ГОСТ 8731-74</t>
+  </si>
+  <si>
+    <t>Труба профильная 80х80х5 ГОСТ 30245-2003/ 325-09Г2С ГОСТ 19281-2014</t>
+  </si>
+  <si>
+    <t>Уголок 25х25х3 ГОСТ 8509-93/ Ст.3 ГОСТ 535-2005</t>
+  </si>
+  <si>
+    <t>Уголок 50х50х3 ГОСТ 8509-93/09Г2С ГОСТ 19281-2014</t>
+  </si>
+  <si>
+    <t>Уголок 63х63х4 ГОСТ 8509-93 / 09Г2С ГОСТ5521-93</t>
+  </si>
+  <si>
+    <t>Уголок 63х63х5 ГОСТ 8509-93/ Ст.09Г2С ГОСТ 19281-89</t>
+  </si>
+  <si>
+    <t>Швеллер 16П ГОСТ 8240-97 / 09Г2С ГОСТ19281-2014</t>
+  </si>
+  <si>
+    <t>Дверь левая с доводчиком 1900х1000 мм(ВхШ) полотно RAL 7036 (серый)/ коробка (RAL 7036) (серый)</t>
+  </si>
+  <si>
+    <t>Дверь левая с доводчиком 2000х1000 мм(ВхШ) полотно RAL 7036 (серый)/ коробка (RAL 7036) (серый)</t>
+  </si>
+  <si>
+    <t>Эмаль ПФ-115 белая</t>
+  </si>
+  <si>
+    <t>Сольвент ГОСТ 10214-78</t>
+  </si>
+  <si>
+    <t>Гайка с насечкой М6 СМ100600</t>
+  </si>
+  <si>
+    <t>Газоанализатор взрывозащищенный СГОЭС (метан) 1Ex d IIC T4 Gb, IP67 Ур1. 10%, ур.2 50% НКПР</t>
+  </si>
+  <si>
+    <t>Провод ПУГВ 1х6,0 ЖЗ ГОСТ 31947-2012</t>
   </si>
 </sst>
 </file>
@@ -905,13 +971,13 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F139"/>
+  <dimension ref="A1:F138"/>
   <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="11.45" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.1640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="46.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="63.6640625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="56.1640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16" style="1" customWidth="1"/>
     <col min="5" max="5" width="13" style="1" customWidth="1"/>
     <col min="6" max="6" width="14.5" style="1" customWidth="1"/>
   </cols>
@@ -942,7 +1008,7 @@
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="8" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="D2" s="5">
         <v>20.399999999999999</v>
@@ -960,7 +1026,7 @@
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="8" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="D3" s="5">
         <v>48.6</v>
@@ -978,7 +1044,7 @@
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="8" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="D4" s="7">
         <v>2000</v>
@@ -996,7 +1062,7 @@
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="8" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="D5" s="7">
         <v>4500</v>
@@ -1032,7 +1098,7 @@
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="8" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="D7" s="5">
         <v>233.85</v>
@@ -1050,7 +1116,7 @@
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="8" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="D8" s="5">
         <v>291.60000000000002</v>
@@ -1068,7 +1134,7 @@
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="8" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="D9" s="5">
         <v>95.25</v>
@@ -1086,7 +1152,7 @@
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="8" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="D10" s="5">
         <v>97.8</v>
@@ -1104,7 +1170,7 @@
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="8" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="D11" s="5">
         <v>57.15</v>
@@ -1122,7 +1188,7 @@
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="8" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="D12" s="5">
         <v>33.75</v>
@@ -1140,7 +1206,7 @@
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="8" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="D13" s="5">
         <v>16.5</v>
@@ -1158,7 +1224,7 @@
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="8" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="D14" s="5">
         <v>7.05</v>
@@ -1176,7 +1242,7 @@
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="8" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="D15" s="5">
         <v>193.2</v>
@@ -1194,16 +1260,16 @@
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D16" s="5">
+        <v>17.84</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F16" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="D16" s="5">
-        <v>26.52</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1212,16 +1278,16 @@
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="8" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="D17" s="5">
-        <v>0.84</v>
+        <v>24.24</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1230,16 +1296,16 @@
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="8" t="s">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="D18" s="5">
-        <v>51.52</v>
+        <v>11.48</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1248,16 +1314,16 @@
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="8" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="D19" s="5">
-        <v>146.4</v>
+        <v>2.87</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1266,7 +1332,7 @@
       </c>
       <c r="B20" s="4"/>
       <c r="C20" s="8" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="D20" s="5">
         <v>1.52</v>
@@ -1275,7 +1341,7 @@
         <v>6</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1284,16 +1350,16 @@
       </c>
       <c r="B21" s="4"/>
       <c r="C21" s="8" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="D21" s="5">
-        <v>11.2</v>
+        <v>36.6</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1302,16 +1368,16 @@
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="8" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D22" s="5">
-        <v>5.68</v>
+        <v>146.4</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1320,16 +1386,16 @@
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="8" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="D23" s="5">
-        <v>2.52</v>
+        <v>5.16</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1338,16 +1404,16 @@
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="8" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="D24" s="5">
-        <v>13.76</v>
+        <v>3.56</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1356,16 +1422,16 @@
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="8" t="s">
-        <v>78</v>
+        <v>104</v>
       </c>
       <c r="D25" s="5">
-        <v>19.440000000000001</v>
+        <v>0.43</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1374,16 +1440,16 @@
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="8" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="D26" s="5">
-        <v>6.06</v>
+        <v>6.64</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1392,16 +1458,16 @@
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="8" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="D27" s="5">
-        <v>2.2400000000000002</v>
+        <v>13.76</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1410,412 +1476,412 @@
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="8" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="D28" s="5">
-        <v>0.43</v>
+        <v>3.97</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="3">
         <v>28</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="8" t="s">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="D29" s="5">
-        <v>5.16</v>
+        <v>40</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="3">
         <v>29</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="8" t="s">
-        <v>96</v>
+        <v>12</v>
       </c>
       <c r="D30" s="5">
-        <v>6.45</v>
+        <v>5</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="3">
         <v>30</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="8" t="s">
-        <v>87</v>
+        <v>14</v>
       </c>
       <c r="D31" s="5">
-        <v>36.6</v>
+        <v>10</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="3">
         <v>31</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="8" t="s">
-        <v>97</v>
+        <v>15</v>
       </c>
       <c r="D32" s="5">
-        <v>1.1950000000000001</v>
+        <v>10</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="3">
         <v>32</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="8" t="s">
-        <v>98</v>
+        <v>16</v>
       </c>
       <c r="D33" s="5">
-        <v>3.97</v>
+        <v>40</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="3">
         <v>33</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="8" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="D34" s="5">
-        <v>17.84</v>
+        <v>5</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3">
         <v>34</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="8" t="s">
-        <v>94</v>
+        <v>17</v>
       </c>
       <c r="D35" s="5">
-        <v>8.9600000000000009</v>
+        <v>20</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="3">
         <v>35</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="8" t="s">
-        <v>95</v>
+        <v>18</v>
       </c>
       <c r="D36" s="5">
-        <v>1.72</v>
+        <v>20</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="3">
         <v>36</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="8" t="s">
-        <v>93</v>
+        <v>19</v>
       </c>
       <c r="D37" s="5">
-        <v>24.24</v>
+        <v>15</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="3">
         <v>37</v>
       </c>
       <c r="B38" s="4"/>
       <c r="C38" s="8" t="s">
-        <v>81</v>
+        <v>20</v>
       </c>
       <c r="D38" s="5">
-        <v>15.24</v>
+        <v>800</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="3">
         <v>38</v>
       </c>
       <c r="B39" s="4"/>
       <c r="C39" s="8" t="s">
-        <v>100</v>
+        <v>22</v>
       </c>
       <c r="D39" s="5">
-        <v>11.48</v>
+        <v>500</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="3">
         <v>39</v>
       </c>
       <c r="B40" s="4"/>
       <c r="C40" s="8" t="s">
-        <v>101</v>
+        <v>24</v>
       </c>
       <c r="D40" s="5">
-        <v>3.56</v>
+        <v>40</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="3">
         <v>40</v>
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="8" t="s">
-        <v>102</v>
+        <v>25</v>
       </c>
       <c r="D41" s="5">
-        <v>10.8</v>
+        <v>10</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="3">
         <v>41</v>
       </c>
       <c r="B42" s="4"/>
       <c r="C42" s="8" t="s">
-        <v>103</v>
+        <v>27</v>
       </c>
       <c r="D42" s="5">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="3">
         <v>42</v>
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="8" t="s">
-        <v>104</v>
+        <v>28</v>
       </c>
       <c r="D43" s="5">
-        <v>21.4</v>
+        <v>10</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="3">
         <v>43</v>
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="8" t="s">
-        <v>83</v>
+        <v>29</v>
       </c>
       <c r="D44" s="5">
-        <v>8.8000000000000007</v>
+        <v>10</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="3">
         <v>44</v>
       </c>
       <c r="B45" s="4"/>
       <c r="C45" s="8" t="s">
-        <v>105</v>
+        <v>30</v>
       </c>
       <c r="D45" s="5">
-        <v>6.64</v>
+        <v>10</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="3">
         <v>45</v>
       </c>
       <c r="B46" s="4"/>
       <c r="C46" s="8" t="s">
-        <v>100</v>
+        <v>31</v>
       </c>
       <c r="D46" s="5">
-        <v>2.87</v>
+        <v>2</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="3">
         <v>46</v>
       </c>
       <c r="B47" s="4"/>
       <c r="C47" s="8" t="s">
-        <v>102</v>
+        <v>32</v>
       </c>
       <c r="D47" s="5">
-        <v>2.7</v>
+        <v>10</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="3">
         <v>47</v>
       </c>
       <c r="B48" s="4"/>
       <c r="C48" s="8" t="s">
-        <v>104</v>
+        <v>33</v>
       </c>
       <c r="D48" s="5">
-        <v>5.35</v>
+        <v>4</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="3">
         <v>48</v>
       </c>
       <c r="B49" s="4"/>
       <c r="C49" s="8" t="s">
-        <v>106</v>
+        <v>34</v>
       </c>
       <c r="D49" s="5">
-        <v>43.48</v>
+        <v>10</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="3">
         <v>49</v>
       </c>
       <c r="B50" s="4"/>
       <c r="C50" s="8" t="s">
-        <v>73</v>
+        <v>36</v>
       </c>
       <c r="D50" s="5">
-        <v>7.72</v>
+        <v>6</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1824,16 +1890,16 @@
       </c>
       <c r="B51" s="4"/>
       <c r="C51" s="8" t="s">
-        <v>107</v>
+        <v>37</v>
       </c>
       <c r="D51" s="5">
-        <v>2.04</v>
+        <v>1</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1842,124 +1908,124 @@
       </c>
       <c r="B52" s="4"/>
       <c r="C52" s="8" t="s">
-        <v>78</v>
+        <v>39</v>
       </c>
       <c r="D52" s="5">
-        <v>77.760000000000005</v>
+        <v>12</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="3">
         <v>52</v>
       </c>
       <c r="B53" s="4"/>
       <c r="C53" s="8" t="s">
-        <v>108</v>
+        <v>40</v>
       </c>
       <c r="D53" s="5">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="3">
         <v>53</v>
       </c>
       <c r="B54" s="4"/>
       <c r="C54" s="8" t="s">
-        <v>13</v>
+        <v>41</v>
       </c>
       <c r="D54" s="5">
         <v>10</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="3">
         <v>54</v>
       </c>
       <c r="B55" s="4"/>
       <c r="C55" s="8" t="s">
-        <v>15</v>
+        <v>42</v>
       </c>
       <c r="D55" s="5">
         <v>20</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="3">
         <v>55</v>
       </c>
       <c r="B56" s="4"/>
       <c r="C56" s="8" t="s">
-        <v>16</v>
+        <v>43</v>
       </c>
       <c r="D56" s="5">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="3">
         <v>56</v>
       </c>
       <c r="B57" s="4"/>
       <c r="C57" s="8" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="D57" s="5">
-        <v>40</v>
+        <v>400</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="3">
         <v>57</v>
       </c>
       <c r="B58" s="4"/>
       <c r="C58" s="8" t="s">
-        <v>109</v>
+        <v>47</v>
       </c>
       <c r="D58" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1968,16 +2034,16 @@
       </c>
       <c r="B59" s="4"/>
       <c r="C59" s="8" t="s">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="D59" s="5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
     </row>
     <row r="60" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1986,16 +2052,16 @@
       </c>
       <c r="B60" s="4"/>
       <c r="C60" s="8" t="s">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="D60" s="5">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
     </row>
     <row r="61" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2004,16 +2070,16 @@
       </c>
       <c r="B61" s="4"/>
       <c r="C61" s="8" t="s">
-        <v>20</v>
+        <v>52</v>
       </c>
       <c r="D61" s="5">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
     </row>
     <row r="62" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2022,232 +2088,232 @@
       </c>
       <c r="B62" s="4"/>
       <c r="C62" s="8" t="s">
-        <v>21</v>
+        <v>109</v>
       </c>
       <c r="D62" s="5">
-        <v>800</v>
+        <v>40</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="3">
         <v>62</v>
       </c>
       <c r="B63" s="4"/>
       <c r="C63" s="8" t="s">
-        <v>23</v>
+        <v>110</v>
       </c>
       <c r="D63" s="5">
-        <v>500</v>
+        <v>4.1399999999999997</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="3">
         <v>63</v>
       </c>
       <c r="B64" s="4"/>
       <c r="C64" s="8" t="s">
-        <v>25</v>
+        <v>111</v>
       </c>
       <c r="D64" s="5">
-        <v>40</v>
+        <v>27.51</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="3">
         <v>64</v>
       </c>
       <c r="B65" s="4"/>
       <c r="C65" s="8" t="s">
-        <v>26</v>
+        <v>112</v>
       </c>
       <c r="D65" s="5">
-        <v>2</v>
+        <v>167.4</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="3">
         <v>65</v>
       </c>
       <c r="B66" s="4"/>
       <c r="C66" s="8" t="s">
-        <v>28</v>
+        <v>113</v>
       </c>
       <c r="D66" s="5">
-        <v>10</v>
+        <v>0.03</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="3">
         <v>66</v>
       </c>
       <c r="B67" s="4"/>
       <c r="C67" s="8" t="s">
-        <v>29</v>
+        <v>114</v>
       </c>
       <c r="D67" s="5">
-        <v>10</v>
+        <v>1.59</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="3">
         <v>67</v>
       </c>
       <c r="B68" s="4"/>
       <c r="C68" s="8" t="s">
-        <v>30</v>
+        <v>115</v>
       </c>
       <c r="D68" s="5">
-        <v>10</v>
+        <v>0.21</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="3">
         <v>68</v>
       </c>
       <c r="B69" s="4"/>
       <c r="C69" s="8" t="s">
-        <v>31</v>
+        <v>116</v>
       </c>
       <c r="D69" s="5">
-        <v>10</v>
+        <v>0.42</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="3">
         <v>69</v>
       </c>
       <c r="B70" s="4"/>
       <c r="C70" s="8" t="s">
-        <v>32</v>
+        <v>117</v>
       </c>
       <c r="D70" s="5">
-        <v>10</v>
+        <v>0.33</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="3">
         <v>70</v>
       </c>
       <c r="B71" s="4"/>
       <c r="C71" s="8" t="s">
-        <v>33</v>
+        <v>118</v>
       </c>
       <c r="D71" s="5">
-        <v>10</v>
+        <v>0.72</v>
       </c>
       <c r="E71" s="6" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="3">
         <v>71</v>
       </c>
       <c r="B72" s="4"/>
       <c r="C72" s="8" t="s">
-        <v>34</v>
+        <v>119</v>
       </c>
       <c r="D72" s="5">
-        <v>10</v>
+        <v>1.62</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="3">
         <v>72</v>
       </c>
       <c r="B73" s="4"/>
       <c r="C73" s="8" t="s">
-        <v>36</v>
+        <v>120</v>
       </c>
       <c r="D73" s="5">
-        <v>6</v>
+        <v>3.6</v>
       </c>
       <c r="E73" s="6" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="3">
         <v>73</v>
       </c>
       <c r="B74" s="4"/>
       <c r="C74" s="8" t="s">
-        <v>37</v>
+        <v>121</v>
       </c>
       <c r="D74" s="5">
-        <v>4</v>
+        <v>4.32</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
     </row>
     <row r="75" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2256,16 +2322,16 @@
       </c>
       <c r="B75" s="4"/>
       <c r="C75" s="8" t="s">
-        <v>38</v>
+        <v>122</v>
       </c>
       <c r="D75" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E75" s="6" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>39</v>
+        <v>56</v>
       </c>
     </row>
     <row r="76" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2274,16 +2340,16 @@
       </c>
       <c r="B76" s="4"/>
       <c r="C76" s="8" t="s">
-        <v>40</v>
+        <v>123</v>
       </c>
       <c r="D76" s="5">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>39</v>
+        <v>56</v>
       </c>
     </row>
     <row r="77" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2292,16 +2358,16 @@
       </c>
       <c r="B77" s="4"/>
       <c r="C77" s="8" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="D77" s="5">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E77" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>39</v>
+        <v>56</v>
       </c>
     </row>
     <row r="78" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2310,16 +2376,16 @@
       </c>
       <c r="B78" s="4"/>
       <c r="C78" s="8" t="s">
-        <v>42</v>
+        <v>89</v>
       </c>
       <c r="D78" s="5">
-        <v>4</v>
+        <v>58.32</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="F78" s="4" t="s">
-        <v>39</v>
+        <v>58</v>
       </c>
     </row>
     <row r="79" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2328,16 +2394,16 @@
       </c>
       <c r="B79" s="4"/>
       <c r="C79" s="8" t="s">
-        <v>43</v>
+        <v>84</v>
       </c>
       <c r="D79" s="5">
-        <v>20</v>
+        <v>4.08</v>
       </c>
       <c r="E79" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F79" s="4" t="s">
-        <v>39</v>
+        <v>58</v>
       </c>
     </row>
     <row r="80" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2346,16 +2412,16 @@
       </c>
       <c r="B80" s="4"/>
       <c r="C80" s="8" t="s">
-        <v>44</v>
+        <v>93</v>
       </c>
       <c r="D80" s="5">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>45</v>
+        <v>58</v>
       </c>
     </row>
     <row r="81" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2364,16 +2430,16 @@
       </c>
       <c r="B81" s="4"/>
       <c r="C81" s="8" t="s">
-        <v>46</v>
+        <v>92</v>
       </c>
       <c r="D81" s="5">
-        <v>400</v>
+        <v>11.43</v>
       </c>
       <c r="E81" s="6" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
     </row>
     <row r="82" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2382,124 +2448,124 @@
       </c>
       <c r="B82" s="4"/>
       <c r="C82" s="8" t="s">
-        <v>48</v>
+        <v>91</v>
       </c>
       <c r="D82" s="5">
-        <v>4</v>
+        <v>19.559999999999999</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="3">
         <v>82</v>
       </c>
       <c r="B83" s="4"/>
       <c r="C83" s="8" t="s">
-        <v>50</v>
+        <v>124</v>
       </c>
       <c r="D83" s="5">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E83" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F83" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="3">
         <v>83</v>
       </c>
       <c r="B84" s="4"/>
       <c r="C84" s="8" t="s">
-        <v>52</v>
+        <v>125</v>
       </c>
       <c r="D84" s="5">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="3">
         <v>84</v>
       </c>
       <c r="B85" s="4"/>
       <c r="C85" s="8" t="s">
-        <v>53</v>
+        <v>126</v>
       </c>
       <c r="D85" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E85" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F85" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="3">
         <v>85</v>
       </c>
       <c r="B86" s="4"/>
       <c r="C86" s="8" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="D86" s="5">
-        <v>256</v>
+        <v>36</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="3">
         <v>86</v>
       </c>
       <c r="B87" s="4"/>
       <c r="C87" s="8" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="D87" s="5">
-        <v>128</v>
+        <v>6</v>
       </c>
       <c r="E87" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="3">
         <v>87</v>
       </c>
       <c r="B88" s="4"/>
       <c r="C88" s="8" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="D88" s="5">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="89" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2508,16 +2574,16 @@
       </c>
       <c r="B89" s="4"/>
       <c r="C89" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="D89" s="7">
-        <v>13486</v>
+        <v>130</v>
+      </c>
+      <c r="D89" s="5">
+        <v>3</v>
       </c>
       <c r="E89" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="90" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2526,250 +2592,250 @@
       </c>
       <c r="B90" s="4"/>
       <c r="C90" s="8" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
       <c r="D90" s="5">
-        <v>4.1399999999999997</v>
+        <v>72</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="3">
         <v>90</v>
       </c>
       <c r="B91" s="4"/>
       <c r="C91" s="8" t="s">
-        <v>115</v>
+        <v>132</v>
       </c>
       <c r="D91" s="5">
-        <v>27.51</v>
+        <v>1</v>
       </c>
       <c r="E91" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="92" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="3">
         <v>91</v>
       </c>
       <c r="B92" s="4"/>
       <c r="C92" s="8" t="s">
-        <v>116</v>
+        <v>133</v>
       </c>
       <c r="D92" s="5">
-        <v>167.4</v>
+        <v>1</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="3">
         <v>92</v>
       </c>
       <c r="B93" s="4"/>
       <c r="C93" s="8" t="s">
-        <v>117</v>
+        <v>134</v>
       </c>
       <c r="D93" s="5">
-        <v>0.03</v>
+        <v>3</v>
       </c>
       <c r="E93" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="3">
         <v>93</v>
       </c>
       <c r="B94" s="4"/>
       <c r="C94" s="8" t="s">
-        <v>118</v>
+        <v>135</v>
       </c>
       <c r="D94" s="5">
-        <v>1.59</v>
+        <v>3</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>6</v>
+        <v>61</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="3">
         <v>94</v>
       </c>
       <c r="B95" s="4"/>
       <c r="C95" s="8" t="s">
-        <v>119</v>
+        <v>136</v>
       </c>
       <c r="D95" s="5">
-        <v>0.21</v>
+        <v>9.9</v>
       </c>
       <c r="E95" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F95" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="3">
         <v>95</v>
       </c>
       <c r="B96" s="4"/>
       <c r="C96" s="8" t="s">
-        <v>120</v>
+        <v>137</v>
       </c>
       <c r="D96" s="5">
-        <v>0.42</v>
+        <v>5</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>6</v>
+        <v>61</v>
       </c>
       <c r="F96" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="3">
         <v>96</v>
       </c>
       <c r="B97" s="4"/>
       <c r="C97" s="8" t="s">
-        <v>121</v>
+        <v>138</v>
       </c>
       <c r="D97" s="5">
-        <v>0.33</v>
+        <v>1</v>
       </c>
       <c r="E97" s="6" t="s">
-        <v>6</v>
+        <v>53</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="98" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="3">
         <v>97</v>
       </c>
       <c r="B98" s="4"/>
       <c r="C98" s="8" t="s">
-        <v>122</v>
+        <v>139</v>
       </c>
       <c r="D98" s="5">
-        <v>0.72</v>
+        <v>30</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="3">
         <v>98</v>
       </c>
       <c r="B99" s="4"/>
       <c r="C99" s="8" t="s">
-        <v>123</v>
+        <v>140</v>
       </c>
       <c r="D99" s="5">
-        <v>1.62</v>
+        <v>30</v>
       </c>
       <c r="E99" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="100" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="3">
         <v>99</v>
       </c>
       <c r="B100" s="4"/>
       <c r="C100" s="8" t="s">
-        <v>124</v>
+        <v>141</v>
       </c>
       <c r="D100" s="5">
-        <v>3.6</v>
+        <v>416</v>
       </c>
       <c r="E100" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F100" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="101" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="3">
         <v>100</v>
       </c>
       <c r="B101" s="4"/>
       <c r="C101" s="8" t="s">
-        <v>125</v>
+        <v>142</v>
       </c>
       <c r="D101" s="5">
-        <v>4.32</v>
+        <v>6</v>
       </c>
       <c r="E101" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F101" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="102" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="3">
         <v>101</v>
       </c>
       <c r="B102" s="4"/>
       <c r="C102" s="8" t="s">
-        <v>126</v>
+        <v>143</v>
       </c>
       <c r="D102" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F102" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="3">
         <v>102</v>
       </c>
       <c r="B103" s="4"/>
       <c r="C103" s="8" t="s">
-        <v>127</v>
+        <v>144</v>
       </c>
       <c r="D103" s="5">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E103" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F103" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="104" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2778,430 +2844,430 @@
       </c>
       <c r="B104" s="4"/>
       <c r="C104" s="8" t="s">
-        <v>128</v>
+        <v>145</v>
       </c>
       <c r="D104" s="5">
-        <v>1</v>
+        <v>250</v>
       </c>
       <c r="E104" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F104" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="3">
         <v>104</v>
       </c>
       <c r="B105" s="4"/>
       <c r="C105" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="D105" s="5">
-        <v>1.62</v>
+        <v>146</v>
+      </c>
+      <c r="D105" s="7">
+        <v>1100</v>
       </c>
       <c r="E105" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F105" s="4" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="106" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="3">
         <v>105</v>
       </c>
       <c r="B106" s="4"/>
       <c r="C106" s="8" t="s">
-        <v>130</v>
+        <v>147</v>
       </c>
       <c r="D106" s="5">
-        <v>2.5</v>
+        <v>400</v>
       </c>
       <c r="E106" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F106" s="4" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="107" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="3">
         <v>106</v>
       </c>
       <c r="B107" s="4"/>
       <c r="C107" s="8" t="s">
-        <v>63</v>
+        <v>148</v>
       </c>
       <c r="D107" s="5">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E107" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F107" s="4" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="3">
         <v>107</v>
       </c>
       <c r="B108" s="4"/>
       <c r="C108" s="8" t="s">
-        <v>131</v>
+        <v>149</v>
       </c>
       <c r="D108" s="5">
-        <v>3</v>
+        <v>120</v>
       </c>
       <c r="E108" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F108" s="4" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="3">
         <v>108</v>
       </c>
       <c r="B109" s="4"/>
       <c r="C109" s="8" t="s">
-        <v>132</v>
+        <v>150</v>
       </c>
       <c r="D109" s="5">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="E109" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F109" s="4" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="3">
         <v>109</v>
       </c>
       <c r="B110" s="4"/>
       <c r="C110" s="8" t="s">
-        <v>74</v>
+        <v>151</v>
       </c>
       <c r="D110" s="5">
-        <v>9.7200000000000006</v>
+        <v>2</v>
       </c>
       <c r="E110" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F110" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="111" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="3">
         <v>110</v>
       </c>
       <c r="B111" s="4"/>
       <c r="C111" s="8" t="s">
-        <v>80</v>
+        <v>152</v>
       </c>
       <c r="D111" s="5">
-        <v>19.559999999999999</v>
+        <v>79.44</v>
       </c>
       <c r="E111" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F111" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="112" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="3">
         <v>111</v>
       </c>
       <c r="B112" s="4"/>
       <c r="C112" s="8" t="s">
-        <v>81</v>
+        <v>153</v>
       </c>
       <c r="D112" s="5">
-        <v>11.43</v>
+        <v>32.659999999999997</v>
       </c>
       <c r="E112" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F112" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="3">
         <v>112</v>
       </c>
       <c r="B113" s="4"/>
       <c r="C113" s="8" t="s">
-        <v>82</v>
+        <v>154</v>
       </c>
       <c r="D113" s="5">
-        <v>18</v>
+        <v>279.08</v>
       </c>
       <c r="E113" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F113" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="114" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="3">
         <v>113</v>
       </c>
       <c r="B114" s="4"/>
       <c r="C114" s="8" t="s">
-        <v>83</v>
+        <v>155</v>
       </c>
       <c r="D114" s="5">
-        <v>3.3</v>
+        <v>50.8</v>
       </c>
       <c r="E114" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F114" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="115" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="3">
         <v>114</v>
       </c>
       <c r="B115" s="4"/>
       <c r="C115" s="8" t="s">
-        <v>84</v>
+        <v>156</v>
       </c>
       <c r="D115" s="5">
-        <v>1.41</v>
+        <v>7.8</v>
       </c>
       <c r="E115" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F115" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="116" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="3">
         <v>115</v>
       </c>
       <c r="B116" s="4"/>
       <c r="C116" s="8" t="s">
-        <v>85</v>
+        <v>157</v>
       </c>
       <c r="D116" s="5">
-        <v>38.64</v>
+        <v>916.44</v>
       </c>
       <c r="E116" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F116" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="117" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="3">
         <v>116</v>
       </c>
       <c r="B117" s="4"/>
       <c r="C117" s="8" t="s">
-        <v>73</v>
+        <v>158</v>
       </c>
       <c r="D117" s="5">
-        <v>4.08</v>
+        <v>12</v>
       </c>
       <c r="E117" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F117" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="118" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="3">
         <v>117</v>
       </c>
       <c r="B118" s="4"/>
       <c r="C118" s="8" t="s">
-        <v>78</v>
+        <v>159</v>
       </c>
       <c r="D118" s="5">
-        <v>58.32</v>
+        <v>21</v>
       </c>
       <c r="E118" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F118" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="119" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="3">
         <v>118</v>
       </c>
       <c r="B119" s="4"/>
       <c r="C119" s="8" t="s">
-        <v>66</v>
+        <v>160</v>
       </c>
       <c r="D119" s="5">
-        <v>5</v>
+        <v>55.64</v>
       </c>
       <c r="E119" s="6" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="F119" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="120" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="3">
         <v>119</v>
       </c>
       <c r="B120" s="4"/>
       <c r="C120" s="8" t="s">
-        <v>133</v>
+        <v>161</v>
       </c>
       <c r="D120" s="5">
-        <v>6</v>
+        <v>41.21</v>
       </c>
       <c r="E120" s="6" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="F120" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="3">
         <v>120</v>
       </c>
       <c r="B121" s="4"/>
       <c r="C121" s="8" t="s">
-        <v>134</v>
+        <v>162</v>
       </c>
       <c r="D121" s="5">
-        <v>12</v>
+        <v>308.89</v>
       </c>
       <c r="E121" s="6" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="F121" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="122" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="3">
         <v>121</v>
       </c>
       <c r="B122" s="4"/>
       <c r="C122" s="8" t="s">
-        <v>135</v>
+        <v>163</v>
       </c>
       <c r="D122" s="5">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="E122" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F122" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="123" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="3">
         <v>122</v>
       </c>
       <c r="B123" s="4"/>
       <c r="C123" s="8" t="s">
-        <v>136</v>
+        <v>65</v>
       </c>
       <c r="D123" s="5">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E123" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F123" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="124" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="3">
         <v>123</v>
       </c>
       <c r="B124" s="4"/>
       <c r="C124" s="8" t="s">
-        <v>137</v>
+        <v>164</v>
       </c>
       <c r="D124" s="5">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E124" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F124" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="125" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="3">
         <v>124</v>
       </c>
       <c r="B125" s="4"/>
       <c r="C125" s="8" t="s">
-        <v>138</v>
+        <v>165</v>
       </c>
       <c r="D125" s="5">
-        <v>3</v>
+        <v>0.5</v>
       </c>
       <c r="E125" s="6" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="F125" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="126" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="3">
         <v>125</v>
       </c>
       <c r="B126" s="4"/>
       <c r="C126" s="8" t="s">
-        <v>139</v>
+        <v>166</v>
       </c>
       <c r="D126" s="5">
-        <v>72</v>
+        <v>0.7</v>
       </c>
       <c r="E126" s="6" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="F126" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="127" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="3">
         <v>126</v>
       </c>
       <c r="B127" s="4"/>
       <c r="C127" s="8" t="s">
-        <v>140</v>
+        <v>66</v>
       </c>
       <c r="D127" s="5">
-        <v>3</v>
+        <v>340</v>
       </c>
       <c r="E127" s="6" t="s">
-        <v>11</v>
+        <v>53</v>
       </c>
       <c r="F127" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="128" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3210,16 +3276,16 @@
       </c>
       <c r="B128" s="4"/>
       <c r="C128" s="8" t="s">
-        <v>141</v>
+        <v>68</v>
       </c>
       <c r="D128" s="5">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E128" s="6" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="F128" s="4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="129" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3228,34 +3294,34 @@
       </c>
       <c r="B129" s="4"/>
       <c r="C129" s="8" t="s">
-        <v>142</v>
+        <v>70</v>
       </c>
       <c r="D129" s="5">
-        <v>5</v>
+        <v>150</v>
       </c>
       <c r="E129" s="6" t="s">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="F129" s="4" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="130" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="3">
         <v>129</v>
       </c>
       <c r="B130" s="4"/>
       <c r="C130" s="8" t="s">
-        <v>143</v>
+        <v>72</v>
       </c>
       <c r="D130" s="5">
-        <v>9.9</v>
+        <v>1</v>
       </c>
       <c r="E130" s="6" t="s">
-        <v>6</v>
+        <v>73</v>
       </c>
       <c r="F130" s="4" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="131" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3264,16 +3330,16 @@
       </c>
       <c r="B131" s="4"/>
       <c r="C131" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="D131" s="5">
-        <v>1</v>
+        <v>75</v>
+      </c>
+      <c r="D131" s="7">
+        <v>1200</v>
       </c>
       <c r="E131" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F131" s="4" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="132" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3282,16 +3348,16 @@
       </c>
       <c r="B132" s="4"/>
       <c r="C132" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="D132" s="5">
-        <v>3</v>
+        <v>167</v>
+      </c>
+      <c r="D132" s="7">
+        <v>1280</v>
       </c>
       <c r="E132" s="6" t="s">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="F132" s="4" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="133" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3300,16 +3366,16 @@
       </c>
       <c r="B133" s="4"/>
       <c r="C133" s="8" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
       <c r="D133" s="5">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E133" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F133" s="4" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="134" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3318,21 +3384,88 @@
       </c>
       <c r="B134" s="4"/>
       <c r="C134" s="8" t="s">
-        <v>147</v>
+        <v>169</v>
       </c>
       <c r="D134" s="5">
-        <v>1</v>
+        <v>360</v>
       </c>
       <c r="E134" s="6" t="s">
-        <v>11</v>
+        <v>53</v>
       </c>
       <c r="F134" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="139" spans="1:6" ht="11.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C139" s="1" t="s">
-        <v>72</v>
+        <v>76</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A135" s="3">
+        <v>134</v>
+      </c>
+      <c r="B135" s="4"/>
+      <c r="C135" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="D135" s="5">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="E135" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="F135" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A136" s="3">
+        <v>135</v>
+      </c>
+      <c r="B136" s="4"/>
+      <c r="C136" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="D136" s="7">
+        <v>1000</v>
+      </c>
+      <c r="E136" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F136" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A137" s="3">
+        <v>136</v>
+      </c>
+      <c r="B137" s="4"/>
+      <c r="C137" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="D137" s="5">
+        <v>3</v>
+      </c>
+      <c r="E137" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F137" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A138" s="3">
+        <v>137</v>
+      </c>
+      <c r="B138" s="4"/>
+      <c r="C138" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="D138" s="5">
+        <v>30</v>
+      </c>
+      <c r="E138" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F138" s="4" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new About, Products and Careers
</commit_message>
<xml_diff>
--- a/public/procurement.xlsx
+++ b/public/procurement.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lka\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D235D03F-DE49-4340-8B94-92219173260F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71C15226-ACA9-414C-A703-D16BBC0C5C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4755" yWindow="3270" windowWidth="23730" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="162">
   <si>
     <t>№ п/п</t>
   </si>
@@ -45,274 +45,181 @@
     <t>Примечание</t>
   </si>
   <si>
+    <t>шт</t>
+  </si>
+  <si>
+    <t>ЛГУП-7413</t>
+  </si>
+  <si>
     <t>кг</t>
   </si>
   <si>
-    <t>ЛГУП-7287</t>
-  </si>
-  <si>
-    <t>Труба D89х12 Ст.09Г2 ГОСТ 19281-89</t>
+    <t>Маркер  краска красный по металлу</t>
+  </si>
+  <si>
+    <t>шт.</t>
+  </si>
+  <si>
+    <t>ЛГУП-7331</t>
+  </si>
+  <si>
+    <t>Каска строительная белая</t>
+  </si>
+  <si>
+    <t>Перчатки х/б трикотажные 5 нитей 10 класс с ПВХ -Камаз 426</t>
+  </si>
+  <si>
+    <t>пара</t>
+  </si>
+  <si>
+    <t>Перчатки с латесным покрытием</t>
+  </si>
+  <si>
+    <t>пар</t>
+  </si>
+  <si>
+    <t>Маркер белый</t>
+  </si>
+  <si>
+    <t>Ветошь</t>
   </si>
   <si>
     <t>Каска строительная оранжевая Исток</t>
   </si>
   <si>
-    <t>шт.</t>
-  </si>
-  <si>
-    <t>ЛГУП-7331</t>
-  </si>
-  <si>
-    <t>шт</t>
-  </si>
-  <si>
-    <t>Ветошь</t>
-  </si>
-  <si>
-    <t>Маркер белый</t>
-  </si>
-  <si>
-    <t>Каска строительная белая</t>
-  </si>
-  <si>
-    <t>Маркер  краска красный по металлу</t>
-  </si>
-  <si>
     <t>Маркер по металлу черный тонкий</t>
   </si>
   <si>
     <t>Маркер по металлу белый</t>
   </si>
   <si>
-    <t>Перчатки х/б трикотажные 5 нитей 10 класс с ПВХ -Камаз 426</t>
-  </si>
-  <si>
-    <t>пара</t>
-  </si>
-  <si>
-    <t>Перчатки с латесным покрытием</t>
-  </si>
-  <si>
-    <t>пар</t>
-  </si>
-  <si>
     <t>Огнетушитель ОП-8</t>
   </si>
   <si>
+    <t>Гайковерт</t>
+  </si>
+  <si>
+    <t>ЛГУП-7332</t>
+  </si>
+  <si>
+    <t>Ключ комбинированные омедненные 41</t>
+  </si>
+  <si>
+    <t>Ключи обмедненные</t>
+  </si>
+  <si>
+    <t>набор</t>
+  </si>
+  <si>
+    <t>Ключ комбинированные омедненные 36</t>
+  </si>
+  <si>
+    <t>Ключ комбинированные омедненные 30</t>
+  </si>
+  <si>
+    <t>Ключ комбинированные омедненные 24</t>
+  </si>
+  <si>
+    <t>Трещетка ключ 1/2</t>
+  </si>
+  <si>
     <t>Кувалда 1 кг.</t>
   </si>
   <si>
-    <t>ЛГУП-7332</t>
-  </si>
-  <si>
     <t>Резак</t>
   </si>
   <si>
     <t>Ножницы по металлу</t>
   </si>
   <si>
-    <t>Трещетка ключ 1/2</t>
-  </si>
-  <si>
-    <t>Ключ комбинированные омедненные 24</t>
-  </si>
-  <si>
-    <t>Ключ комбинированные омедненные 30</t>
-  </si>
-  <si>
-    <t>Ключ комбинированные омедненные 36</t>
-  </si>
-  <si>
-    <t>Ключ комбинированные омедненные 41</t>
-  </si>
-  <si>
-    <t>Гайковерт</t>
-  </si>
-  <si>
-    <t>Ключи обмедненные</t>
-  </si>
-  <si>
-    <t>набор</t>
-  </si>
-  <si>
-    <t>Дробемет для швеллера с конвейерной сеткой</t>
-  </si>
-  <si>
-    <t>ЛГУП-7338</t>
-  </si>
-  <si>
-    <t>Строительство фундамента лестничной клетки(без учета материала)</t>
-  </si>
-  <si>
-    <t>ЛГУП-7342</t>
-  </si>
-  <si>
-    <t>Строительство Промышленного пола(без учета материала)</t>
-  </si>
-  <si>
-    <t>Строительство Отмоски и цоколя(без учета материала)</t>
-  </si>
-  <si>
-    <t>ЛГУП-7357</t>
-  </si>
-  <si>
-    <t>л (дм3)</t>
-  </si>
-  <si>
-    <t>ЛГУП-7367</t>
-  </si>
-  <si>
-    <t>ЛГУП-7375</t>
-  </si>
-  <si>
-    <t>ЛГУП-7378</t>
-  </si>
-  <si>
-    <t>Окно 1100х900 мм /шт/ (ПВХ-профили морозостойкого исп) рал9016 белый</t>
-  </si>
-  <si>
-    <t>Труба 377х10, 09Г2с / тн</t>
-  </si>
-  <si>
-    <t>т</t>
-  </si>
-  <si>
-    <t>НТУП-017990</t>
-  </si>
-  <si>
-    <t>Труба 720х12 ст.09Г2С/кг</t>
-  </si>
-  <si>
-    <t>Лист Б-ПН 2,0 ГОСТ 19903-80/ 20 ГОСТ 16523-89</t>
-  </si>
-  <si>
-    <t>ЛГУП-7391</t>
+    <t>ЛГУП-7428</t>
+  </si>
+  <si>
+    <t>Днище 820х14-09Г2С ГОСТ 6533-78</t>
+  </si>
+  <si>
+    <t>Днище 720х12 ст09Г2С ГОСТ 6533-78</t>
+  </si>
+  <si>
+    <t>Днище 377х10 09Г2С ГОСТ 6533-78</t>
+  </si>
+  <si>
+    <t>Распылитель Тесла Трибо</t>
+  </si>
+  <si>
+    <t>ЛГУП-7429</t>
+  </si>
+  <si>
+    <t>ЛГУП-7445</t>
+  </si>
+  <si>
+    <t>ЛГУП-7446</t>
+  </si>
+  <si>
+    <t>ЛГУП-7447</t>
   </si>
   <si>
     <t>м</t>
   </si>
   <si>
-    <t>Средство для чистки сантехники Антиржавчина Grass WC-gel 0,75 л</t>
-  </si>
-  <si>
-    <t>ЛГУП-7408</t>
-  </si>
-  <si>
-    <t>Средство чистящее для стекол Grass Clean Glass голубая лагуна 600мл</t>
-  </si>
-  <si>
-    <t>Метла</t>
-  </si>
-  <si>
-    <t>Средство для чистки универсальное Пемоксоль санитарный 500г.</t>
-  </si>
-  <si>
-    <t>Туалетная бумага</t>
-  </si>
-  <si>
-    <t>Средство для мытья пола 5 л</t>
-  </si>
-  <si>
-    <t>Салфетка для уборки и полировки микрофибра 25х25см 5шт</t>
-  </si>
-  <si>
-    <t>компл</t>
-  </si>
-  <si>
-    <t>Карандаш</t>
-  </si>
-  <si>
-    <t>ЛГУП-7409</t>
-  </si>
-  <si>
-    <t>Ручка</t>
-  </si>
-  <si>
-    <t>Папка-вкладыш с расширением (на 250 листов) ПВХ 180мкм</t>
-  </si>
-  <si>
-    <t>Файл-вкладыш А4 прозрачный гладкий 100 шт. в упаковке</t>
-  </si>
-  <si>
-    <t>Фланец 100-40-11-1-E-09Г2С ГОСТ 33259-2015</t>
-  </si>
-  <si>
-    <t>ЛГУП-7410</t>
-  </si>
-  <si>
-    <t>Фланец 80-40-11-1-F-09Г2С ГОСТ 33259-2015</t>
-  </si>
-  <si>
-    <t>Фланец 80-40-11-1-E-09Г2С-IV ГОСТ 33259-2015</t>
-  </si>
-  <si>
-    <t>Фланец 50-40-11-1-Е 09ГСФ-IV ГОСТ 33259-2015 (п/ф)</t>
-  </si>
-  <si>
-    <t>Фланец 150-40-11-1-F-09Г2С ГОСТ 33259-2015</t>
-  </si>
-  <si>
-    <t>Фланец 50-40-11-1-F-09Г2С ГОСТ 33259-2015</t>
-  </si>
-  <si>
-    <t>Фланец 150-40-11-1-Е-09Г2С-IV ГОСТ 33259-2015 (п/ф из поковки)</t>
-  </si>
-  <si>
-    <t>Фланец 100-40-11-1-F-09Г2С ГОСТ 33259-2015</t>
-  </si>
-  <si>
-    <t>Валик велюр тканный беж. 6х15х60мм ворс 4мм (2шт/уп) 1190062</t>
-  </si>
-  <si>
-    <t>АХУП-000663</t>
-  </si>
-  <si>
-    <t>ЛГУП-7413</t>
-  </si>
-  <si>
-    <t>ЛГУП-7415</t>
-  </si>
-  <si>
-    <t>м2</t>
-  </si>
-  <si>
-    <t>Труба D25х7 ст.10Г2 ГОСТ 8733-74</t>
-  </si>
-  <si>
-    <t>Уголок 40х40х3 ГОСТ 8509-93/ Ст3пс ГОСТ 535-88</t>
-  </si>
-  <si>
-    <t>Труба D377х12 ст.09Г2С-К50 ГОСТ 8731-78</t>
-  </si>
-  <si>
-    <t>Труба D720х12 Ст.09Г2С-К50 ГОСТ 20295-85</t>
-  </si>
-  <si>
-    <t>Труба D159х10 ГОСТ 8732-78/ 09Г2С ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>Труба D219х18 Ст.09ГС ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>Труба D219х4 ГОСТ 8734-75/ Ст.В20 ГОСТ 8733-74</t>
-  </si>
-  <si>
-    <t>Труба D89х8 ГОСТ 872-78 В 09Г2С ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>Труба D68х12 ст.265-09Г2С-4 ГОСТ 19281-89</t>
-  </si>
-  <si>
-    <t>Труба D57х6 ГОСТ 8732-78/ 09Г2С ГОСТ 4543-2016</t>
-  </si>
-  <si>
-    <t>Труба D38х9 Ст.09Г2С ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>Труба D34х4 Ст.09Г2С ГОСТ8733-75</t>
-  </si>
-  <si>
-    <t>Труба D273х10 ГОСТ 8732-78/ 09Г2С ГОСТ 30564-98</t>
+    <t>ЛГУП-7448</t>
+  </si>
+  <si>
+    <t>Перемычка и наконечник НКИ 6-0-6</t>
+  </si>
+  <si>
+    <t>Держатель проводника Rd8</t>
+  </si>
+  <si>
+    <t>МИП-24 исп.20 (МИП-24-2/П5-Р-RS), до двух АКБ 12 В 17 Ач</t>
+  </si>
+  <si>
+    <t>Блок коммутации 24В БК-24-RS485-01</t>
+  </si>
+  <si>
+    <t>Индикатор положения поплавка ИПП 01.00.000</t>
+  </si>
+  <si>
+    <t>ЛГУП-7450</t>
+  </si>
+  <si>
+    <t>ЛГУП-7451</t>
+  </si>
+  <si>
+    <t>Обогреватель взрывозащищенный ОВЭ-4 ТК-1.0 1 кВт, 220В, 50 Гц.</t>
+  </si>
+  <si>
+    <t>Коробка клеммная К-СП 16.18.09 24/20П 4КВе-Л-М20(А)-4КВе-Л-М20(В) 1ЕхеLLCGbXT6, ip66, 160х180х90</t>
+  </si>
+  <si>
+    <t>Коробка соед взрывозащК-СП 16.26.09 24/31 П 8КВе-Л-М20(А) 8КВе-Л-М20(В) 1ЕхеLLCGb ip66, 160х260х90</t>
+  </si>
+  <si>
+    <t>К-СП 16.26.09 32/26П 6КВе-Л-М20(А)-6КВе-Л-М20(В)-1КВе-Л-М20(D) 1ExeLLCGbXT6 ip66 120х260х90</t>
+  </si>
+  <si>
+    <t>Газоанализатор взрывозащищенный СГОЭС 1Ex d IIC T4 Gb, IP67</t>
+  </si>
+  <si>
+    <t>Палитра цветов</t>
+  </si>
+  <si>
+    <t>ЛГУП-7454</t>
+  </si>
+  <si>
+    <t>ЛГУП-7457</t>
+  </si>
+  <si>
+    <t>ЛГУП-7460</t>
+  </si>
+  <si>
+    <t>ЛГУП-7462</t>
+  </si>
+  <si>
+    <t>Кольцо 350-360-58-2-2 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Смола ЭД-20 ГОСТ 10587-84</t>
   </si>
   <si>
     <t>Маркер черный</t>
@@ -321,130 +228,289 @@
     <t>Фумлента</t>
   </si>
   <si>
-    <t>Разбавитель Procore Universal Thinner</t>
-  </si>
-  <si>
-    <t>Растворитель Р-4 ГОСТ 7827-74</t>
-  </si>
-  <si>
-    <t>Краска-спрей SABOTAGE (желтая)</t>
-  </si>
-  <si>
-    <t>Краска-спрей SABOTAGE 39(черный)</t>
-  </si>
-  <si>
-    <t>Прокладка Б-50-40-ПМБ ГОСТ 15180-86</t>
-  </si>
-  <si>
-    <t>Грунт-эмаль Дюропокс ДТМ 70 цвет серый (наружка)</t>
-  </si>
-  <si>
-    <t>Труба профильная 50х25х4 09Г2С ГОСТ 8645-68</t>
-  </si>
-  <si>
-    <t>Труба D89х6 ГОСТ 8732-78/ 09Г2С ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>Труба профильная 50х25х3 Ст.3сп5 ГОСТ 8645-68</t>
-  </si>
-  <si>
-    <t>Труба профильная 60х60х5 ГОСТ 8639-82/09Г2С ГОСТ 19281-2014</t>
-  </si>
-  <si>
-    <t>Швеллер 16П ГОСТ 8240-97 / 09Г2С ГОСТ19281-2014</t>
-  </si>
-  <si>
-    <t>Уголок 63х63х5 ГОСТ 8509-93/ Ст.09Г2С ГОСТ 19281-89</t>
-  </si>
-  <si>
-    <t>Уголок 63х63х4 ГОСТ 8509-93 / 09Г2С ГОСТ5521-93</t>
-  </si>
-  <si>
-    <t>Уголок 50х50х3 ГОСТ 8509-93/09Г2С ГОСТ 19281-2014</t>
-  </si>
-  <si>
-    <t>Профиль 50х25х3 ст.09Г2С ГОСТ 30245-2012</t>
-  </si>
-  <si>
-    <t>Уголок 25х25х3 ГОСТ 8509-93/ Ст.3 ГОСТ 535-2005</t>
-  </si>
-  <si>
-    <t>Труба профильная 80х80х5 ГОСТ 30245-2003/ 325-09Г2С ГОСТ 19281-2014</t>
-  </si>
-  <si>
-    <t>Сольвент ГОСТ 10214-78</t>
-  </si>
-  <si>
-    <t>Эмаль ПФ-115 белая</t>
-  </si>
-  <si>
-    <t>Дверь левая с доводчиком 1900х1000 мм(ВхШ) полотно RAL 7036 (серый)/ коробка (RAL 7036) (серый)</t>
-  </si>
-  <si>
-    <t>Дверь левая с доводчиком 2000х1000 мм(ВхШ) полотно RAL 7036 (серый)/ коробка (RAL 7036) (серый)</t>
-  </si>
-  <si>
-    <t>Лента ПВХ облицовочная декоративн самоклеющаяся, шириной 19мм</t>
-  </si>
-  <si>
-    <t>Плита П-А,I,М,Ш,Е1(600х450х19) ГОСТ 10632-89</t>
-  </si>
-  <si>
-    <t>Лист гладкий 0,5 1250х2500мм RAL полиуретан 7036(Серый)</t>
-  </si>
-  <si>
-    <t>Лист чечевица В-К-ПУ-3,0 Ст.09Г2С ГОСТ 8568-77</t>
-  </si>
-  <si>
-    <t>Лист оцинкованный ОЦ Б-ПН-НО-0,5 ГОСТ 19904-90/ОН-КР ГОСТ 14918-80 (кг)</t>
-  </si>
-  <si>
-    <t>Лист S=5 Ст.3 ГОСТ 380-2005</t>
-  </si>
-  <si>
-    <t>Лист S=4 ст.09Г2С ГОСТ 14637-89</t>
-  </si>
-  <si>
-    <t>Лист S=3,0 ГОСТ 19903-74/09Г2С ГОСТ 19281-89</t>
-  </si>
-  <si>
-    <t>Лист S=2 ГОСТ 19903-74/ Ст.09Г2С ГОСТ 19281-2014</t>
-  </si>
-  <si>
-    <t>Лист S=10 ГОСТ19903-74/Ст.09Г2С ГОСТ 19281-89</t>
-  </si>
-  <si>
-    <t>Круг D25 ГОСТ 2590-06/ 345-09Г2С ГОСТ 19281-2014</t>
-  </si>
-  <si>
-    <t>Круг D20 09Г2С ГОСТ 19281-2014</t>
-  </si>
-  <si>
-    <t>Круг D10 ГОСТ 2590-2006/ Ст.20 ГОСТ 1050-88</t>
-  </si>
-  <si>
-    <t>Лист Б-ПН-2,0 ГОСТ 19903-74 / Ст3 ГОСТ 14637-89</t>
+    <t>Днище 219х4-25 ст.20 ГОСТ 6533-78</t>
+  </si>
+  <si>
+    <t>Шайба 16 ГОСТ 6958-78</t>
+  </si>
+  <si>
+    <t>Труба ГКРХХ 110х17,5 БрАЖН 10-4-4 ГОСТ 1208-90</t>
+  </si>
+  <si>
+    <t>Труба 10х1,0 М3-ПТ ГОСТ 617-90</t>
+  </si>
+  <si>
+    <t>Фланец х-80-40 ГОСТ12821 (заготовка-поковка ст.20 гр.IV КП 195 ГОСТ 8479-70)</t>
+  </si>
+  <si>
+    <t>Труба D89х6 ГОСТ 8732-78 Ст.20 ГОСТ 8731-74</t>
+  </si>
+  <si>
+    <t>Труба D83х9 Ст.40Х ГОСТ 8731-87</t>
+  </si>
+  <si>
+    <t>Труба D108х16 ГОСТ 8732-78/ Ст.40Х  ГОСТ 8731-74</t>
+  </si>
+  <si>
+    <t>Труба D426х50 Ст.20 ГОСТ 8732-78</t>
+  </si>
+  <si>
+    <t>Труба D114х28 ГОСТ 8732-78/ Ст.20 ГОСТ 8731-74</t>
+  </si>
+  <si>
+    <t>Труба D65х14 Ст.20 ГОСТ 8731-74</t>
+  </si>
+  <si>
+    <t>Труба D194х14 В20 ГОСТ 8732-78</t>
+  </si>
+  <si>
+    <t>Лента самоклеящаяся уплотнительная ППЭ 5х15 МКС</t>
+  </si>
+  <si>
+    <t>Зажим клеммный винтовой 2,5 мм2 (50/1500/36000) Б0033416 ЭРА арт. Б0033416</t>
+  </si>
+  <si>
+    <t>Клемма WAGO 222-415, 5 клеммных зажимов, номинальное сечение проводника 0.08-2.5 мм2</t>
+  </si>
+  <si>
+    <t>Заглушка NO-550-07 для винтовых клемм 2,5мм2 арт. Б0035737</t>
+  </si>
+  <si>
+    <t>Фиксатор ФК-102-01 на DIN-рейку 32057DEK Dekraft 2 арт. 32057DEK</t>
+  </si>
+  <si>
+    <t>DIN-рейка 50см перфорированная adr-50 EKF арт. adr-50</t>
+  </si>
+  <si>
+    <t>Разъем РпИм 1.25-5-0.8 плоский</t>
+  </si>
+  <si>
+    <t>Наконечник кабельный НШвИ 0,75мм</t>
+  </si>
+  <si>
+    <t>Наконечник кабельный НШвИ 1,5мм</t>
+  </si>
+  <si>
+    <t>Наконечник кабельный НШвИ 2,5мм</t>
+  </si>
+  <si>
+    <t>Крышка Угол горизонтальный CPO 90 (100х50)</t>
+  </si>
+  <si>
+    <t>Угол вертикальный внешний CD 90 (100х50)</t>
+  </si>
+  <si>
+    <t>Крышка на угол вертикальный внешний CD90 (100х50)</t>
+  </si>
+  <si>
+    <t>Угол вертикальный внутренний CS 90 100 х 50мм</t>
+  </si>
+  <si>
+    <t>Крышка на угол вертикальный внутренний CS 90 100 х 50мм</t>
+  </si>
+  <si>
+    <t>Монтажная рама РВМ 4.1.1</t>
+  </si>
+  <si>
+    <t>Ответная рама РВО 4.1.1</t>
+  </si>
+  <si>
+    <t>Уплотнительный модуль МКС 40/Ø 17-34 мм</t>
+  </si>
+  <si>
+    <t>Уплотнительный модуль МКС 20/Ø 5-14 мм</t>
+  </si>
+  <si>
+    <t>Компрессионный блок МКС КБ 120</t>
+  </si>
+  <si>
+    <t>Пластина анкерная 120</t>
+  </si>
+  <si>
+    <t>Кабель ВВГнг(А)-LS-ХЛ 3x2,5 d8мм</t>
+  </si>
+  <si>
+    <t>Короб ПВХ  40х25 мм</t>
+  </si>
+  <si>
+    <t>Короб ПВХ 40х40 мм</t>
+  </si>
+  <si>
+    <t>Металлорукав в ПВХ изоляции РЗ-ЦП-15</t>
+  </si>
+  <si>
+    <t>Провод Rd8</t>
+  </si>
+  <si>
+    <t>Провод ПуГВнг(А)-LS 1x1,5</t>
+  </si>
+  <si>
+    <t>Провод ПуГВнг(А)-LS 1x0,75</t>
+  </si>
+  <si>
+    <t>Кабель-канал 40х40 перфорированный Plast kk40-40 EKF</t>
+  </si>
+  <si>
+    <t>Кабель КПСЭнг(A)-FRLS 4х2х0,75</t>
+  </si>
+  <si>
+    <t>Кабель ВВГнг(А)-LS-ХЛ 3x2,5 d7.2мм</t>
+  </si>
+  <si>
+    <t>Кабель КВВГЭнг(А)-LS-ХЛ 7х1,0</t>
+  </si>
+  <si>
+    <t>Кабель КВВГЭнг(А)-LS-ХЛ 4х1,0</t>
+  </si>
+  <si>
+    <t>Кабель ВВГнг(А)-LS-ХЛ 4x1,5 d10,2мм</t>
+  </si>
+  <si>
+    <t>Шина заземления на DIN-изолятор ШНИ-6х9-8</t>
+  </si>
+  <si>
+    <t>Выключатель автоматический двухполюсный 3А B ВА47-29 4.5кА MVA20-2-003-B IEK</t>
+  </si>
+  <si>
+    <t>Угол горизонтальный CPO 90 (100 х 50)</t>
+  </si>
+  <si>
+    <t>Резьбовой крепежный элемент с внутренней резьбой Ркв-15</t>
+  </si>
+  <si>
+    <t>Резьбовой крепежный элемент с наружной резьбой РКН-15 (ММРн-15)</t>
+  </si>
+  <si>
+    <t>Крепление для труб ПВХ с защелкой, 16 мм</t>
+  </si>
+  <si>
+    <t>Скоба металлическая СМО 16-17 49152 КВТ</t>
+  </si>
+  <si>
+    <t>MV-клемма проводника Rd8</t>
+  </si>
+  <si>
+    <t>Держатель для полосы заземления К-188 У2 (цинк)</t>
+  </si>
+  <si>
+    <t>Коробка клеммная К-СП 08.13.09 24/11П 2КВе-Л-М20(А)-2КВе-Л-М20(В) 1ExeLLCGbXT6 ip66,80х130х90</t>
+  </si>
+  <si>
+    <t>Выключатель двухклавишный IP55</t>
+  </si>
+  <si>
+    <t>Выключатель автоматический двухполюсный IEK ARMAT M10N 2P B 10А AR-M10N-2-B010</t>
+  </si>
+  <si>
+    <t>Контроллер доступа "С2000-2"</t>
+  </si>
+  <si>
+    <t>Корпус металлический ЩМП-3-0 (650х500х220мм) У2 IP54 YKM40-03-54 IEK арт. YKM40-03-54</t>
+  </si>
+  <si>
+    <t>Карта proximity стандартная ST-PC010EM</t>
+  </si>
+  <si>
+    <t>Считыватель бесконтактный для proxi-карт, Proxy-3МA IP20</t>
+  </si>
+  <si>
+    <t>Крышка на Угол вертикальный внутренний CS 90 (50 х 50)</t>
+  </si>
+  <si>
+    <t>Угол вертикальный внутренний CS 90 (50 х 50)</t>
+  </si>
+  <si>
+    <t>Крышка на Угол вертикальный внешний CD 90 (50 х 50)</t>
+  </si>
+  <si>
+    <t>Угол вертикальный внешний CD 90 (50 х 50)</t>
+  </si>
+  <si>
+    <t>Крышка Угол горизонтальный CPO 90 (50х50)</t>
+  </si>
+  <si>
+    <t>Угол горизонтальный CPO 90 (50 х 50)</t>
+  </si>
+  <si>
+    <t>Прокладка медная 8х11-II ГОСТ 19752-84</t>
   </si>
   <si>
     <t>Кольцо 080-090-58 ГОСТ 9833-73</t>
   </si>
   <si>
-    <t>Пружина №467 НТ.200.000.029.0</t>
-  </si>
-  <si>
-    <t>Кольцо уплотнительное НТ 202.003.004.0</t>
-  </si>
-  <si>
-    <t>Кольцо 350-360-58-2-2 ГОСТ 9833-73</t>
-  </si>
-  <si>
-    <t>Проволока D1.8 Ст.60C2А ГОСТ14963-78</t>
-  </si>
-  <si>
-    <t>Круг D90 Ст.20Х13 ГОСТ 5632-72</t>
-  </si>
-  <si>
-    <t>Сетка полутомпаковая 008Н Л80 ГОСТ 6613-86</t>
+    <t>Кольцо 112-118-36 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Кольцо 055-060-30-2-2 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Пружина ПСМНТ.001.000.030</t>
+  </si>
+  <si>
+    <t>Кольцо 080-090-58-2-2 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Кольцо 065-075-58 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Уплотнение ПСМНТ.001.022.002</t>
+  </si>
+  <si>
+    <t>Обогреватель взрывозащищенный ОВЭ-4-УХЛ3 1,8 кВт, 380В IExdIIАТ3, IP54</t>
+  </si>
+  <si>
+    <t>Пост кнопочный взрывозащищенный ПВК-15 IP65 2ExеdIIСТ6</t>
+  </si>
+  <si>
+    <t>Пост кнопочный взрывозащищенный ПВК-25-ХЛ1 управление обогревом IP65 2ExеdIIСТ6</t>
+  </si>
+  <si>
+    <t>Светильник взрывозащищенный ДБП 09-15-001 УХЛ1 ExdllBT6G IP65</t>
+  </si>
+  <si>
+    <t>Датчик давления взрывозащ. СТИ775Ц-E-1-M-D-B-H-T-1</t>
+  </si>
+  <si>
+    <t>Лист Б-ПР-1,0 ГОСТ 19904-74/ 4-III-Ст3кп ГОСТ 16523-89</t>
+  </si>
+  <si>
+    <t>Шестигранник S=14 Ст.45 ГОСТ 1050-88</t>
+  </si>
+  <si>
+    <t>Круг D370 Ст.20 ГОСТ1050-88</t>
+  </si>
+  <si>
+    <t>Круг D45 Ст.40Х ГОСТ 4543-71</t>
+  </si>
+  <si>
+    <t>Круг D70 Ст.40Х ГОСТ 4543-71</t>
+  </si>
+  <si>
+    <t>Круг D430 Ст.16ГС ГОСТ 19281-14</t>
+  </si>
+  <si>
+    <t>Круг D195 Ст.16ГС-3 ГОСТ 5520-79</t>
+  </si>
+  <si>
+    <t>Шарик 25,4-100 ГОСТ 3722-81</t>
+  </si>
+  <si>
+    <t>Шпилька М18х40.56.019 ГОСТ 22034-76</t>
+  </si>
+  <si>
+    <t>Заклепка 2х4х37 Ан.Окс.хр. ГОСТ10299-80</t>
+  </si>
+  <si>
+    <t>Винт М16х50.56.019 ГОСТ 1481-84</t>
+  </si>
+  <si>
+    <t>Кабель ВВГнг(А)-FRLS 3x1,5 d7,2мм</t>
+  </si>
+  <si>
+    <t>Оповещатель светозвуковой Маяк-24К IP53</t>
+  </si>
+  <si>
+    <t>Извещатель пожарный дымовой ИП 212-141М</t>
   </si>
 </sst>
 </file>
@@ -881,12 +947,12 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F112"/>
+  <dimension ref="A1:F138"/>
   <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="11.45" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.1640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="46.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="74.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="74.83203125" style="1" customWidth="1"/>
     <col min="4" max="4" width="14.1640625" style="1" customWidth="1"/>
     <col min="5" max="5" width="13" style="1" customWidth="1"/>
     <col min="6" max="6" width="14.5" style="1" customWidth="1"/>
@@ -912,16 +978,16 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>1</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="8" t="s">
-        <v>83</v>
+        <v>63</v>
       </c>
       <c r="D2" s="5">
-        <v>20.399999999999999</v>
+        <v>120</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>6</v>
@@ -930,19 +996,19 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>2</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="8" t="s">
-        <v>84</v>
+        <v>64</v>
       </c>
       <c r="D3" s="5">
-        <v>48.6</v>
+        <v>0.25</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>7</v>
@@ -954,16 +1020,16 @@
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="D4" s="7">
-        <v>2000</v>
+        <v>9</v>
+      </c>
+      <c r="D4" s="5">
+        <v>40</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -972,16 +1038,16 @@
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="D5" s="7">
-        <v>4500</v>
+        <v>12</v>
+      </c>
+      <c r="D5" s="5">
+        <v>5</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -990,16 +1056,16 @@
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="8" t="s">
-        <v>8</v>
+        <v>65</v>
       </c>
       <c r="D6" s="5">
-        <v>47.85</v>
+        <v>40</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1008,16 +1074,16 @@
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="8" t="s">
-        <v>87</v>
+        <v>13</v>
       </c>
       <c r="D7" s="5">
-        <v>233.85</v>
+        <v>500</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1026,16 +1092,16 @@
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="8" t="s">
-        <v>88</v>
+        <v>15</v>
       </c>
       <c r="D8" s="5">
-        <v>291.60000000000002</v>
+        <v>800</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1044,16 +1110,16 @@
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="8" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="D9" s="5">
-        <v>95.25</v>
+        <v>5</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1062,16 +1128,16 @@
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="8" t="s">
-        <v>90</v>
+        <v>17</v>
       </c>
       <c r="D10" s="5">
-        <v>97.8</v>
+        <v>40</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1080,16 +1146,16 @@
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="8" t="s">
-        <v>91</v>
+        <v>18</v>
       </c>
       <c r="D11" s="5">
-        <v>57.15</v>
+        <v>10</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1098,16 +1164,16 @@
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="8" t="s">
-        <v>92</v>
+        <v>19</v>
       </c>
       <c r="D12" s="5">
-        <v>33.75</v>
+        <v>10</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1116,16 +1182,16 @@
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="8" t="s">
-        <v>93</v>
+        <v>20</v>
       </c>
       <c r="D13" s="5">
-        <v>16.5</v>
+        <v>20</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1134,16 +1200,16 @@
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="8" t="s">
-        <v>94</v>
+        <v>21</v>
       </c>
       <c r="D14" s="5">
-        <v>7.05</v>
+        <v>20</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1152,304 +1218,304 @@
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="8" t="s">
-        <v>95</v>
+        <v>22</v>
       </c>
       <c r="D15" s="5">
-        <v>193.2</v>
+        <v>15</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>15</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="8" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="D16" s="5">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>16</v>
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="8" t="s">
-        <v>96</v>
+        <v>25</v>
       </c>
       <c r="D17" s="5">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>17</v>
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="8" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="D18" s="5">
         <v>10</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>18</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="8" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="D19" s="5">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>19</v>
       </c>
       <c r="B20" s="4"/>
       <c r="C20" s="8" t="s">
-        <v>97</v>
+        <v>29</v>
       </c>
       <c r="D20" s="5">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>20</v>
       </c>
       <c r="B21" s="4"/>
       <c r="C21" s="8" t="s">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="D21" s="5">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>21</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="8" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="D22" s="5">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>22</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="8" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="D23" s="5">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>23</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="8" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="D24" s="5">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>24</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="8" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="D25" s="5">
-        <v>500</v>
+        <v>10</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="3">
         <v>25</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="8" t="s">
-        <v>21</v>
+        <v>67</v>
       </c>
       <c r="D26" s="5">
-        <v>800</v>
+        <v>10</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="3">
         <v>26</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="8" t="s">
-        <v>23</v>
+        <v>68</v>
       </c>
       <c r="D27" s="5">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="3">
         <v>27</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="8" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="D28" s="5">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="3">
         <v>28</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="8" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="D29" s="5">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="E29" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="3">
         <v>29</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="8" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="D30" s="5">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="3">
         <v>30</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="8" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="D31" s="5">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1458,16 +1524,16 @@
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="8" t="s">
-        <v>29</v>
+        <v>69</v>
       </c>
       <c r="D32" s="5">
-        <v>10</v>
+        <v>53.25</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1476,16 +1542,16 @@
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="8" t="s">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="D33" s="5">
-        <v>10</v>
+        <v>0.2</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1494,16 +1560,16 @@
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="8" t="s">
-        <v>31</v>
+        <v>71</v>
       </c>
       <c r="D34" s="5">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1512,16 +1578,16 @@
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="8" t="s">
-        <v>32</v>
+        <v>72</v>
       </c>
       <c r="D35" s="5">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1530,16 +1596,16 @@
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="8" t="s">
-        <v>33</v>
+        <v>73</v>
       </c>
       <c r="D36" s="5">
-        <v>2</v>
+        <v>99.25</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1548,34 +1614,34 @@
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="8" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="D37" s="5">
-        <v>10</v>
+        <v>18.25</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="3">
         <v>37</v>
       </c>
       <c r="B38" s="4"/>
       <c r="C38" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D38" s="5">
-        <v>1</v>
+        <v>75</v>
+      </c>
+      <c r="D38" s="7">
+        <v>4286.5</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1584,16 +1650,16 @@
       </c>
       <c r="B39" s="4"/>
       <c r="C39" s="8" t="s">
-        <v>38</v>
+        <v>76</v>
       </c>
       <c r="D39" s="5">
-        <v>1</v>
+        <v>148.5</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1602,16 +1668,16 @@
       </c>
       <c r="B40" s="4"/>
       <c r="C40" s="8" t="s">
-        <v>40</v>
+        <v>77</v>
       </c>
       <c r="D40" s="5">
-        <v>1</v>
+        <v>37.35</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1620,106 +1686,106 @@
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="8" t="s">
-        <v>41</v>
+        <v>78</v>
       </c>
       <c r="D41" s="5">
-        <v>1</v>
+        <v>271.75</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="3">
         <v>41</v>
       </c>
       <c r="B42" s="4"/>
       <c r="C42" s="8" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="D42" s="5">
-        <v>11.43</v>
+        <v>2.1</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="3">
         <v>42</v>
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="8" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="D43" s="5">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="3">
         <v>43</v>
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="8" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D44" s="5">
-        <v>4.08</v>
+        <v>4</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="3">
         <v>44</v>
       </c>
       <c r="B45" s="4"/>
       <c r="C45" s="8" t="s">
-        <v>88</v>
+        <v>46</v>
       </c>
       <c r="D45" s="5">
-        <v>58.32</v>
+        <v>20</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="3">
         <v>45</v>
       </c>
       <c r="B46" s="4"/>
       <c r="C46" s="8" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="D46" s="5">
-        <v>19.559999999999999</v>
+        <v>2</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1728,16 +1794,16 @@
       </c>
       <c r="B47" s="4"/>
       <c r="C47" s="8" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="D47" s="5">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>43</v>
+        <v>6</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1746,16 +1812,16 @@
       </c>
       <c r="B48" s="4"/>
       <c r="C48" s="8" t="s">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="D48" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>43</v>
+        <v>6</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1764,16 +1830,16 @@
       </c>
       <c r="B49" s="4"/>
       <c r="C49" s="8" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="D49" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1782,16 +1848,16 @@
       </c>
       <c r="B50" s="4"/>
       <c r="C50" s="8" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="D50" s="5">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1800,16 +1866,16 @@
       </c>
       <c r="B51" s="4"/>
       <c r="C51" s="8" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
       <c r="D51" s="5">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1818,16 +1884,16 @@
       </c>
       <c r="B52" s="4"/>
       <c r="C52" s="8" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
       <c r="D52" s="5">
-        <v>9.9</v>
+        <v>20</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1836,10 +1902,10 @@
       </c>
       <c r="B53" s="4"/>
       <c r="C53" s="8" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="D53" s="5">
-        <v>32.659999999999997</v>
+        <v>4</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>6</v>
@@ -1854,10 +1920,10 @@
       </c>
       <c r="B54" s="4"/>
       <c r="C54" s="8" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="D54" s="5">
-        <v>7.8</v>
+        <v>4</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>6</v>
@@ -1872,10 +1938,10 @@
       </c>
       <c r="B55" s="4"/>
       <c r="C55" s="8" t="s">
-        <v>106</v>
+        <v>91</v>
       </c>
       <c r="D55" s="5">
-        <v>79.44</v>
+        <v>4</v>
       </c>
       <c r="E55" s="6" t="s">
         <v>6</v>
@@ -1890,10 +1956,10 @@
       </c>
       <c r="B56" s="4"/>
       <c r="C56" s="8" t="s">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="D56" s="5">
-        <v>279.08</v>
+        <v>4</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>6</v>
@@ -1908,10 +1974,10 @@
       </c>
       <c r="B57" s="4"/>
       <c r="C57" s="8" t="s">
-        <v>108</v>
+        <v>93</v>
       </c>
       <c r="D57" s="5">
-        <v>308.89</v>
+        <v>4</v>
       </c>
       <c r="E57" s="6" t="s">
         <v>6</v>
@@ -1926,10 +1992,10 @@
       </c>
       <c r="B58" s="4"/>
       <c r="C58" s="8" t="s">
-        <v>109</v>
+        <v>94</v>
       </c>
       <c r="D58" s="5">
-        <v>41.21</v>
+        <v>1</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>6</v>
@@ -1944,10 +2010,10 @@
       </c>
       <c r="B59" s="4"/>
       <c r="C59" s="8" t="s">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="D59" s="5">
-        <v>55.64</v>
+        <v>1</v>
       </c>
       <c r="E59" s="6" t="s">
         <v>6</v>
@@ -1962,10 +2028,10 @@
       </c>
       <c r="B60" s="4"/>
       <c r="C60" s="8" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
       <c r="D60" s="5">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>6</v>
@@ -1980,10 +2046,10 @@
       </c>
       <c r="B61" s="4"/>
       <c r="C61" s="8" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="D61" s="5">
-        <v>50.8</v>
+        <v>30</v>
       </c>
       <c r="E61" s="6" t="s">
         <v>6</v>
@@ -1998,10 +2064,10 @@
       </c>
       <c r="B62" s="4"/>
       <c r="C62" s="8" t="s">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="D62" s="5">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>6</v>
@@ -2016,10 +2082,10 @@
       </c>
       <c r="B63" s="4"/>
       <c r="C63" s="8" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="D63" s="5">
-        <v>916.44</v>
+        <v>7</v>
       </c>
       <c r="E63" s="6" t="s">
         <v>6</v>
@@ -2034,16 +2100,16 @@
       </c>
       <c r="B64" s="4"/>
       <c r="C64" s="8" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="D64" s="5">
-        <v>0.7</v>
+        <v>15</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="65" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2052,16 +2118,16 @@
       </c>
       <c r="B65" s="4"/>
       <c r="C65" s="8" t="s">
-        <v>47</v>
+        <v>101</v>
       </c>
       <c r="D65" s="5">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="66" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2070,16 +2136,16 @@
       </c>
       <c r="B66" s="4"/>
       <c r="C66" s="8" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="D66" s="5">
-        <v>0.5</v>
+        <v>8</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="67" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2088,16 +2154,16 @@
       </c>
       <c r="B67" s="4"/>
       <c r="C67" s="8" t="s">
-        <v>117</v>
+        <v>103</v>
       </c>
       <c r="D67" s="5">
-        <v>1</v>
+        <v>130</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="68" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2106,16 +2172,16 @@
       </c>
       <c r="B68" s="4"/>
       <c r="C68" s="8" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="D68" s="5">
-        <v>2</v>
+        <v>35</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="69" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2124,16 +2190,16 @@
       </c>
       <c r="B69" s="4"/>
       <c r="C69" s="8" t="s">
-        <v>48</v>
+        <v>105</v>
       </c>
       <c r="D69" s="5">
-        <v>2.2999999999999998</v>
+        <v>8</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="70" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2142,646 +2208,646 @@
       </c>
       <c r="B70" s="4"/>
       <c r="C70" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="D70" s="7">
-        <v>1000</v>
+        <v>106</v>
+      </c>
+      <c r="D70" s="5">
+        <v>2</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="3">
         <v>70</v>
       </c>
       <c r="B71" s="4"/>
       <c r="C71" s="8" t="s">
-        <v>52</v>
+        <v>107</v>
       </c>
       <c r="D71" s="5">
-        <v>26.84</v>
+        <v>1</v>
       </c>
       <c r="E71" s="6" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="3">
         <v>71</v>
       </c>
       <c r="B72" s="4"/>
       <c r="C72" s="8" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="D72" s="5">
-        <v>2.15</v>
+        <v>16</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="3">
         <v>72</v>
       </c>
       <c r="B73" s="4"/>
       <c r="C73" s="8" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="D73" s="5">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E73" s="6" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="3">
         <v>73</v>
       </c>
       <c r="B74" s="4"/>
       <c r="C74" s="8" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="D74" s="5">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="3">
         <v>74</v>
       </c>
       <c r="B75" s="4"/>
       <c r="C75" s="8" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
       <c r="D75" s="5">
-        <v>411</v>
+        <v>112</v>
       </c>
       <c r="E75" s="6" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="3">
         <v>75</v>
       </c>
       <c r="B76" s="4"/>
       <c r="C76" s="8" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="D76" s="5">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="3">
         <v>76</v>
       </c>
       <c r="B77" s="4"/>
       <c r="C77" s="8" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="D77" s="5">
-        <v>8.1999999999999993</v>
+        <v>1</v>
       </c>
       <c r="E77" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="3">
         <v>77</v>
       </c>
       <c r="B78" s="4"/>
       <c r="C78" s="8" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="D78" s="5">
-        <v>49</v>
+        <v>1</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F78" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="3">
         <v>78</v>
       </c>
       <c r="B79" s="4"/>
       <c r="C79" s="8" t="s">
-        <v>126</v>
+        <v>115</v>
       </c>
       <c r="D79" s="5">
-        <v>212.17</v>
+        <v>4</v>
       </c>
       <c r="E79" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F79" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="3">
         <v>79</v>
       </c>
       <c r="B80" s="4"/>
       <c r="C80" s="8" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="D80" s="5">
-        <v>3.41</v>
+        <v>48</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="3">
         <v>80</v>
       </c>
       <c r="B81" s="4"/>
       <c r="C81" s="8" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="D81" s="5">
-        <v>24.14</v>
+        <v>39</v>
       </c>
       <c r="E81" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="3">
         <v>81</v>
       </c>
       <c r="B82" s="4"/>
       <c r="C82" s="8" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="D82" s="5">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="3">
         <v>82</v>
       </c>
       <c r="B83" s="4"/>
       <c r="C83" s="8" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
       <c r="D83" s="5">
-        <v>6.52</v>
+        <v>135</v>
       </c>
       <c r="E83" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F83" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="3">
         <v>83</v>
       </c>
       <c r="B84" s="4"/>
       <c r="C84" s="8" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="D84" s="5">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="3">
         <v>84</v>
       </c>
       <c r="B85" s="4"/>
       <c r="C85" s="8" t="s">
-        <v>132</v>
+        <v>47</v>
       </c>
       <c r="D85" s="5">
-        <v>4.01</v>
+        <v>70</v>
       </c>
       <c r="E85" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F85" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="3">
         <v>85</v>
       </c>
       <c r="B86" s="4"/>
       <c r="C86" s="8" t="s">
-        <v>55</v>
+        <v>121</v>
       </c>
       <c r="D86" s="5">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="3">
         <v>86</v>
       </c>
       <c r="B87" s="4"/>
       <c r="C87" s="8" t="s">
-        <v>57</v>
+        <v>122</v>
       </c>
       <c r="D87" s="5">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E87" s="6" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="3">
         <v>87</v>
       </c>
       <c r="B88" s="4"/>
       <c r="C88" s="8" t="s">
-        <v>58</v>
+        <v>123</v>
       </c>
       <c r="D88" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="3">
         <v>88</v>
       </c>
       <c r="B89" s="4"/>
       <c r="C89" s="8" t="s">
-        <v>59</v>
+        <v>124</v>
       </c>
       <c r="D89" s="5">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E89" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="3">
         <v>89</v>
       </c>
       <c r="B90" s="4"/>
       <c r="C90" s="8" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="D90" s="5">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="3">
         <v>90</v>
       </c>
       <c r="B91" s="4"/>
       <c r="C91" s="8" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="D91" s="5">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E91" s="6" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="92" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="3">
         <v>91</v>
       </c>
       <c r="B92" s="4"/>
       <c r="C92" s="8" t="s">
-        <v>62</v>
+        <v>125</v>
       </c>
       <c r="D92" s="5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>63</v>
+        <v>6</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="3">
         <v>92</v>
       </c>
       <c r="B93" s="4"/>
       <c r="C93" s="8" t="s">
-        <v>64</v>
+        <v>126</v>
       </c>
       <c r="D93" s="5">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E93" s="6" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="3">
         <v>93</v>
       </c>
       <c r="B94" s="4"/>
       <c r="C94" s="8" t="s">
-        <v>66</v>
+        <v>127</v>
       </c>
       <c r="D94" s="5">
         <v>10</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="3">
         <v>94</v>
       </c>
       <c r="B95" s="4"/>
       <c r="C95" s="8" t="s">
-        <v>67</v>
+        <v>128</v>
       </c>
       <c r="D95" s="5">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E95" s="6" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F95" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="3">
         <v>95</v>
       </c>
       <c r="B96" s="4"/>
       <c r="C96" s="8" t="s">
-        <v>68</v>
+        <v>129</v>
       </c>
       <c r="D96" s="5">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F96" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="3">
         <v>96</v>
       </c>
       <c r="B97" s="4"/>
       <c r="C97" s="8" t="s">
-        <v>69</v>
+        <v>130</v>
       </c>
       <c r="D97" s="5">
-        <v>100</v>
+        <v>8</v>
       </c>
       <c r="E97" s="6" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="98" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="3">
         <v>97</v>
       </c>
       <c r="B98" s="4"/>
       <c r="C98" s="8" t="s">
-        <v>71</v>
+        <v>131</v>
       </c>
       <c r="D98" s="5">
-        <v>300</v>
+        <v>8</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="3">
         <v>98</v>
       </c>
       <c r="B99" s="4"/>
       <c r="C99" s="8" t="s">
-        <v>72</v>
+        <v>132</v>
       </c>
       <c r="D99" s="5">
-        <v>300</v>
+        <v>8</v>
       </c>
       <c r="E99" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="100" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="3">
         <v>99</v>
       </c>
       <c r="B100" s="4"/>
       <c r="C100" s="8" t="s">
-        <v>73</v>
+        <v>133</v>
       </c>
       <c r="D100" s="5">
-        <v>100</v>
+        <v>8</v>
       </c>
       <c r="E100" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F100" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="101" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="3">
         <v>100</v>
       </c>
       <c r="B101" s="4"/>
       <c r="C101" s="8" t="s">
-        <v>74</v>
+        <v>50</v>
       </c>
       <c r="D101" s="5">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="E101" s="6" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F101" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="102" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="3">
         <v>101</v>
       </c>
       <c r="B102" s="4"/>
       <c r="C102" s="8" t="s">
-        <v>75</v>
+        <v>134</v>
       </c>
       <c r="D102" s="5">
-        <v>100</v>
+        <v>8</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F102" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="3">
         <v>102</v>
       </c>
       <c r="B103" s="4"/>
       <c r="C103" s="8" t="s">
-        <v>76</v>
+        <v>135</v>
       </c>
       <c r="D103" s="5">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="E103" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F103" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="3">
         <v>103</v>
       </c>
       <c r="B104" s="4"/>
       <c r="C104" s="8" t="s">
-        <v>77</v>
+        <v>136</v>
       </c>
       <c r="D104" s="5">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="E104" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F104" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="3">
         <v>104</v>
       </c>
       <c r="B105" s="4"/>
       <c r="C105" s="8" t="s">
-        <v>78</v>
+        <v>137</v>
       </c>
       <c r="D105" s="5">
         <v>50</v>
       </c>
       <c r="E105" s="6" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F105" s="4" t="s">
-        <v>79</v>
+        <v>51</v>
       </c>
     </row>
     <row r="106" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2790,16 +2856,16 @@
       </c>
       <c r="B106" s="4"/>
       <c r="C106" s="8" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="D106" s="5">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="E106" s="6" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F106" s="4" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
     </row>
     <row r="107" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2808,16 +2874,16 @@
       </c>
       <c r="B107" s="4"/>
       <c r="C107" s="8" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="D107" s="5">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E107" s="6" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F107" s="4" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
     </row>
     <row r="108" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2826,16 +2892,16 @@
       </c>
       <c r="B108" s="4"/>
       <c r="C108" s="8" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="D108" s="5">
-        <v>150</v>
+        <v>25</v>
       </c>
       <c r="E108" s="6" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F108" s="4" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
     </row>
     <row r="109" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2844,16 +2910,16 @@
       </c>
       <c r="B109" s="4"/>
       <c r="C109" s="8" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="D109" s="5">
-        <v>120</v>
+        <v>170</v>
       </c>
       <c r="E109" s="6" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F109" s="4" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
     </row>
     <row r="110" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2862,16 +2928,16 @@
       </c>
       <c r="B110" s="4"/>
       <c r="C110" s="8" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D110" s="5">
-        <v>0.3</v>
+        <v>25</v>
       </c>
       <c r="E110" s="6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F110" s="4" t="s">
-        <v>81</v>
+        <v>51</v>
       </c>
     </row>
     <row r="111" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2880,16 +2946,16 @@
       </c>
       <c r="B111" s="4"/>
       <c r="C111" s="8" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="D111" s="5">
-        <v>31.7</v>
+        <v>2</v>
       </c>
       <c r="E111" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F111" s="4" t="s">
-        <v>81</v>
+        <v>52</v>
       </c>
     </row>
     <row r="112" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2898,16 +2964,484 @@
       </c>
       <c r="B112" s="4"/>
       <c r="C112" s="8" t="s">
-        <v>139</v>
+        <v>53</v>
       </c>
       <c r="D112" s="5">
-        <v>0.15</v>
+        <v>2</v>
       </c>
       <c r="E112" s="6" t="s">
-        <v>82</v>
+        <v>6</v>
       </c>
       <c r="F112" s="4" t="s">
-        <v>81</v>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A113" s="3">
+        <v>112</v>
+      </c>
+      <c r="B113" s="4"/>
+      <c r="C113" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="D113" s="5">
+        <v>2</v>
+      </c>
+      <c r="E113" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F113" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A114" s="3">
+        <v>113</v>
+      </c>
+      <c r="B114" s="4"/>
+      <c r="C114" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="D114" s="5">
+        <v>2</v>
+      </c>
+      <c r="E114" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F114" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A115" s="3">
+        <v>114</v>
+      </c>
+      <c r="B115" s="4"/>
+      <c r="C115" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D115" s="5">
+        <v>2</v>
+      </c>
+      <c r="E115" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F115" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A116" s="3">
+        <v>115</v>
+      </c>
+      <c r="B116" s="4"/>
+      <c r="C116" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D116" s="5">
+        <v>1</v>
+      </c>
+      <c r="E116" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F116" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A117" s="3">
+        <v>116</v>
+      </c>
+      <c r="B117" s="4"/>
+      <c r="C117" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D117" s="5">
+        <v>1</v>
+      </c>
+      <c r="E117" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F117" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A118" s="3">
+        <v>117</v>
+      </c>
+      <c r="B118" s="4"/>
+      <c r="C118" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="D118" s="5">
+        <v>6</v>
+      </c>
+      <c r="E118" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F118" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A119" s="3">
+        <v>118</v>
+      </c>
+      <c r="B119" s="4"/>
+      <c r="C119" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="D119" s="5">
+        <v>4</v>
+      </c>
+      <c r="E119" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F119" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A120" s="3">
+        <v>119</v>
+      </c>
+      <c r="B120" s="4"/>
+      <c r="C120" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D120" s="5">
+        <v>1</v>
+      </c>
+      <c r="E120" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F120" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A121" s="3">
+        <v>120</v>
+      </c>
+      <c r="B121" s="4"/>
+      <c r="C121" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D121" s="5">
+        <v>1</v>
+      </c>
+      <c r="E121" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F121" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A122" s="3">
+        <v>121</v>
+      </c>
+      <c r="B122" s="4"/>
+      <c r="C122" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="D122" s="5">
+        <v>1.5</v>
+      </c>
+      <c r="E122" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F122" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A123" s="3">
+        <v>122</v>
+      </c>
+      <c r="B123" s="4"/>
+      <c r="C123" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="D123" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="E123" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F123" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A124" s="3">
+        <v>123</v>
+      </c>
+      <c r="B124" s="4"/>
+      <c r="C124" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="D124" s="5">
+        <v>950</v>
+      </c>
+      <c r="E124" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F124" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A125" s="3">
+        <v>124</v>
+      </c>
+      <c r="B125" s="4"/>
+      <c r="C125" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="D125" s="5">
+        <v>131</v>
+      </c>
+      <c r="E125" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A126" s="3">
+        <v>125</v>
+      </c>
+      <c r="B126" s="4"/>
+      <c r="C126" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="D126" s="5">
+        <v>26.5</v>
+      </c>
+      <c r="E126" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F126" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A127" s="3">
+        <v>126</v>
+      </c>
+      <c r="B127" s="4"/>
+      <c r="C127" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="D127" s="7">
+        <v>1415.25</v>
+      </c>
+      <c r="E127" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F127" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A128" s="3">
+        <v>127</v>
+      </c>
+      <c r="B128" s="4"/>
+      <c r="C128" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="D128" s="5">
+        <v>291</v>
+      </c>
+      <c r="E128" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F128" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A129" s="3">
+        <v>128</v>
+      </c>
+      <c r="B129" s="4"/>
+      <c r="C129" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="D129" s="5">
+        <v>25</v>
+      </c>
+      <c r="E129" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F129" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A130" s="3">
+        <v>129</v>
+      </c>
+      <c r="B130" s="4"/>
+      <c r="C130" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="D130" s="5">
+        <v>500</v>
+      </c>
+      <c r="E130" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F130" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A131" s="3">
+        <v>130</v>
+      </c>
+      <c r="B131" s="4"/>
+      <c r="C131" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="D131" s="5">
+        <v>50</v>
+      </c>
+      <c r="E131" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F131" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A132" s="3">
+        <v>131</v>
+      </c>
+      <c r="B132" s="4"/>
+      <c r="C132" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="D132" s="5">
+        <v>100</v>
+      </c>
+      <c r="E132" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F132" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A133" s="3">
+        <v>132</v>
+      </c>
+      <c r="B133" s="4"/>
+      <c r="C133" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="D133" s="5">
+        <v>36</v>
+      </c>
+      <c r="E133" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F133" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A134" s="3">
+        <v>133</v>
+      </c>
+      <c r="B134" s="4"/>
+      <c r="C134" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="D134" s="5">
+        <v>24</v>
+      </c>
+      <c r="E134" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F134" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A135" s="3">
+        <v>134</v>
+      </c>
+      <c r="B135" s="4"/>
+      <c r="C135" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="D135" s="5">
+        <v>2</v>
+      </c>
+      <c r="E135" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F135" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A136" s="3">
+        <v>135</v>
+      </c>
+      <c r="B136" s="4"/>
+      <c r="C136" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="D136" s="5">
+        <v>2</v>
+      </c>
+      <c r="E136" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F136" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A137" s="3">
+        <v>136</v>
+      </c>
+      <c r="B137" s="4"/>
+      <c r="C137" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="D137" s="5">
+        <v>30</v>
+      </c>
+      <c r="E137" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F137" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A138" s="3">
+        <v>137</v>
+      </c>
+      <c r="B138" s="4"/>
+      <c r="C138" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="D138" s="5">
+        <v>6</v>
+      </c>
+      <c r="E138" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F138" s="4" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new Procurement, Careers, Calculator, Layout and LayoutBack
</commit_message>
<xml_diff>
--- a/public/procurement.xlsx
+++ b/public/procurement.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lka\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71C15226-ACA9-414C-A703-D16BBC0C5C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{899FF701-B3E4-4D5E-B966-3ED39BF75F9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4755" yWindow="3270" windowWidth="23730" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="166">
   <si>
     <t>№ п/п</t>
   </si>
@@ -54,63 +54,75 @@
     <t>кг</t>
   </si>
   <si>
+    <t>ЛГУП-7331</t>
+  </si>
+  <si>
     <t>Маркер  краска красный по металлу</t>
   </si>
   <si>
     <t>шт.</t>
   </si>
   <si>
-    <t>ЛГУП-7331</t>
+    <t>Перчатки х/б трикотажные 5 нитей 10 класс с ПВХ -Камаз 426</t>
+  </si>
+  <si>
+    <t>пара</t>
+  </si>
+  <si>
+    <t>Перчатки с латесным покрытием</t>
+  </si>
+  <si>
+    <t>пар</t>
+  </si>
+  <si>
+    <t>Каска строительная оранжевая Исток</t>
+  </si>
+  <si>
+    <t>Огнетушитель ОП-8</t>
+  </si>
+  <si>
+    <t>Маркер по металлу белый</t>
+  </si>
+  <si>
+    <t>Маркер по металлу черный тонкий</t>
   </si>
   <si>
     <t>Каска строительная белая</t>
   </si>
   <si>
-    <t>Перчатки х/б трикотажные 5 нитей 10 класс с ПВХ -Камаз 426</t>
-  </si>
-  <si>
-    <t>пара</t>
-  </si>
-  <si>
-    <t>Перчатки с латесным покрытием</t>
-  </si>
-  <si>
-    <t>пар</t>
-  </si>
-  <si>
     <t>Маркер белый</t>
   </si>
   <si>
     <t>Ветошь</t>
   </si>
   <si>
-    <t>Каска строительная оранжевая Исток</t>
-  </si>
-  <si>
-    <t>Маркер по металлу черный тонкий</t>
-  </si>
-  <si>
-    <t>Маркер по металлу белый</t>
-  </si>
-  <si>
-    <t>Огнетушитель ОП-8</t>
+    <t>Резак</t>
+  </si>
+  <si>
+    <t>ЛГУП-7332</t>
+  </si>
+  <si>
+    <t>Кувалда 1 кг.</t>
+  </si>
+  <si>
+    <t>Ножницы по металлу</t>
+  </si>
+  <si>
+    <t>Ключи обмедненные</t>
+  </si>
+  <si>
+    <t>набор</t>
+  </si>
+  <si>
+    <t>Трещетка ключ 1/2</t>
   </si>
   <si>
     <t>Гайковерт</t>
   </si>
   <si>
-    <t>ЛГУП-7332</t>
-  </si>
-  <si>
     <t>Ключ комбинированные омедненные 41</t>
   </si>
   <si>
-    <t>Ключи обмедненные</t>
-  </si>
-  <si>
-    <t>набор</t>
-  </si>
-  <si>
     <t>Ключ комбинированные омедненные 36</t>
   </si>
   <si>
@@ -120,27 +132,15 @@
     <t>Ключ комбинированные омедненные 24</t>
   </si>
   <si>
-    <t>Трещетка ключ 1/2</t>
-  </si>
-  <si>
-    <t>Кувалда 1 кг.</t>
-  </si>
-  <si>
-    <t>Резак</t>
-  </si>
-  <si>
-    <t>Ножницы по металлу</t>
-  </si>
-  <si>
     <t>ЛГУП-7428</t>
   </si>
   <si>
+    <t>Днище 720х12 ст09Г2С ГОСТ 6533-78</t>
+  </si>
+  <si>
     <t>Днище 820х14-09Г2С ГОСТ 6533-78</t>
   </si>
   <si>
-    <t>Днище 720х12 ст09Г2С ГОСТ 6533-78</t>
-  </si>
-  <si>
     <t>Днище 377х10 09Г2С ГОСТ 6533-78</t>
   </si>
   <si>
@@ -171,49 +171,67 @@
     <t>Держатель проводника Rd8</t>
   </si>
   <si>
+    <t>Индикатор положения поплавка ИПП 01.00.000</t>
+  </si>
+  <si>
     <t>МИП-24 исп.20 (МИП-24-2/П5-Р-RS), до двух АКБ 12 В 17 Ач</t>
   </si>
   <si>
     <t>Блок коммутации 24В БК-24-RS485-01</t>
   </si>
   <si>
-    <t>Индикатор положения поплавка ИПП 01.00.000</t>
-  </si>
-  <si>
     <t>ЛГУП-7450</t>
   </si>
   <si>
-    <t>ЛГУП-7451</t>
-  </si>
-  <si>
-    <t>Обогреватель взрывозащищенный ОВЭ-4 ТК-1.0 1 кВт, 220В, 50 Гц.</t>
-  </si>
-  <si>
-    <t>Коробка клеммная К-СП 16.18.09 24/20П 4КВе-Л-М20(А)-4КВе-Л-М20(В) 1ЕхеLLCGbXT6, ip66, 160х180х90</t>
-  </si>
-  <si>
-    <t>Коробка соед взрывозащК-СП 16.26.09 24/31 П 8КВе-Л-М20(А) 8КВе-Л-М20(В) 1ЕхеLLCGb ip66, 160х260х90</t>
-  </si>
-  <si>
-    <t>К-СП 16.26.09 32/26П 6КВе-Л-М20(А)-6КВе-Л-М20(В)-1КВе-Л-М20(D) 1ExeLLCGbXT6 ip66 120х260х90</t>
+    <t>Палитра цветов</t>
+  </si>
+  <si>
+    <t>ЛГУП-7454</t>
+  </si>
+  <si>
+    <t>ЛГУП-7457</t>
+  </si>
+  <si>
+    <t>ЛГУП-7460</t>
   </si>
   <si>
     <t>Газоанализатор взрывозащищенный СГОЭС 1Ex d IIC T4 Gb, IP67</t>
   </si>
   <si>
-    <t>Палитра цветов</t>
-  </si>
-  <si>
-    <t>ЛГУП-7454</t>
-  </si>
-  <si>
-    <t>ЛГУП-7457</t>
-  </si>
-  <si>
-    <t>ЛГУП-7460</t>
-  </si>
-  <si>
-    <t>ЛГУП-7462</t>
+    <t>ЛГУП-7475</t>
+  </si>
+  <si>
+    <t>Наконечник штыревой втулочный изолированный НШВИ 0.5-8 79435</t>
+  </si>
+  <si>
+    <t>ЛГУП-7477</t>
+  </si>
+  <si>
+    <t>Провод силовой ПуГВнг(А)-LS 1х0.5 белый</t>
+  </si>
+  <si>
+    <t>ЛГУП-7478</t>
+  </si>
+  <si>
+    <t>ЛГУП-7480</t>
+  </si>
+  <si>
+    <t>00УП-000005</t>
+  </si>
+  <si>
+    <t>Дюбель-молли М6х50</t>
+  </si>
+  <si>
+    <t>ЛГУП-7485</t>
+  </si>
+  <si>
+    <t>Контргайка 20 ГОСТ 8968-75 (12Х18Н10Т)</t>
+  </si>
+  <si>
+    <t>Удалитель наклеек Lavr Антискотч</t>
+  </si>
+  <si>
+    <t>ЛГУП-7486</t>
   </si>
   <si>
     <t>Кольцо 350-360-58-2-2 ГОСТ 9833-73</t>
@@ -228,61 +246,145 @@
     <t>Фумлента</t>
   </si>
   <si>
+    <t>Шайба 16 ГОСТ 6958-78</t>
+  </si>
+  <si>
     <t>Днище 219х4-25 ст.20 ГОСТ 6533-78</t>
   </si>
   <si>
-    <t>Шайба 16 ГОСТ 6958-78</t>
+    <t>Труба 10х1,0 М3-ПТ ГОСТ 617-90</t>
   </si>
   <si>
     <t>Труба ГКРХХ 110х17,5 БрАЖН 10-4-4 ГОСТ 1208-90</t>
   </si>
   <si>
-    <t>Труба 10х1,0 М3-ПТ ГОСТ 617-90</t>
-  </si>
-  <si>
     <t>Фланец х-80-40 ГОСТ12821 (заготовка-поковка ст.20 гр.IV КП 195 ГОСТ 8479-70)</t>
   </si>
   <si>
+    <t>Труба D194х14 В20 ГОСТ 8732-78</t>
+  </si>
+  <si>
+    <t>Труба D426х50 Ст.20 ГОСТ 8732-78</t>
+  </si>
+  <si>
+    <t>Труба D108х16 ГОСТ 8732-78/ Ст.40Х  ГОСТ 8731-74</t>
+  </si>
+  <si>
+    <t>Труба D83х9 Ст.40Х ГОСТ 8731-87</t>
+  </si>
+  <si>
     <t>Труба D89х6 ГОСТ 8732-78 Ст.20 ГОСТ 8731-74</t>
   </si>
   <si>
-    <t>Труба D83х9 Ст.40Х ГОСТ 8731-87</t>
-  </si>
-  <si>
-    <t>Труба D108х16 ГОСТ 8732-78/ Ст.40Х  ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>Труба D426х50 Ст.20 ГОСТ 8732-78</t>
+    <t>Труба D65х14 Ст.20 ГОСТ 8731-74</t>
   </si>
   <si>
     <t>Труба D114х28 ГОСТ 8732-78/ Ст.20 ГОСТ 8731-74</t>
   </si>
   <si>
-    <t>Труба D65х14 Ст.20 ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>Труба D194х14 В20 ГОСТ 8732-78</t>
+    <t>Металлорукав в ПВХ изоляции РЗ-ЦП-15</t>
+  </si>
+  <si>
+    <t>Пластина анкерная 120</t>
+  </si>
+  <si>
+    <t>Клемма WAGO 222-415, 5 клеммных зажимов, номинальное сечение проводника 0.08-2.5 мм2</t>
+  </si>
+  <si>
+    <t>Компрессионный блок МКС КБ 120</t>
+  </si>
+  <si>
+    <t>Уплотнительный модуль МКС 20/Ø 5-14 мм</t>
+  </si>
+  <si>
+    <t>Уплотнительный модуль МКС 40/Ø 17-34 мм</t>
+  </si>
+  <si>
+    <t>Ответная рама РВО 4.1.1</t>
+  </si>
+  <si>
+    <t>Монтажная рама РВМ 4.1.1</t>
+  </si>
+  <si>
+    <t>Крышка на угол вертикальный внутренний CS 90 100 х 50мм</t>
+  </si>
+  <si>
+    <t>Угол вертикальный внутренний CS 90 100 х 50мм</t>
+  </si>
+  <si>
+    <t>Скоба металлическая СМО 16-17 49152 КВТ</t>
+  </si>
+  <si>
+    <t>MV-клемма проводника Rd8</t>
+  </si>
+  <si>
+    <t>Держатель для полосы заземления К-188 У2 (цинк)</t>
+  </si>
+  <si>
+    <t>Коробка клеммная К-СП 08.13.09 24/11П 2КВе-Л-М20(А)-2КВе-Л-М20(В) 1ExeLLCGbXT6 ip66,80х130х90</t>
+  </si>
+  <si>
+    <t>Выключатель двухклавишный IP55</t>
+  </si>
+  <si>
+    <t>Разъем РпИм 1.25-5-0.8 плоский</t>
+  </si>
+  <si>
+    <t>DIN-рейка 50см перфорированная adr-50 EKF арт. adr-50</t>
+  </si>
+  <si>
+    <t>Фиксатор ФК-102-01 на DIN-рейку 32057DEK Dekraft 2 арт. 32057DEK</t>
+  </si>
+  <si>
+    <t>Заглушка NO-550-07 для винтовых клемм 2,5мм2 арт. Б0035737</t>
+  </si>
+  <si>
+    <t>Зажим клеммный винтовой 2,5 мм2 (50/1500/36000) Б0033416 ЭРА арт. Б0033416</t>
+  </si>
+  <si>
+    <t>Шина заземления на DIN-изолятор ШНИ-6х9-8</t>
+  </si>
+  <si>
+    <t>Короб ПВХ 40х40 мм</t>
+  </si>
+  <si>
+    <t>Короб ПВХ  40х25 мм</t>
+  </si>
+  <si>
+    <t>Кабель ВВГнг(А)-LS-ХЛ 3x2,5 d8мм</t>
+  </si>
+  <si>
+    <t>Кабель ВВГнг(А)-LS-ХЛ 4x1,5 d10,2мм</t>
   </si>
   <si>
     <t>Лента самоклеящаяся уплотнительная ППЭ 5х15 МКС</t>
   </si>
   <si>
-    <t>Зажим клеммный винтовой 2,5 мм2 (50/1500/36000) Б0033416 ЭРА арт. Б0033416</t>
-  </si>
-  <si>
-    <t>Клемма WAGO 222-415, 5 клеммных зажимов, номинальное сечение проводника 0.08-2.5 мм2</t>
-  </si>
-  <si>
-    <t>Заглушка NO-550-07 для винтовых клемм 2,5мм2 арт. Б0035737</t>
-  </si>
-  <si>
-    <t>Фиксатор ФК-102-01 на DIN-рейку 32057DEK Dekraft 2 арт. 32057DEK</t>
-  </si>
-  <si>
-    <t>DIN-рейка 50см перфорированная adr-50 EKF арт. adr-50</t>
-  </si>
-  <si>
-    <t>Разъем РпИм 1.25-5-0.8 плоский</t>
+    <t>Кабель КВВГЭнг(А)-LS-ХЛ 4х1,0</t>
+  </si>
+  <si>
+    <t>Кабель КВВГЭнг(А)-LS-ХЛ 7х1,0</t>
+  </si>
+  <si>
+    <t>Кабель ВВГнг(А)-LS-ХЛ 3x2,5 d7.2мм</t>
+  </si>
+  <si>
+    <t>Кабель КПСЭнг(A)-FRLS 4х2х0,75</t>
+  </si>
+  <si>
+    <t>Кабель-канал 40х40 перфорированный Plast kk40-40 EKF</t>
+  </si>
+  <si>
+    <t>Провод ПуГВнг(А)-LS 1x0,75</t>
+  </si>
+  <si>
+    <t>Провод ПуГВнг(А)-LS 1x1,5</t>
+  </si>
+  <si>
+    <t>Провод Rd8</t>
+  </si>
+  <si>
+    <t>Угол горизонтальный CPO 90 (50 х 50)</t>
   </si>
   <si>
     <t>Наконечник кабельный НШвИ 0,75мм</t>
@@ -294,6 +396,18 @@
     <t>Наконечник кабельный НШвИ 2,5мм</t>
   </si>
   <si>
+    <t>Крепление для труб ПВХ с защелкой, 16 мм</t>
+  </si>
+  <si>
+    <t>Резьбовой крепежный элемент с наружной резьбой РКН-15 (ММРн-15)</t>
+  </si>
+  <si>
+    <t>Резьбовой крепежный элемент с внутренней резьбой Ркв-15</t>
+  </si>
+  <si>
+    <t>Угол горизонтальный CPO 90 (100 х 50)</t>
+  </si>
+  <si>
     <t>Крышка Угол горизонтальный CPO 90 (100х50)</t>
   </si>
   <si>
@@ -303,102 +417,12 @@
     <t>Крышка на угол вертикальный внешний CD90 (100х50)</t>
   </si>
   <si>
-    <t>Угол вертикальный внутренний CS 90 100 х 50мм</t>
-  </si>
-  <si>
-    <t>Крышка на угол вертикальный внутренний CS 90 100 х 50мм</t>
-  </si>
-  <si>
-    <t>Монтажная рама РВМ 4.1.1</t>
-  </si>
-  <si>
-    <t>Ответная рама РВО 4.1.1</t>
-  </si>
-  <si>
-    <t>Уплотнительный модуль МКС 40/Ø 17-34 мм</t>
-  </si>
-  <si>
-    <t>Уплотнительный модуль МКС 20/Ø 5-14 мм</t>
-  </si>
-  <si>
-    <t>Компрессионный блок МКС КБ 120</t>
-  </si>
-  <si>
-    <t>Пластина анкерная 120</t>
-  </si>
-  <si>
-    <t>Кабель ВВГнг(А)-LS-ХЛ 3x2,5 d8мм</t>
-  </si>
-  <si>
-    <t>Короб ПВХ  40х25 мм</t>
-  </si>
-  <si>
-    <t>Короб ПВХ 40х40 мм</t>
-  </si>
-  <si>
-    <t>Металлорукав в ПВХ изоляции РЗ-ЦП-15</t>
-  </si>
-  <si>
-    <t>Провод Rd8</t>
-  </si>
-  <si>
-    <t>Провод ПуГВнг(А)-LS 1x1,5</t>
-  </si>
-  <si>
-    <t>Провод ПуГВнг(А)-LS 1x0,75</t>
-  </si>
-  <si>
-    <t>Кабель-канал 40х40 перфорированный Plast kk40-40 EKF</t>
-  </si>
-  <si>
-    <t>Кабель КПСЭнг(A)-FRLS 4х2х0,75</t>
-  </si>
-  <si>
-    <t>Кабель ВВГнг(А)-LS-ХЛ 3x2,5 d7.2мм</t>
-  </si>
-  <si>
-    <t>Кабель КВВГЭнг(А)-LS-ХЛ 7х1,0</t>
-  </si>
-  <si>
-    <t>Кабель КВВГЭнг(А)-LS-ХЛ 4х1,0</t>
-  </si>
-  <si>
-    <t>Кабель ВВГнг(А)-LS-ХЛ 4x1,5 d10,2мм</t>
-  </si>
-  <si>
-    <t>Шина заземления на DIN-изолятор ШНИ-6х9-8</t>
+    <t>Крышка Угол горизонтальный CPO 90 (50х50)</t>
   </si>
   <si>
     <t>Выключатель автоматический двухполюсный 3А B ВА47-29 4.5кА MVA20-2-003-B IEK</t>
   </si>
   <si>
-    <t>Угол горизонтальный CPO 90 (100 х 50)</t>
-  </si>
-  <si>
-    <t>Резьбовой крепежный элемент с внутренней резьбой Ркв-15</t>
-  </si>
-  <si>
-    <t>Резьбовой крепежный элемент с наружной резьбой РКН-15 (ММРн-15)</t>
-  </si>
-  <si>
-    <t>Крепление для труб ПВХ с защелкой, 16 мм</t>
-  </si>
-  <si>
-    <t>Скоба металлическая СМО 16-17 49152 КВТ</t>
-  </si>
-  <si>
-    <t>MV-клемма проводника Rd8</t>
-  </si>
-  <si>
-    <t>Держатель для полосы заземления К-188 У2 (цинк)</t>
-  </si>
-  <si>
-    <t>Коробка клеммная К-СП 08.13.09 24/11П 2КВе-Л-М20(А)-2КВе-Л-М20(В) 1ExeLLCGbXT6 ip66,80х130х90</t>
-  </si>
-  <si>
-    <t>Выключатель двухклавишный IP55</t>
-  </si>
-  <si>
     <t>Выключатель автоматический двухполюсный IEK ARMAT M10N 2P B 10А AR-M10N-2-B010</t>
   </si>
   <si>
@@ -426,10 +450,16 @@
     <t>Угол вертикальный внешний CD 90 (50 х 50)</t>
   </si>
   <si>
-    <t>Крышка Угол горизонтальный CPO 90 (50х50)</t>
-  </si>
-  <si>
-    <t>Угол горизонтальный CPO 90 (50 х 50)</t>
+    <t>Кольцо 055-060-30-2-2 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Кольцо 065-075-58 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Кольцо 080-090-58-2-2 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Пружина ПСМНТ.001.000.030</t>
   </si>
   <si>
     <t>Прокладка медная 8х11-II ГОСТ 19752-84</t>
@@ -441,76 +471,58 @@
     <t>Кольцо 112-118-36 ГОСТ 9833-73</t>
   </si>
   <si>
-    <t>Кольцо 055-060-30-2-2 ГОСТ 9833-73</t>
-  </si>
-  <si>
-    <t>Пружина ПСМНТ.001.000.030</t>
-  </si>
-  <si>
-    <t>Кольцо 080-090-58-2-2 ГОСТ 9833-73</t>
-  </si>
-  <si>
-    <t>Кольцо 065-075-58 ГОСТ 9833-73</t>
-  </si>
-  <si>
     <t>Уплотнение ПСМНТ.001.022.002</t>
   </si>
   <si>
-    <t>Обогреватель взрывозащищенный ОВЭ-4-УХЛ3 1,8 кВт, 380В IExdIIАТ3, IP54</t>
-  </si>
-  <si>
-    <t>Пост кнопочный взрывозащищенный ПВК-15 IP65 2ExеdIIСТ6</t>
-  </si>
-  <si>
-    <t>Пост кнопочный взрывозащищенный ПВК-25-ХЛ1 управление обогревом IP65 2ExеdIIСТ6</t>
-  </si>
-  <si>
-    <t>Светильник взрывозащищенный ДБП 09-15-001 УХЛ1 ExdllBT6G IP65</t>
-  </si>
-  <si>
-    <t>Датчик давления взрывозащ. СТИ775Ц-E-1-M-D-B-H-T-1</t>
+    <t>Круг D195 Ст.16ГС-3 ГОСТ 5520-79</t>
+  </si>
+  <si>
+    <t>Круг D430 Ст.16ГС ГОСТ 19281-14</t>
+  </si>
+  <si>
+    <t>Круг D70 Ст.40Х ГОСТ 4543-71</t>
+  </si>
+  <si>
+    <t>Круг D45 Ст.40Х ГОСТ 4543-71</t>
+  </si>
+  <si>
+    <t>Круг D370 Ст.20 ГОСТ1050-88</t>
+  </si>
+  <si>
+    <t>Шестигранник S=14 Ст.45 ГОСТ 1050-88</t>
   </si>
   <si>
     <t>Лист Б-ПР-1,0 ГОСТ 19904-74/ 4-III-Ст3кп ГОСТ 16523-89</t>
   </si>
   <si>
-    <t>Шестигранник S=14 Ст.45 ГОСТ 1050-88</t>
-  </si>
-  <si>
-    <t>Круг D370 Ст.20 ГОСТ1050-88</t>
-  </si>
-  <si>
-    <t>Круг D45 Ст.40Х ГОСТ 4543-71</t>
-  </si>
-  <si>
-    <t>Круг D70 Ст.40Х ГОСТ 4543-71</t>
-  </si>
-  <si>
-    <t>Круг D430 Ст.16ГС ГОСТ 19281-14</t>
-  </si>
-  <si>
-    <t>Круг D195 Ст.16ГС-3 ГОСТ 5520-79</t>
-  </si>
-  <si>
     <t>Шарик 25,4-100 ГОСТ 3722-81</t>
   </si>
   <si>
+    <t>Винт М16х50.56.019 ГОСТ 1481-84</t>
+  </si>
+  <si>
+    <t>Заклепка 2х4х37 Ан.Окс.хр. ГОСТ10299-80</t>
+  </si>
+  <si>
     <t>Шпилька М18х40.56.019 ГОСТ 22034-76</t>
   </si>
   <si>
-    <t>Заклепка 2х4х37 Ан.Окс.хр. ГОСТ10299-80</t>
-  </si>
-  <si>
-    <t>Винт М16х50.56.019 ГОСТ 1481-84</t>
-  </si>
-  <si>
-    <t>Кабель ВВГнг(А)-FRLS 3x1,5 d7,2мм</t>
-  </si>
-  <si>
-    <t>Оповещатель светозвуковой Маяк-24К IP53</t>
-  </si>
-  <si>
-    <t>Извещатель пожарный дымовой ИП 212-141М</t>
+    <t>Розетка для реле 2 СО</t>
+  </si>
+  <si>
+    <t>Промежуточное реле 2 CO контакта 24в DC</t>
+  </si>
+  <si>
+    <t>Клемма пружинная Push-in CP-ML 2 ур. 4мм2 серая IEK YCT23-00-2-K03-004 IEK</t>
+  </si>
+  <si>
+    <t>Заглушка для CP-ML 2 ур. 4мм2 серая IEK YCT23-00-2-K03-004-ZGL IEK</t>
+  </si>
+  <si>
+    <t>Фланец 3-450-40 09Г2С ГОСТ 12815-80 (из поковки гр.IV КП 245 ГОСТ 8479-70)</t>
+  </si>
+  <si>
+    <t>Сгон ДУ20 L-120 12Х18Н10Т</t>
   </si>
 </sst>
 </file>
@@ -947,12 +959,12 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F138"/>
+  <dimension ref="A1:F146"/>
   <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="11.45" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.1640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="46.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="74.83203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="75" style="1" customWidth="1"/>
     <col min="4" max="4" width="14.1640625" style="1" customWidth="1"/>
     <col min="5" max="5" width="13" style="1" customWidth="1"/>
     <col min="6" max="6" width="14.5" style="1" customWidth="1"/>
@@ -984,7 +996,7 @@
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="8" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="D2" s="5">
         <v>120</v>
@@ -1002,7 +1014,7 @@
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="8" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="D3" s="5">
         <v>0.25</v>
@@ -1020,16 +1032,16 @@
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="8" t="s">
-        <v>9</v>
+        <v>71</v>
       </c>
       <c r="D4" s="5">
         <v>40</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1038,16 +1050,16 @@
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D5" s="5">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1056,16 +1068,16 @@
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="8" t="s">
-        <v>65</v>
+        <v>12</v>
       </c>
       <c r="D6" s="5">
-        <v>40</v>
+        <v>500</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1074,16 +1086,16 @@
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D7" s="5">
-        <v>500</v>
+        <v>800</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1092,16 +1104,16 @@
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D8" s="5">
-        <v>800</v>
+        <v>10</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1110,16 +1122,16 @@
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="8" t="s">
-        <v>66</v>
+        <v>17</v>
       </c>
       <c r="D9" s="5">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1128,16 +1140,16 @@
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D10" s="5">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1146,16 +1158,16 @@
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D11" s="5">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1164,16 +1176,16 @@
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D12" s="5">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1182,16 +1194,16 @@
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="8" t="s">
-        <v>20</v>
+        <v>72</v>
       </c>
       <c r="D13" s="5">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1203,13 +1215,13 @@
         <v>21</v>
       </c>
       <c r="D14" s="5">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1221,13 +1233,13 @@
         <v>22</v>
       </c>
       <c r="D15" s="5">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1239,10 +1251,10 @@
         <v>23</v>
       </c>
       <c r="D16" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F16" s="4" t="s">
         <v>24</v>
@@ -1257,10 +1269,10 @@
         <v>25</v>
       </c>
       <c r="D17" s="5">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>24</v>
@@ -1278,7 +1290,7 @@
         <v>10</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>24</v>
@@ -1290,13 +1302,13 @@
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D19" s="5">
         <v>10</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>24</v>
@@ -1314,7 +1326,7 @@
         <v>10</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>24</v>
@@ -1329,10 +1341,10 @@
         <v>30</v>
       </c>
       <c r="D21" s="5">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F21" s="4" t="s">
         <v>24</v>
@@ -1350,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F22" s="4" t="s">
         <v>24</v>
@@ -1365,10 +1377,10 @@
         <v>32</v>
       </c>
       <c r="D23" s="5">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>24</v>
@@ -1383,10 +1395,10 @@
         <v>33</v>
       </c>
       <c r="D24" s="5">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>24</v>
@@ -1404,7 +1416,7 @@
         <v>10</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>24</v>
@@ -1416,10 +1428,10 @@
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="8" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="D26" s="5">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>6</v>
@@ -1434,10 +1446,10 @@
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="8" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D27" s="5">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>6</v>
@@ -1455,10 +1467,10 @@
         <v>36</v>
       </c>
       <c r="D28" s="5">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F28" s="4" t="s">
         <v>35</v>
@@ -1473,10 +1485,10 @@
         <v>37</v>
       </c>
       <c r="D29" s="5">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F29" s="4" t="s">
         <v>35</v>
@@ -1494,7 +1506,7 @@
         <v>18</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F30" s="4" t="s">
         <v>35</v>
@@ -1524,10 +1536,10 @@
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="8" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="D32" s="5">
-        <v>53.25</v>
+        <v>0.2</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>8</v>
@@ -1542,10 +1554,10 @@
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="8" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="D33" s="5">
-        <v>0.2</v>
+        <v>53.25</v>
       </c>
       <c r="E33" s="6" t="s">
         <v>8</v>
@@ -1560,7 +1572,7 @@
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="8" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="D34" s="5">
         <v>25</v>
@@ -1578,10 +1590,10 @@
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="8" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="D35" s="5">
-        <v>49</v>
+        <v>271.75</v>
       </c>
       <c r="E35" s="6" t="s">
         <v>8</v>
@@ -1596,10 +1608,10 @@
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="D36" s="5">
-        <v>99.25</v>
+        <v>79</v>
+      </c>
+      <c r="D36" s="7">
+        <v>4286.5</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>8</v>
@@ -1614,7 +1626,7 @@
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="8" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="D37" s="5">
         <v>18.25</v>
@@ -1632,10 +1644,10 @@
       </c>
       <c r="B38" s="4"/>
       <c r="C38" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="D38" s="7">
-        <v>4286.5</v>
+        <v>81</v>
+      </c>
+      <c r="D38" s="5">
+        <v>99.25</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>8</v>
@@ -1650,10 +1662,10 @@
       </c>
       <c r="B39" s="4"/>
       <c r="C39" s="8" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="D39" s="5">
-        <v>148.5</v>
+        <v>49</v>
       </c>
       <c r="E39" s="6" t="s">
         <v>8</v>
@@ -1668,7 +1680,7 @@
       </c>
       <c r="B40" s="4"/>
       <c r="C40" s="8" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="D40" s="5">
         <v>37.35</v>
@@ -1686,10 +1698,10 @@
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="8" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D41" s="5">
-        <v>271.75</v>
+        <v>148.5</v>
       </c>
       <c r="E41" s="6" t="s">
         <v>8</v>
@@ -1704,10 +1716,10 @@
       </c>
       <c r="B42" s="4"/>
       <c r="C42" s="8" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="D42" s="5">
-        <v>2.1</v>
+        <v>130</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>44</v>
@@ -1722,10 +1734,10 @@
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="8" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="D43" s="5">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>6</v>
@@ -1740,10 +1752,10 @@
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="8" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
       <c r="D44" s="5">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>6</v>
@@ -1758,10 +1770,10 @@
       </c>
       <c r="B45" s="4"/>
       <c r="C45" s="8" t="s">
-        <v>46</v>
+        <v>87</v>
       </c>
       <c r="D45" s="5">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>6</v>
@@ -1776,7 +1788,7 @@
       </c>
       <c r="B46" s="4"/>
       <c r="C46" s="8" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="D46" s="5">
         <v>2</v>
@@ -1794,10 +1806,10 @@
       </c>
       <c r="B47" s="4"/>
       <c r="C47" s="8" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="D47" s="5">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>6</v>
@@ -1812,10 +1824,10 @@
       </c>
       <c r="B48" s="4"/>
       <c r="C48" s="8" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="D48" s="5">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>6</v>
@@ -1830,10 +1842,10 @@
       </c>
       <c r="B49" s="4"/>
       <c r="C49" s="8" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="D49" s="5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E49" s="6" t="s">
         <v>6</v>
@@ -1848,10 +1860,10 @@
       </c>
       <c r="B50" s="4"/>
       <c r="C50" s="8" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="D50" s="5">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>6</v>
@@ -1866,10 +1878,10 @@
       </c>
       <c r="B51" s="4"/>
       <c r="C51" s="8" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="D51" s="5">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>6</v>
@@ -1884,10 +1896,10 @@
       </c>
       <c r="B52" s="4"/>
       <c r="C52" s="8" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="D52" s="5">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>6</v>
@@ -1902,10 +1914,10 @@
       </c>
       <c r="B53" s="4"/>
       <c r="C53" s="8" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="D53" s="5">
-        <v>4</v>
+        <v>135</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>6</v>
@@ -1920,7 +1932,7 @@
       </c>
       <c r="B54" s="4"/>
       <c r="C54" s="8" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D54" s="5">
         <v>4</v>
@@ -1938,10 +1950,10 @@
       </c>
       <c r="B55" s="4"/>
       <c r="C55" s="8" t="s">
-        <v>91</v>
+        <v>47</v>
       </c>
       <c r="D55" s="5">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="E55" s="6" t="s">
         <v>6</v>
@@ -1956,10 +1968,10 @@
       </c>
       <c r="B56" s="4"/>
       <c r="C56" s="8" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D56" s="5">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>6</v>
@@ -1974,10 +1986,10 @@
       </c>
       <c r="B57" s="4"/>
       <c r="C57" s="8" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D57" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E57" s="6" t="s">
         <v>6</v>
@@ -1992,7 +2004,7 @@
       </c>
       <c r="B58" s="4"/>
       <c r="C58" s="8" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="D58" s="5">
         <v>1</v>
@@ -2010,10 +2022,10 @@
       </c>
       <c r="B59" s="4"/>
       <c r="C59" s="8" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="D59" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E59" s="6" t="s">
         <v>6</v>
@@ -2028,10 +2040,10 @@
       </c>
       <c r="B60" s="4"/>
       <c r="C60" s="8" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="D60" s="5">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>6</v>
@@ -2046,10 +2058,10 @@
       </c>
       <c r="B61" s="4"/>
       <c r="C61" s="8" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="D61" s="5">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E61" s="6" t="s">
         <v>6</v>
@@ -2064,7 +2076,7 @@
       </c>
       <c r="B62" s="4"/>
       <c r="C62" s="8" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="D62" s="5">
         <v>2</v>
@@ -2082,10 +2094,10 @@
       </c>
       <c r="B63" s="4"/>
       <c r="C63" s="8" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="D63" s="5">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E63" s="6" t="s">
         <v>6</v>
@@ -2100,13 +2112,13 @@
       </c>
       <c r="B64" s="4"/>
       <c r="C64" s="8" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="D64" s="5">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="F64" s="4" t="s">
         <v>45</v>
@@ -2118,10 +2130,10 @@
       </c>
       <c r="B65" s="4"/>
       <c r="C65" s="8" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D65" s="5">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E65" s="6" t="s">
         <v>44</v>
@@ -2136,10 +2148,10 @@
       </c>
       <c r="B66" s="4"/>
       <c r="C66" s="8" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D66" s="5">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>44</v>
@@ -2154,10 +2166,10 @@
       </c>
       <c r="B67" s="4"/>
       <c r="C67" s="8" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="D67" s="5">
-        <v>130</v>
+        <v>15</v>
       </c>
       <c r="E67" s="6" t="s">
         <v>44</v>
@@ -2172,10 +2184,10 @@
       </c>
       <c r="B68" s="4"/>
       <c r="C68" s="8" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="D68" s="5">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>44</v>
@@ -2190,10 +2202,10 @@
       </c>
       <c r="B69" s="4"/>
       <c r="C69" s="8" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="D69" s="5">
-        <v>8</v>
+        <v>2.1</v>
       </c>
       <c r="E69" s="6" t="s">
         <v>44</v>
@@ -2208,10 +2220,10 @@
       </c>
       <c r="B70" s="4"/>
       <c r="C70" s="8" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D70" s="5">
-        <v>2</v>
+        <v>112</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>44</v>
@@ -2226,10 +2238,10 @@
       </c>
       <c r="B71" s="4"/>
       <c r="C71" s="8" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="D71" s="5">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="E71" s="6" t="s">
         <v>44</v>
@@ -2244,10 +2256,10 @@
       </c>
       <c r="B72" s="4"/>
       <c r="C72" s="8" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="D72" s="5">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>44</v>
@@ -2262,10 +2274,10 @@
       </c>
       <c r="B73" s="4"/>
       <c r="C73" s="8" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D73" s="5">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E73" s="6" t="s">
         <v>44</v>
@@ -2280,10 +2292,10 @@
       </c>
       <c r="B74" s="4"/>
       <c r="C74" s="8" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="D74" s="5">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>44</v>
@@ -2298,10 +2310,10 @@
       </c>
       <c r="B75" s="4"/>
       <c r="C75" s="8" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="D75" s="5">
-        <v>112</v>
+        <v>2</v>
       </c>
       <c r="E75" s="6" t="s">
         <v>44</v>
@@ -2316,10 +2328,10 @@
       </c>
       <c r="B76" s="4"/>
       <c r="C76" s="8" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="D76" s="5">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>44</v>
@@ -2334,13 +2346,13 @@
       </c>
       <c r="B77" s="4"/>
       <c r="C77" s="8" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="D77" s="5">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E77" s="6" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="F77" s="4" t="s">
         <v>45</v>
@@ -2352,7 +2364,7 @@
       </c>
       <c r="B78" s="4"/>
       <c r="C78" s="8" t="s">
-        <v>114</v>
+        <v>48</v>
       </c>
       <c r="D78" s="5">
         <v>1</v>
@@ -2370,10 +2382,10 @@
       </c>
       <c r="B79" s="4"/>
       <c r="C79" s="8" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D79" s="5">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E79" s="6" t="s">
         <v>6</v>
@@ -2388,10 +2400,10 @@
       </c>
       <c r="B80" s="4"/>
       <c r="C80" s="8" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="D80" s="5">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>6</v>
@@ -2406,10 +2418,10 @@
       </c>
       <c r="B81" s="4"/>
       <c r="C81" s="8" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D81" s="5">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="E81" s="6" t="s">
         <v>6</v>
@@ -2424,10 +2436,10 @@
       </c>
       <c r="B82" s="4"/>
       <c r="C82" s="8" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D82" s="5">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>6</v>
@@ -2442,10 +2454,10 @@
       </c>
       <c r="B83" s="4"/>
       <c r="C83" s="8" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D83" s="5">
-        <v>135</v>
+        <v>40</v>
       </c>
       <c r="E83" s="6" t="s">
         <v>6</v>
@@ -2460,10 +2472,10 @@
       </c>
       <c r="B84" s="4"/>
       <c r="C84" s="8" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="D84" s="5">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>6</v>
@@ -2478,10 +2490,10 @@
       </c>
       <c r="B85" s="4"/>
       <c r="C85" s="8" t="s">
-        <v>47</v>
+        <v>125</v>
       </c>
       <c r="D85" s="5">
-        <v>70</v>
+        <v>48</v>
       </c>
       <c r="E85" s="6" t="s">
         <v>6</v>
@@ -2496,10 +2508,10 @@
       </c>
       <c r="B86" s="4"/>
       <c r="C86" s="8" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="D86" s="5">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>6</v>
@@ -2514,10 +2526,10 @@
       </c>
       <c r="B87" s="4"/>
       <c r="C87" s="8" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D87" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E87" s="6" t="s">
         <v>6</v>
@@ -2532,10 +2544,10 @@
       </c>
       <c r="B88" s="4"/>
       <c r="C88" s="8" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="D88" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>6</v>
@@ -2550,10 +2562,10 @@
       </c>
       <c r="B89" s="4"/>
       <c r="C89" s="8" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="D89" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E89" s="6" t="s">
         <v>6</v>
@@ -2568,10 +2580,10 @@
       </c>
       <c r="B90" s="4"/>
       <c r="C90" s="8" t="s">
-        <v>48</v>
+        <v>130</v>
       </c>
       <c r="D90" s="5">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>6</v>
@@ -2586,7 +2598,7 @@
       </c>
       <c r="B91" s="4"/>
       <c r="C91" s="8" t="s">
-        <v>49</v>
+        <v>131</v>
       </c>
       <c r="D91" s="5">
         <v>1</v>
@@ -2604,7 +2616,7 @@
       </c>
       <c r="B92" s="4"/>
       <c r="C92" s="8" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="D92" s="5">
         <v>1</v>
@@ -2622,7 +2634,7 @@
       </c>
       <c r="B93" s="4"/>
       <c r="C93" s="8" t="s">
-        <v>126</v>
+        <v>49</v>
       </c>
       <c r="D93" s="5">
         <v>1</v>
@@ -2640,10 +2652,10 @@
       </c>
       <c r="B94" s="4"/>
       <c r="C94" s="8" t="s">
-        <v>127</v>
+        <v>50</v>
       </c>
       <c r="D94" s="5">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>6</v>
@@ -2658,7 +2670,7 @@
       </c>
       <c r="B95" s="4"/>
       <c r="C95" s="8" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D95" s="5">
         <v>1</v>
@@ -2676,10 +2688,10 @@
       </c>
       <c r="B96" s="4"/>
       <c r="C96" s="8" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="D96" s="5">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>6</v>
@@ -2694,10 +2706,10 @@
       </c>
       <c r="B97" s="4"/>
       <c r="C97" s="8" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="D97" s="5">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E97" s="6" t="s">
         <v>6</v>
@@ -2712,10 +2724,10 @@
       </c>
       <c r="B98" s="4"/>
       <c r="C98" s="8" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="D98" s="5">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>6</v>
@@ -2730,7 +2742,7 @@
       </c>
       <c r="B99" s="4"/>
       <c r="C99" s="8" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="D99" s="5">
         <v>8</v>
@@ -2748,7 +2760,7 @@
       </c>
       <c r="B100" s="4"/>
       <c r="C100" s="8" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="D100" s="5">
         <v>8</v>
@@ -2766,10 +2778,10 @@
       </c>
       <c r="B101" s="4"/>
       <c r="C101" s="8" t="s">
-        <v>50</v>
+        <v>139</v>
       </c>
       <c r="D101" s="5">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E101" s="6" t="s">
         <v>6</v>
@@ -2784,7 +2796,7 @@
       </c>
       <c r="B102" s="4"/>
       <c r="C102" s="8" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="D102" s="5">
         <v>8</v>
@@ -2802,10 +2814,10 @@
       </c>
       <c r="B103" s="4"/>
       <c r="C103" s="8" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="D103" s="5">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="E103" s="6" t="s">
         <v>6</v>
@@ -2820,10 +2832,10 @@
       </c>
       <c r="B104" s="4"/>
       <c r="C104" s="8" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="D104" s="5">
-        <v>80</v>
+        <v>170</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>6</v>
@@ -2838,10 +2850,10 @@
       </c>
       <c r="B105" s="4"/>
       <c r="C105" s="8" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="D105" s="5">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="E105" s="6" t="s">
         <v>6</v>
@@ -2856,7 +2868,7 @@
       </c>
       <c r="B106" s="4"/>
       <c r="C106" s="8" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D106" s="5">
         <v>25</v>
@@ -2874,10 +2886,10 @@
       </c>
       <c r="B107" s="4"/>
       <c r="C107" s="8" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="D107" s="5">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="E107" s="6" t="s">
         <v>6</v>
@@ -2892,10 +2904,10 @@
       </c>
       <c r="B108" s="4"/>
       <c r="C108" s="8" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="D108" s="5">
-        <v>25</v>
+        <v>80</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>6</v>
@@ -2910,10 +2922,10 @@
       </c>
       <c r="B109" s="4"/>
       <c r="C109" s="8" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="D109" s="5">
-        <v>170</v>
+        <v>50</v>
       </c>
       <c r="E109" s="6" t="s">
         <v>6</v>
@@ -2928,160 +2940,160 @@
       </c>
       <c r="B110" s="4"/>
       <c r="C110" s="8" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="D110" s="5">
         <v>25</v>
       </c>
       <c r="E110" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F110" s="4" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="111" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="3">
         <v>110</v>
       </c>
       <c r="B111" s="4"/>
       <c r="C111" s="8" t="s">
-        <v>143</v>
+        <v>52</v>
       </c>
       <c r="D111" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E111" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F111" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="112" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="3">
         <v>111</v>
       </c>
       <c r="B112" s="4"/>
       <c r="C112" s="8" t="s">
-        <v>53</v>
+        <v>149</v>
       </c>
       <c r="D112" s="5">
-        <v>2</v>
+        <v>291</v>
       </c>
       <c r="E112" s="6" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F112" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="3">
         <v>112</v>
       </c>
       <c r="B113" s="4"/>
       <c r="C113" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="D113" s="5">
-        <v>2</v>
+        <v>150</v>
+      </c>
+      <c r="D113" s="7">
+        <v>1415.25</v>
       </c>
       <c r="E113" s="6" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F113" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="114" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="3">
         <v>113</v>
       </c>
       <c r="B114" s="4"/>
       <c r="C114" s="8" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="D114" s="5">
-        <v>2</v>
+        <v>26.5</v>
       </c>
       <c r="E114" s="6" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F114" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="115" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="3">
         <v>114</v>
       </c>
       <c r="B115" s="4"/>
       <c r="C115" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="D115" s="5">
+        <v>131</v>
+      </c>
+      <c r="E115" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F115" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D115" s="5">
-        <v>2</v>
-      </c>
-      <c r="E115" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="F115" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="116" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="116" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="3">
         <v>115</v>
       </c>
       <c r="B116" s="4"/>
       <c r="C116" s="8" t="s">
-        <v>55</v>
+        <v>153</v>
       </c>
       <c r="D116" s="5">
-        <v>1</v>
+        <v>950</v>
       </c>
       <c r="E116" s="6" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F116" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="117" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="3">
         <v>116</v>
       </c>
       <c r="B117" s="4"/>
       <c r="C117" s="8" t="s">
-        <v>56</v>
+        <v>154</v>
       </c>
       <c r="D117" s="5">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="E117" s="6" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F117" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="118" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="3">
         <v>117</v>
       </c>
       <c r="B118" s="4"/>
       <c r="C118" s="8" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="D118" s="5">
-        <v>6</v>
+        <v>1.5</v>
       </c>
       <c r="E118" s="6" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F118" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="119" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3090,16 +3102,16 @@
       </c>
       <c r="B119" s="4"/>
       <c r="C119" s="8" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="D119" s="5">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="E119" s="6" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="F119" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="120" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3108,160 +3120,160 @@
       </c>
       <c r="B120" s="4"/>
       <c r="C120" s="8" t="s">
-        <v>57</v>
+        <v>157</v>
       </c>
       <c r="D120" s="5">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="E120" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F120" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="3">
         <v>120</v>
       </c>
       <c r="B121" s="4"/>
       <c r="C121" s="8" t="s">
-        <v>58</v>
+        <v>158</v>
       </c>
       <c r="D121" s="5">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="E121" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F121" s="4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="122" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="3">
         <v>121</v>
       </c>
       <c r="B122" s="4"/>
       <c r="C122" s="8" t="s">
-        <v>148</v>
+        <v>159</v>
       </c>
       <c r="D122" s="5">
-        <v>1.5</v>
+        <v>500</v>
       </c>
       <c r="E122" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F122" s="4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="123" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="3">
         <v>122</v>
       </c>
       <c r="B123" s="4"/>
       <c r="C123" s="8" t="s">
-        <v>149</v>
+        <v>56</v>
       </c>
       <c r="D123" s="5">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="E123" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F123" s="4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="124" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="3">
         <v>123</v>
       </c>
       <c r="B124" s="4"/>
       <c r="C124" s="8" t="s">
-        <v>150</v>
+        <v>58</v>
       </c>
       <c r="D124" s="5">
-        <v>950</v>
+        <v>40</v>
       </c>
       <c r="E124" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F124" s="4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="125" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="3">
         <v>124</v>
       </c>
       <c r="B125" s="4"/>
       <c r="C125" s="8" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="D125" s="5">
-        <v>131</v>
+        <v>3</v>
       </c>
       <c r="E125" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F125" s="4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="126" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="3">
         <v>125</v>
       </c>
       <c r="B126" s="4"/>
       <c r="C126" s="8" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="D126" s="5">
-        <v>26.5</v>
+        <v>3</v>
       </c>
       <c r="E126" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F126" s="4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="127" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="3">
         <v>126</v>
       </c>
       <c r="B127" s="4"/>
       <c r="C127" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="D127" s="7">
-        <v>1415.25</v>
+        <v>162</v>
+      </c>
+      <c r="D127" s="5">
+        <v>16</v>
       </c>
       <c r="E127" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F127" s="4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="128" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="3">
         <v>127</v>
       </c>
       <c r="B128" s="4"/>
       <c r="C128" s="8" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="D128" s="5">
-        <v>291</v>
+        <v>6</v>
       </c>
       <c r="E128" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F128" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="129" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3270,16 +3282,16 @@
       </c>
       <c r="B129" s="4"/>
       <c r="C129" s="8" t="s">
-        <v>155</v>
+        <v>60</v>
       </c>
       <c r="D129" s="5">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E129" s="6" t="s">
-        <v>10</v>
+        <v>44</v>
       </c>
       <c r="F129" s="4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="130" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3288,10 +3300,10 @@
       </c>
       <c r="B130" s="4"/>
       <c r="C130" s="8" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="D130" s="5">
-        <v>500</v>
+        <v>9</v>
       </c>
       <c r="E130" s="6" t="s">
         <v>6</v>
@@ -3306,10 +3318,10 @@
       </c>
       <c r="B131" s="4"/>
       <c r="C131" s="8" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="D131" s="5">
-        <v>50</v>
+        <v>9</v>
       </c>
       <c r="E131" s="6" t="s">
         <v>6</v>
@@ -3324,10 +3336,10 @@
       </c>
       <c r="B132" s="4"/>
       <c r="C132" s="8" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="D132" s="5">
-        <v>100</v>
+        <v>48</v>
       </c>
       <c r="E132" s="6" t="s">
         <v>6</v>
@@ -3336,70 +3348,70 @@
         <v>61</v>
       </c>
     </row>
-    <row r="133" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" s="3">
         <v>132</v>
       </c>
       <c r="B133" s="4"/>
       <c r="C133" s="8" t="s">
-        <v>159</v>
+        <v>60</v>
       </c>
       <c r="D133" s="5">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="E133" s="6" t="s">
         <v>44</v>
       </c>
       <c r="F133" s="4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="134" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" s="3">
         <v>133</v>
       </c>
       <c r="B134" s="4"/>
       <c r="C134" s="8" t="s">
-        <v>101</v>
+        <v>58</v>
       </c>
       <c r="D134" s="5">
-        <v>24</v>
+        <v>120</v>
       </c>
       <c r="E134" s="6" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="F134" s="4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="135" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" s="3">
         <v>134</v>
       </c>
       <c r="B135" s="4"/>
       <c r="C135" s="8" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="D135" s="5">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="E135" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F135" s="4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="136" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="3">
         <v>135</v>
       </c>
       <c r="B136" s="4"/>
       <c r="C136" s="8" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D136" s="5">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="E136" s="6" t="s">
         <v>6</v>
@@ -3408,40 +3420,184 @@
         <v>62</v>
       </c>
     </row>
-    <row r="137" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="3">
         <v>136</v>
       </c>
       <c r="B137" s="4"/>
       <c r="C137" s="8" t="s">
-        <v>118</v>
+        <v>58</v>
       </c>
       <c r="D137" s="5">
-        <v>30</v>
+        <v>160</v>
       </c>
       <c r="E137" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F137" s="4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="138" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="3">
         <v>137</v>
       </c>
       <c r="B138" s="4"/>
       <c r="C138" s="8" t="s">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="D138" s="5">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E138" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F138" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A139" s="3">
+        <v>138</v>
+      </c>
+      <c r="B139" s="4"/>
+      <c r="C139" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="D139" s="5">
+        <v>12</v>
+      </c>
+      <c r="E139" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F139" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A140" s="3">
+        <v>139</v>
+      </c>
+      <c r="B140" s="4"/>
+      <c r="C140" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="D140" s="5">
+        <v>64</v>
+      </c>
+      <c r="E140" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F140" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A141" s="3">
+        <v>140</v>
+      </c>
+      <c r="B141" s="4"/>
+      <c r="C141" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="D141" s="5">
+        <v>24</v>
+      </c>
+      <c r="E141" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F141" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A142" s="3">
+        <v>141</v>
+      </c>
+      <c r="B142" s="4"/>
+      <c r="C142" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D142" s="5">
+        <v>80</v>
+      </c>
+      <c r="E142" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F142" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A143" s="3">
+        <v>142</v>
+      </c>
+      <c r="B143" s="4"/>
+      <c r="C143" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D143" s="5">
+        <v>250</v>
+      </c>
+      <c r="E143" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F143" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A144" s="3">
+        <v>143</v>
+      </c>
+      <c r="B144" s="4"/>
+      <c r="C144" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="D144" s="5">
+        <v>150</v>
+      </c>
+      <c r="E144" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F144" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A145" s="3">
+        <v>144</v>
+      </c>
+      <c r="B145" s="4"/>
+      <c r="C145" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="D145" s="5">
+        <v>300</v>
+      </c>
+      <c r="E145" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F145" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A146" s="3">
+        <v>145</v>
+      </c>
+      <c r="B146" s="4"/>
+      <c r="C146" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D146" s="5">
+        <v>5</v>
+      </c>
+      <c r="E146" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F146" s="4" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new Careers, BigPhoto, Question and back-to-top
</commit_message>
<xml_diff>
--- a/public/procurement.xlsx
+++ b/public/procurement.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lka\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{899FF701-B3E4-4D5E-B966-3ED39BF75F9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2E8650F-B0FA-43C8-AEFE-246D339F49B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4755" yWindow="3270" windowWidth="23730" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="210">
   <si>
     <t>№ п/п</t>
   </si>
@@ -48,108 +48,99 @@
     <t>шт</t>
   </si>
   <si>
-    <t>ЛГУП-7413</t>
+    <t>ЛГУП-7331</t>
+  </si>
+  <si>
+    <t>Маркер  краска красный по металлу</t>
+  </si>
+  <si>
+    <t>шт.</t>
+  </si>
+  <si>
+    <t>Перчатки х/б трикотажные 5 нитей 10 класс с ПВХ -Камаз 426</t>
+  </si>
+  <si>
+    <t>пара</t>
+  </si>
+  <si>
+    <t>Перчатки с латесным покрытием</t>
+  </si>
+  <si>
+    <t>пар</t>
+  </si>
+  <si>
+    <t>Огнетушитель ОП-8</t>
+  </si>
+  <si>
+    <t>Маркер по металлу белый</t>
+  </si>
+  <si>
+    <t>Каска строительная оранжевая Исток</t>
+  </si>
+  <si>
+    <t>Ветошь</t>
+  </si>
+  <si>
+    <t>Маркер по металлу черный тонкий</t>
+  </si>
+  <si>
+    <t>Каска строительная белая</t>
+  </si>
+  <si>
+    <t>Маркер белый</t>
+  </si>
+  <si>
+    <t>Ключ комбинированные омедненные 30</t>
+  </si>
+  <si>
+    <t>ЛГУП-7332</t>
+  </si>
+  <si>
+    <t>Ключ комбинированные омедненные 36</t>
+  </si>
+  <si>
+    <t>Ключ комбинированные омедненные 41</t>
+  </si>
+  <si>
+    <t>Гайковерт</t>
+  </si>
+  <si>
+    <t>Ключ комбинированные омедненные 24</t>
+  </si>
+  <si>
+    <t>Трещетка ключ 1/2</t>
+  </si>
+  <si>
+    <t>Ножницы по металлу</t>
+  </si>
+  <si>
+    <t>Резак</t>
+  </si>
+  <si>
+    <t>Ключи обмедненные</t>
+  </si>
+  <si>
+    <t>набор</t>
+  </si>
+  <si>
+    <t>Кувалда 1 кг.</t>
+  </si>
+  <si>
+    <t>Днище 377х10 09Г2С ГОСТ 6533-78</t>
+  </si>
+  <si>
+    <t>ЛГУП-7428</t>
+  </si>
+  <si>
+    <t>Днище 720х12 ст09Г2С ГОСТ 6533-78</t>
+  </si>
+  <si>
+    <t>Днище 820х14-09Г2С ГОСТ 6533-78</t>
   </si>
   <si>
     <t>кг</t>
   </si>
   <si>
-    <t>ЛГУП-7331</t>
-  </si>
-  <si>
-    <t>Маркер  краска красный по металлу</t>
-  </si>
-  <si>
-    <t>шт.</t>
-  </si>
-  <si>
-    <t>Перчатки х/б трикотажные 5 нитей 10 класс с ПВХ -Камаз 426</t>
-  </si>
-  <si>
-    <t>пара</t>
-  </si>
-  <si>
-    <t>Перчатки с латесным покрытием</t>
-  </si>
-  <si>
-    <t>пар</t>
-  </si>
-  <si>
-    <t>Каска строительная оранжевая Исток</t>
-  </si>
-  <si>
-    <t>Огнетушитель ОП-8</t>
-  </si>
-  <si>
-    <t>Маркер по металлу белый</t>
-  </si>
-  <si>
-    <t>Маркер по металлу черный тонкий</t>
-  </si>
-  <si>
-    <t>Каска строительная белая</t>
-  </si>
-  <si>
-    <t>Маркер белый</t>
-  </si>
-  <si>
-    <t>Ветошь</t>
-  </si>
-  <si>
-    <t>Резак</t>
-  </si>
-  <si>
-    <t>ЛГУП-7332</t>
-  </si>
-  <si>
-    <t>Кувалда 1 кг.</t>
-  </si>
-  <si>
-    <t>Ножницы по металлу</t>
-  </si>
-  <si>
-    <t>Ключи обмедненные</t>
-  </si>
-  <si>
-    <t>набор</t>
-  </si>
-  <si>
-    <t>Трещетка ключ 1/2</t>
-  </si>
-  <si>
-    <t>Гайковерт</t>
-  </si>
-  <si>
-    <t>Ключ комбинированные омедненные 41</t>
-  </si>
-  <si>
-    <t>Ключ комбинированные омедненные 36</t>
-  </si>
-  <si>
-    <t>Ключ комбинированные омедненные 30</t>
-  </si>
-  <si>
-    <t>Ключ комбинированные омедненные 24</t>
-  </si>
-  <si>
-    <t>ЛГУП-7428</t>
-  </si>
-  <si>
-    <t>Днище 720х12 ст09Г2С ГОСТ 6533-78</t>
-  </si>
-  <si>
-    <t>Днище 820х14-09Г2С ГОСТ 6533-78</t>
-  </si>
-  <si>
-    <t>Днище 377х10 09Г2С ГОСТ 6533-78</t>
-  </si>
-  <si>
-    <t>Распылитель Тесла Трибо</t>
-  </si>
-  <si>
-    <t>ЛГУП-7429</t>
-  </si>
-  <si>
     <t>ЛГУП-7445</t>
   </si>
   <si>
@@ -159,27 +150,27 @@
     <t>ЛГУП-7447</t>
   </si>
   <si>
+    <t>ЛГУП-7448</t>
+  </si>
+  <si>
+    <t>Блок коммутации 24В БК-24-RS485-01</t>
+  </si>
+  <si>
+    <t>МИП-24 исп.20 (МИП-24-2/П5-Р-RS), до двух АКБ 12 В 17 Ач</t>
+  </si>
+  <si>
+    <t>Держатель проводника Rd8</t>
+  </si>
+  <si>
+    <t>Индикатор положения поплавка ИПП 01.00.000</t>
+  </si>
+  <si>
+    <t>Перемычка и наконечник НКИ 6-0-6</t>
+  </si>
+  <si>
     <t>м</t>
   </si>
   <si>
-    <t>ЛГУП-7448</t>
-  </si>
-  <si>
-    <t>Перемычка и наконечник НКИ 6-0-6</t>
-  </si>
-  <si>
-    <t>Держатель проводника Rd8</t>
-  </si>
-  <si>
-    <t>Индикатор положения поплавка ИПП 01.00.000</t>
-  </si>
-  <si>
-    <t>МИП-24 исп.20 (МИП-24-2/П5-Р-RS), до двух АКБ 12 В 17 Ач</t>
-  </si>
-  <si>
-    <t>Блок коммутации 24В БК-24-RS485-01</t>
-  </si>
-  <si>
     <t>ЛГУП-7450</t>
   </si>
   <si>
@@ -216,28 +207,82 @@
     <t>ЛГУП-7480</t>
   </si>
   <si>
-    <t>00УП-000005</t>
+    <t>ЛГУП-7485</t>
   </si>
   <si>
     <t>Дюбель-молли М6х50</t>
   </si>
   <si>
-    <t>ЛГУП-7485</t>
-  </si>
-  <si>
     <t>Контргайка 20 ГОСТ 8968-75 (12Х18Н10Т)</t>
   </si>
   <si>
-    <t>Удалитель наклеек Lavr Антискотч</t>
-  </si>
-  <si>
-    <t>ЛГУП-7486</t>
-  </si>
-  <si>
-    <t>Кольцо 350-360-58-2-2 ГОСТ 9833-73</t>
-  </si>
-  <si>
-    <t>Смола ЭД-20 ГОСТ 10587-84</t>
+    <t>ЛГУП-7489</t>
+  </si>
+  <si>
+    <t>ЛГУП-7490</t>
+  </si>
+  <si>
+    <t>Сапоги летние</t>
+  </si>
+  <si>
+    <t>НТУП-018048</t>
+  </si>
+  <si>
+    <t>спец одежда летняя</t>
+  </si>
+  <si>
+    <t>ЛГУП-7491</t>
+  </si>
+  <si>
+    <t>м2</t>
+  </si>
+  <si>
+    <t>ЛГУП-7492</t>
+  </si>
+  <si>
+    <t>Лист гладкий 0,5 1250х2500мм RAL полиуретан 9016(белый)</t>
+  </si>
+  <si>
+    <t>ЛГУП-7493</t>
+  </si>
+  <si>
+    <t>ЛГУП-7496</t>
+  </si>
+  <si>
+    <t>ЛГУП-7497</t>
+  </si>
+  <si>
+    <t>ЛГУП-7498</t>
+  </si>
+  <si>
+    <t>Вал ПСМНТ.001.015.000 св.загот (нормализация "стоя" при темп-ре 350-400 град 30 мин и отпуск в печи)</t>
+  </si>
+  <si>
+    <t>ЛГУП-7499</t>
+  </si>
+  <si>
+    <t>Корпус ПСМНТ.001.018.001 (14 скв) - наплавка ПНЖ</t>
+  </si>
+  <si>
+    <t>Крышка ПСМНТ.001.000.001 (заготовка-отливка СЧ14-18 ГОСТ 1412-85)</t>
+  </si>
+  <si>
+    <t>Сегмент ПСМНТ.001.014.000</t>
+  </si>
+  <si>
+    <t>Оцинкование шпилек М16х80 ГОСТ 9066-75</t>
+  </si>
+  <si>
+    <t>ЛГУП-7500</t>
+  </si>
+  <si>
+    <t>Оцинкование шпилек М24х130 ГОСТ 9066-75</t>
+  </si>
+  <si>
+    <t>ЛГУП-7501</t>
+  </si>
+  <si>
+    <t>ЛГУП-7502</t>
   </si>
   <si>
     <t>Маркер черный</t>
@@ -261,219 +306,219 @@
     <t>Фланец х-80-40 ГОСТ12821 (заготовка-поковка ст.20 гр.IV КП 195 ГОСТ 8479-70)</t>
   </si>
   <si>
+    <t>Труба D89х6 ГОСТ 8732-78 Ст.20 ГОСТ 8731-74</t>
+  </si>
+  <si>
+    <t>Труба D108х16 ГОСТ 8732-78/ Ст.40Х  ГОСТ 8731-74</t>
+  </si>
+  <si>
+    <t>Труба D426х50 Ст.20 ГОСТ 8732-78</t>
+  </si>
+  <si>
+    <t>Труба D114х28 ГОСТ 8732-78/ Ст.20 ГОСТ 8731-74</t>
+  </si>
+  <si>
+    <t>Труба D65х14 Ст.20 ГОСТ 8731-74</t>
+  </si>
+  <si>
     <t>Труба D194х14 В20 ГОСТ 8732-78</t>
   </si>
   <si>
-    <t>Труба D426х50 Ст.20 ГОСТ 8732-78</t>
-  </si>
-  <si>
-    <t>Труба D108х16 ГОСТ 8732-78/ Ст.40Х  ГОСТ 8731-74</t>
-  </si>
-  <si>
     <t>Труба D83х9 Ст.40Х ГОСТ 8731-87</t>
   </si>
   <si>
-    <t>Труба D89х6 ГОСТ 8732-78 Ст.20 ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>Труба D65х14 Ст.20 ГОСТ 8731-74</t>
-  </si>
-  <si>
-    <t>Труба D114х28 ГОСТ 8732-78/ Ст.20 ГОСТ 8731-74</t>
+    <t>Корпус металлический ЩМП-3-0 (650х500х220мм) У2 IP54 YKM40-03-54 IEK арт. YKM40-03-54</t>
+  </si>
+  <si>
+    <t>Контроллер доступа "С2000-2"</t>
+  </si>
+  <si>
+    <t>Выключатель автоматический двухполюсный IEK ARMAT M10N 2P B 10А AR-M10N-2-B010</t>
+  </si>
+  <si>
+    <t>Выключатель автоматический двухполюсный 3А B ВА47-29 4.5кА MVA20-2-003-B IEK</t>
+  </si>
+  <si>
+    <t>Шина заземления на DIN-изолятор ШНИ-6х9-8</t>
+  </si>
+  <si>
+    <t>Зажим клеммный винтовой 2,5 мм2 (50/1500/36000) Б0033416 ЭРА арт. Б0033416</t>
+  </si>
+  <si>
+    <t>Заглушка NO-550-07 для винтовых клемм 2,5мм2 арт. Б0035737</t>
+  </si>
+  <si>
+    <t>Фиксатор ФК-102-01 на DIN-рейку 32057DEK Dekraft 2 арт. 32057DEK</t>
+  </si>
+  <si>
+    <t>DIN-рейка 50см перфорированная adr-50 EKF арт. adr-50</t>
+  </si>
+  <si>
+    <t>Разъем РпИм 1.25-5-0.8 плоский</t>
+  </si>
+  <si>
+    <t>Наконечник кабельный НШвИ 0,75мм</t>
+  </si>
+  <si>
+    <t>Коробка клеммная К-СП 08.13.09 24/11П 2КВе-Л-М20(А)-2КВе-Л-М20(В) 1ExeLLCGbXT6 ip66,80х130х90</t>
+  </si>
+  <si>
+    <t>Держатель для полосы заземления К-188 У2 (цинк)</t>
+  </si>
+  <si>
+    <t>MV-клемма проводника Rd8</t>
+  </si>
+  <si>
+    <t>Скоба металлическая СМО 16-17 49152 КВТ</t>
+  </si>
+  <si>
+    <t>Крышка на угол вертикальный внутренний CS 90 100 х 50мм</t>
+  </si>
+  <si>
+    <t>Монтажная рама РВМ 4.1.1</t>
+  </si>
+  <si>
+    <t>Крепление для труб ПВХ с защелкой, 16 мм</t>
+  </si>
+  <si>
+    <t>Ответная рама РВО 4.1.1</t>
+  </si>
+  <si>
+    <t>Уплотнительный модуль МКС 40/Ø 17-34 мм</t>
+  </si>
+  <si>
+    <t>Клемма WAGO 222-415, 5 клеммных зажимов, номинальное сечение проводника 0.08-2.5 мм2</t>
+  </si>
+  <si>
+    <t>Пластина анкерная 120</t>
+  </si>
+  <si>
+    <t>Компрессионный блок МКС КБ 120</t>
+  </si>
+  <si>
+    <t>Уплотнительный модуль МКС 20/Ø 5-14 мм</t>
+  </si>
+  <si>
+    <t>Угол горизонтальный CPO 90 (50 х 50)</t>
   </si>
   <si>
     <t>Металлорукав в ПВХ изоляции РЗ-ЦП-15</t>
   </si>
   <si>
-    <t>Пластина анкерная 120</t>
-  </si>
-  <si>
-    <t>Клемма WAGO 222-415, 5 клеммных зажимов, номинальное сечение проводника 0.08-2.5 мм2</t>
-  </si>
-  <si>
-    <t>Компрессионный блок МКС КБ 120</t>
-  </si>
-  <si>
-    <t>Уплотнительный модуль МКС 20/Ø 5-14 мм</t>
-  </si>
-  <si>
-    <t>Уплотнительный модуль МКС 40/Ø 17-34 мм</t>
-  </si>
-  <si>
-    <t>Ответная рама РВО 4.1.1</t>
-  </si>
-  <si>
-    <t>Монтажная рама РВМ 4.1.1</t>
-  </si>
-  <si>
-    <t>Крышка на угол вертикальный внутренний CS 90 100 х 50мм</t>
+    <t>Короб ПВХ 40х40 мм</t>
+  </si>
+  <si>
+    <t>Короб ПВХ  40х25 мм</t>
+  </si>
+  <si>
+    <t>Кабель ВВГнг(А)-LS-ХЛ 3x2,5 d8мм</t>
+  </si>
+  <si>
+    <t>Кабель ВВГнг(А)-LS-ХЛ 4x1,5 d10,2мм</t>
+  </si>
+  <si>
+    <t>Лента самоклеящаяся уплотнительная ППЭ 5х15 МКС</t>
+  </si>
+  <si>
+    <t>Кабель КВВГЭнг(А)-LS-ХЛ 4х1,0</t>
+  </si>
+  <si>
+    <t>Кабель КВВГЭнг(А)-LS-ХЛ 7х1,0</t>
+  </si>
+  <si>
+    <t>Кабель ВВГнг(А)-LS-ХЛ 3x2,5 d7.2мм</t>
+  </si>
+  <si>
+    <t>Кабель КПСЭнг(A)-FRLS 4х2х0,75</t>
+  </si>
+  <si>
+    <t>Кабель-канал 40х40 перфорированный Plast kk40-40 EKF</t>
+  </si>
+  <si>
+    <t>Провод ПуГВнг(А)-LS 1x0,75</t>
+  </si>
+  <si>
+    <t>Провод ПуГВнг(А)-LS 1x1,5</t>
+  </si>
+  <si>
+    <t>Провод Rd8</t>
+  </si>
+  <si>
+    <t>Крышка Угол горизонтальный CPO 90 (50х50)</t>
+  </si>
+  <si>
+    <t>Угол вертикальный внешний CD 90 (50 х 50)</t>
+  </si>
+  <si>
+    <t>Выключатель двухклавишный IP55</t>
+  </si>
+  <si>
+    <t>Наконечник кабельный НШвИ 1,5мм</t>
+  </si>
+  <si>
+    <t>Наконечник кабельный НШвИ 2,5мм</t>
+  </si>
+  <si>
+    <t>Резьбовой крепежный элемент с наружной резьбой РКН-15 (ММРн-15)</t>
+  </si>
+  <si>
+    <t>Резьбовой крепежный элемент с внутренней резьбой Ркв-15</t>
+  </si>
+  <si>
+    <t>Угол горизонтальный CPO 90 (100 х 50)</t>
+  </si>
+  <si>
+    <t>Крышка Угол горизонтальный CPO 90 (100х50)</t>
+  </si>
+  <si>
+    <t>Угол вертикальный внешний CD 90 (100х50)</t>
+  </si>
+  <si>
+    <t>Крышка на угол вертикальный внешний CD90 (100х50)</t>
   </si>
   <si>
     <t>Угол вертикальный внутренний CS 90 100 х 50мм</t>
   </si>
   <si>
-    <t>Скоба металлическая СМО 16-17 49152 КВТ</t>
-  </si>
-  <si>
-    <t>MV-клемма проводника Rd8</t>
-  </si>
-  <si>
-    <t>Держатель для полосы заземления К-188 У2 (цинк)</t>
-  </si>
-  <si>
-    <t>Коробка клеммная К-СП 08.13.09 24/11П 2КВе-Л-М20(А)-2КВе-Л-М20(В) 1ExeLLCGbXT6 ip66,80х130х90</t>
-  </si>
-  <si>
-    <t>Выключатель двухклавишный IP55</t>
-  </si>
-  <si>
-    <t>Разъем РпИм 1.25-5-0.8 плоский</t>
-  </si>
-  <si>
-    <t>DIN-рейка 50см перфорированная adr-50 EKF арт. adr-50</t>
-  </si>
-  <si>
-    <t>Фиксатор ФК-102-01 на DIN-рейку 32057DEK Dekraft 2 арт. 32057DEK</t>
-  </si>
-  <si>
-    <t>Заглушка NO-550-07 для винтовых клемм 2,5мм2 арт. Б0035737</t>
-  </si>
-  <si>
-    <t>Зажим клеммный винтовой 2,5 мм2 (50/1500/36000) Б0033416 ЭРА арт. Б0033416</t>
-  </si>
-  <si>
-    <t>Шина заземления на DIN-изолятор ШНИ-6х9-8</t>
-  </si>
-  <si>
-    <t>Короб ПВХ 40х40 мм</t>
-  </si>
-  <si>
-    <t>Короб ПВХ  40х25 мм</t>
-  </si>
-  <si>
-    <t>Кабель ВВГнг(А)-LS-ХЛ 3x2,5 d8мм</t>
-  </si>
-  <si>
-    <t>Кабель ВВГнг(А)-LS-ХЛ 4x1,5 d10,2мм</t>
-  </si>
-  <si>
-    <t>Лента самоклеящаяся уплотнительная ППЭ 5х15 МКС</t>
-  </si>
-  <si>
-    <t>Кабель КВВГЭнг(А)-LS-ХЛ 4х1,0</t>
-  </si>
-  <si>
-    <t>Кабель КВВГЭнг(А)-LS-ХЛ 7х1,0</t>
-  </si>
-  <si>
-    <t>Кабель ВВГнг(А)-LS-ХЛ 3x2,5 d7.2мм</t>
-  </si>
-  <si>
-    <t>Кабель КПСЭнг(A)-FRLS 4х2х0,75</t>
-  </si>
-  <si>
-    <t>Кабель-канал 40х40 перфорированный Plast kk40-40 EKF</t>
-  </si>
-  <si>
-    <t>Провод ПуГВнг(А)-LS 1x0,75</t>
-  </si>
-  <si>
-    <t>Провод ПуГВнг(А)-LS 1x1,5</t>
-  </si>
-  <si>
-    <t>Провод Rd8</t>
-  </si>
-  <si>
-    <t>Угол горизонтальный CPO 90 (50 х 50)</t>
-  </si>
-  <si>
-    <t>Наконечник кабельный НШвИ 0,75мм</t>
-  </si>
-  <si>
-    <t>Наконечник кабельный НШвИ 1,5мм</t>
-  </si>
-  <si>
-    <t>Наконечник кабельный НШвИ 2,5мм</t>
-  </si>
-  <si>
-    <t>Крепление для труб ПВХ с защелкой, 16 мм</t>
-  </si>
-  <si>
-    <t>Резьбовой крепежный элемент с наружной резьбой РКН-15 (ММРн-15)</t>
-  </si>
-  <si>
-    <t>Резьбовой крепежный элемент с внутренней резьбой Ркв-15</t>
-  </si>
-  <si>
-    <t>Угол горизонтальный CPO 90 (100 х 50)</t>
-  </si>
-  <si>
-    <t>Крышка Угол горизонтальный CPO 90 (100х50)</t>
-  </si>
-  <si>
-    <t>Угол вертикальный внешний CD 90 (100х50)</t>
-  </si>
-  <si>
-    <t>Крышка на угол вертикальный внешний CD90 (100х50)</t>
-  </si>
-  <si>
-    <t>Крышка Угол горизонтальный CPO 90 (50х50)</t>
-  </si>
-  <si>
-    <t>Выключатель автоматический двухполюсный 3А B ВА47-29 4.5кА MVA20-2-003-B IEK</t>
-  </si>
-  <si>
-    <t>Выключатель автоматический двухполюсный IEK ARMAT M10N 2P B 10А AR-M10N-2-B010</t>
-  </si>
-  <si>
-    <t>Контроллер доступа "С2000-2"</t>
-  </si>
-  <si>
-    <t>Корпус металлический ЩМП-3-0 (650х500х220мм) У2 IP54 YKM40-03-54 IEK арт. YKM40-03-54</t>
+    <t>Крышка на Угол вертикальный внешний CD 90 (50 х 50)</t>
+  </si>
+  <si>
+    <t>Угол вертикальный внутренний CS 90 (50 х 50)</t>
+  </si>
+  <si>
+    <t>Крышка на Угол вертикальный внутренний CS 90 (50 х 50)</t>
+  </si>
+  <si>
+    <t>Считыватель бесконтактный для proxi-карт, Proxy-3МA IP20</t>
   </si>
   <si>
     <t>Карта proximity стандартная ST-PC010EM</t>
   </si>
   <si>
-    <t>Считыватель бесконтактный для proxi-карт, Proxy-3МA IP20</t>
-  </si>
-  <si>
-    <t>Крышка на Угол вертикальный внутренний CS 90 (50 х 50)</t>
-  </si>
-  <si>
-    <t>Угол вертикальный внутренний CS 90 (50 х 50)</t>
-  </si>
-  <si>
-    <t>Крышка на Угол вертикальный внешний CD 90 (50 х 50)</t>
-  </si>
-  <si>
-    <t>Угол вертикальный внешний CD 90 (50 х 50)</t>
+    <t>Кольцо 112-118-36 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Кольцо 080-090-58 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Прокладка медная 8х11-II ГОСТ 19752-84</t>
+  </si>
+  <si>
+    <t>Пружина ПСМНТ.001.000.030</t>
+  </si>
+  <si>
+    <t>Кольцо 080-090-58-2-2 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Кольцо 065-075-58 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Уплотнение ПСМНТ.001.022.002</t>
   </si>
   <si>
     <t>Кольцо 055-060-30-2-2 ГОСТ 9833-73</t>
   </si>
   <si>
-    <t>Кольцо 065-075-58 ГОСТ 9833-73</t>
-  </si>
-  <si>
-    <t>Кольцо 080-090-58-2-2 ГОСТ 9833-73</t>
-  </si>
-  <si>
-    <t>Пружина ПСМНТ.001.000.030</t>
-  </si>
-  <si>
-    <t>Прокладка медная 8х11-II ГОСТ 19752-84</t>
-  </si>
-  <si>
-    <t>Кольцо 080-090-58 ГОСТ 9833-73</t>
-  </si>
-  <si>
-    <t>Кольцо 112-118-36 ГОСТ 9833-73</t>
-  </si>
-  <si>
-    <t>Уплотнение ПСМНТ.001.022.002</t>
-  </si>
-  <si>
     <t>Круг D195 Ст.16ГС-3 ГОСТ 5520-79</t>
   </si>
   <si>
@@ -507,22 +552,109 @@
     <t>Шпилька М18х40.56.019 ГОСТ 22034-76</t>
   </si>
   <si>
+    <t>Заглушка для CP-ML 2 ур. 4мм2 серая IEK YCT23-00-2-K03-004-ZGL IEK</t>
+  </si>
+  <si>
+    <t>Клемма пружинная Push-in CP-ML 2 ур. 4мм2 серая IEK YCT23-00-2-K03-004 IEK</t>
+  </si>
+  <si>
+    <t>Промежуточное реле 2 CO контакта 24в DC</t>
+  </si>
+  <si>
     <t>Розетка для реле 2 СО</t>
   </si>
   <si>
-    <t>Промежуточное реле 2 CO контакта 24в DC</t>
-  </si>
-  <si>
-    <t>Клемма пружинная Push-in CP-ML 2 ур. 4мм2 серая IEK YCT23-00-2-K03-004 IEK</t>
-  </si>
-  <si>
-    <t>Заглушка для CP-ML 2 ур. 4мм2 серая IEK YCT23-00-2-K03-004-ZGL IEK</t>
-  </si>
-  <si>
     <t>Фланец 3-450-40 09Г2С ГОСТ 12815-80 (из поковки гр.IV КП 245 ГОСТ 8479-70)</t>
   </si>
   <si>
     <t>Сгон ДУ20 L-120 12Х18Н10Т</t>
+  </si>
+  <si>
+    <t>Гайка 2М14х1,5 ГОСТ 15522-70</t>
+  </si>
+  <si>
+    <t>Болт М8-6gх25.58.019 ГОСТ 7798-70</t>
+  </si>
+  <si>
+    <t>Гайка М14х1,5 ГОСТ 15522-70</t>
+  </si>
+  <si>
+    <t>Шайба 8 ГОСТ 6402-70</t>
+  </si>
+  <si>
+    <t>Шайба А8 ГОСТ 10450-78</t>
+  </si>
+  <si>
+    <t>Шайба А14 ГОСТ 10450-78</t>
+  </si>
+  <si>
+    <t>Труба D102х5 Ст.20 ГОСТ 8732-78</t>
+  </si>
+  <si>
+    <t>Труба D219х5 Ст.20 ГОСТ 1050-88</t>
+  </si>
+  <si>
+    <t>Труба ДКРПТ 8х1 М2 ГОСТ 617-90 (отгружать L кратно 2,5м, либо бухтами)</t>
+  </si>
+  <si>
+    <t>Круг D160 Ст.3 ГОСТ 535-2005</t>
+  </si>
+  <si>
+    <t>Круг D265 ст.20 ГОСТ 1050-13</t>
+  </si>
+  <si>
+    <t>Круг D26 Ст.3 ГОСТ 535-88</t>
+  </si>
+  <si>
+    <t>Сетка полутомпаковая 008Н Л80 ГОСТ 6613-86</t>
+  </si>
+  <si>
+    <t>Круг D6-h10 ГОСТ 7417-75/ Ст.10 ГОСТ 1051-73</t>
+  </si>
+  <si>
+    <t>Сетка П160 ГОСТ 3187-76</t>
+  </si>
+  <si>
+    <t>Двигатель АИМЛ 63 В4IM3081</t>
+  </si>
+  <si>
+    <t>Полумуфта насоса НТ.3.00.00.00.002 (изготовление шлицов)</t>
+  </si>
+  <si>
+    <t>Полумуфта привода НТ.3.00.00.00.003 (изготовление паза)</t>
+  </si>
+  <si>
+    <t>Картонная коробка - 400 (Д) х 400 (Ш) х 610 (В) мм (картон Т23 ГОСТ 7376-89)</t>
+  </si>
+  <si>
+    <t>Лист А0.М1(анод) 0,5 ГОСТ 21631-76 (черный)</t>
+  </si>
+  <si>
+    <t>Скотч 50мм*120м PROFITTO /6/54 прозрачн</t>
+  </si>
+  <si>
+    <t>Круг D170 Ст.20 ГОСТ 1050-88</t>
+  </si>
+  <si>
+    <t>Тройник 89х6 ст.09Г2С ГОСТ 17376-2001</t>
+  </si>
+  <si>
+    <t>Газоанализатор взрывозащищенный СГОЭС (метан) 1Ex d IIC T4 Gb, IP67 Ур1. 10%, ур.2 50% НКПР</t>
+  </si>
+  <si>
+    <t>Шпилька А1М36-6gx220.09Г2С (оцинк.) ГОСТ 9066-75</t>
+  </si>
+  <si>
+    <t>Гайка М36-6Н ст.09Г2С (оцинк.) ГОСТ 9064-75</t>
+  </si>
+  <si>
+    <t>Кольцо 210-220-58-2-2 ГОСТ 9833-73</t>
+  </si>
+  <si>
+    <t>Грунт-эмаль 2К ПУ, RAL 9003 (белый)</t>
+  </si>
+  <si>
+    <t>Паронит ПОН-Б 1мм</t>
   </si>
 </sst>
 </file>
@@ -959,13 +1091,13 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F146"/>
+  <dimension ref="A1:F175"/>
   <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="11.45" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.1640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="46.6640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="75" style="1" customWidth="1"/>
-    <col min="4" max="4" width="14.1640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="18.6640625" style="1" customWidth="1"/>
     <col min="5" max="5" width="13" style="1" customWidth="1"/>
     <col min="6" max="6" width="14.5" style="1" customWidth="1"/>
   </cols>
@@ -990,16 +1122,16 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>1</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="8" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="D2" s="5">
-        <v>120</v>
+        <v>40</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>6</v>
@@ -1008,19 +1140,19 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>2</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="8" t="s">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="D3" s="5">
-        <v>0.25</v>
+        <v>40</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>7</v>
@@ -1032,16 +1164,16 @@
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="8" t="s">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="D4" s="5">
-        <v>40</v>
+        <v>500</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1050,16 +1182,16 @@
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="8" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D5" s="5">
-        <v>40</v>
+        <v>800</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1068,16 +1200,16 @@
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="8" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D6" s="5">
-        <v>500</v>
+        <v>15</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1086,16 +1218,16 @@
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="8" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D7" s="5">
-        <v>800</v>
+        <v>20</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1110,10 +1242,10 @@
         <v>10</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1125,13 +1257,13 @@
         <v>17</v>
       </c>
       <c r="D9" s="5">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1146,10 +1278,10 @@
         <v>20</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1161,13 +1293,13 @@
         <v>19</v>
       </c>
       <c r="D11" s="5">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1176,16 +1308,16 @@
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="8" t="s">
-        <v>20</v>
+        <v>87</v>
       </c>
       <c r="D12" s="5">
         <v>5</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1194,16 +1326,16 @@
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="8" t="s">
-        <v>72</v>
+        <v>20</v>
       </c>
       <c r="D13" s="5">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1215,13 +1347,13 @@
         <v>21</v>
       </c>
       <c r="D14" s="5">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1230,16 +1362,16 @@
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D15" s="5">
         <v>10</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1248,16 +1380,16 @@
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D16" s="5">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1269,13 +1401,13 @@
         <v>25</v>
       </c>
       <c r="D17" s="5">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1290,10 +1422,10 @@
         <v>10</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1308,10 +1440,10 @@
         <v>10</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1320,16 +1452,16 @@
       </c>
       <c r="B20" s="4"/>
       <c r="C20" s="8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D20" s="5">
         <v>10</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1338,16 +1470,16 @@
       </c>
       <c r="B21" s="4"/>
       <c r="C21" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D21" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1356,16 +1488,16 @@
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D22" s="5">
         <v>10</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1377,13 +1509,13 @@
         <v>32</v>
       </c>
       <c r="D23" s="5">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1395,13 +1527,13 @@
         <v>33</v>
       </c>
       <c r="D24" s="5">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1410,16 +1542,16 @@
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D25" s="5">
+        <v>23</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F25" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="D25" s="5">
-        <v>10</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1428,16 +1560,16 @@
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="8" t="s">
-        <v>73</v>
+        <v>36</v>
       </c>
       <c r="D26" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1446,16 +1578,16 @@
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="8" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="D27" s="5">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1464,70 +1596,70 @@
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="8" t="s">
-        <v>36</v>
+        <v>89</v>
       </c>
       <c r="D28" s="5">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="3">
         <v>28</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="D29" s="5">
+        <v>0.2</v>
+      </c>
+      <c r="E29" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D29" s="5">
-        <v>4</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>11</v>
-      </c>
       <c r="F29" s="4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="3">
         <v>29</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="D30" s="5">
+        <v>53.25</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F30" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D30" s="5">
-        <v>18</v>
-      </c>
-      <c r="E30" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="F30" s="4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="31" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="3">
         <v>30</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="D31" s="5">
+        <v>25</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F31" s="4" t="s">
         <v>39</v>
-      </c>
-      <c r="D31" s="5">
-        <v>1</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="F31" s="4" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1536,16 +1668,16 @@
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="8" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="D32" s="5">
-        <v>0.2</v>
+        <v>49</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1554,16 +1686,16 @@
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="8" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="D33" s="5">
-        <v>53.25</v>
+        <v>18.25</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1572,16 +1704,16 @@
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="D34" s="5">
-        <v>25</v>
+        <v>95</v>
+      </c>
+      <c r="D34" s="7">
+        <v>4286.5</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>6</v>
+        <v>37</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1590,16 +1722,16 @@
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="8" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="D35" s="5">
-        <v>271.75</v>
+        <v>148.5</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1608,16 +1740,16 @@
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="D36" s="7">
-        <v>4286.5</v>
+        <v>97</v>
+      </c>
+      <c r="D36" s="5">
+        <v>37.35</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1626,16 +1758,16 @@
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="8" t="s">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="D37" s="5">
-        <v>18.25</v>
+        <v>271.75</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1644,16 +1776,16 @@
       </c>
       <c r="B38" s="4"/>
       <c r="C38" s="8" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="D38" s="5">
         <v>99.25</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1662,16 +1794,16 @@
       </c>
       <c r="B39" s="4"/>
       <c r="C39" s="8" t="s">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="D39" s="5">
-        <v>49</v>
+        <v>1</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1680,16 +1812,16 @@
       </c>
       <c r="B40" s="4"/>
       <c r="C40" s="8" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="D40" s="5">
-        <v>37.35</v>
+        <v>1</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1698,16 +1830,16 @@
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="8" t="s">
-        <v>84</v>
+        <v>42</v>
       </c>
       <c r="D41" s="5">
-        <v>148.5</v>
+        <v>1</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1716,16 +1848,16 @@
       </c>
       <c r="B42" s="4"/>
       <c r="C42" s="8" t="s">
-        <v>85</v>
+        <v>43</v>
       </c>
       <c r="D42" s="5">
-        <v>130</v>
+        <v>1</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1734,16 +1866,16 @@
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="8" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="D43" s="5">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1752,16 +1884,16 @@
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="8" t="s">
-        <v>46</v>
+        <v>103</v>
       </c>
       <c r="D44" s="5">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1770,16 +1902,16 @@
       </c>
       <c r="B45" s="4"/>
       <c r="C45" s="8" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="D45" s="5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1788,16 +1920,16 @@
       </c>
       <c r="B46" s="4"/>
       <c r="C46" s="8" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="D46" s="5">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1806,16 +1938,16 @@
       </c>
       <c r="B47" s="4"/>
       <c r="C47" s="8" t="s">
-        <v>89</v>
+        <v>106</v>
       </c>
       <c r="D47" s="5">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1824,16 +1956,16 @@
       </c>
       <c r="B48" s="4"/>
       <c r="C48" s="8" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="D48" s="5">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1842,16 +1974,16 @@
       </c>
       <c r="B49" s="4"/>
       <c r="C49" s="8" t="s">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="D49" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E49" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1860,16 +1992,16 @@
       </c>
       <c r="B50" s="4"/>
       <c r="C50" s="8" t="s">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="D50" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1878,16 +2010,16 @@
       </c>
       <c r="B51" s="4"/>
       <c r="C51" s="8" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="D51" s="5">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1896,16 +2028,16 @@
       </c>
       <c r="B52" s="4"/>
       <c r="C52" s="8" t="s">
-        <v>94</v>
+        <v>111</v>
       </c>
       <c r="D52" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1914,16 +2046,16 @@
       </c>
       <c r="B53" s="4"/>
       <c r="C53" s="8" t="s">
-        <v>95</v>
+        <v>112</v>
       </c>
       <c r="D53" s="5">
-        <v>135</v>
+        <v>50</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1932,16 +2064,16 @@
       </c>
       <c r="B54" s="4"/>
       <c r="C54" s="8" t="s">
-        <v>96</v>
+        <v>44</v>
       </c>
       <c r="D54" s="5">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="55" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1950,16 +2082,16 @@
       </c>
       <c r="B55" s="4"/>
       <c r="C55" s="8" t="s">
-        <v>47</v>
+        <v>113</v>
       </c>
       <c r="D55" s="5">
-        <v>70</v>
+        <v>4</v>
       </c>
       <c r="E55" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="56" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1968,16 +2100,16 @@
       </c>
       <c r="B56" s="4"/>
       <c r="C56" s="8" t="s">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="D56" s="5">
-        <v>50</v>
+        <v>135</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="57" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -1986,16 +2118,16 @@
       </c>
       <c r="B57" s="4"/>
       <c r="C57" s="8" t="s">
-        <v>98</v>
+        <v>115</v>
       </c>
       <c r="D57" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E57" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="58" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2004,7 +2136,7 @@
       </c>
       <c r="B58" s="4"/>
       <c r="C58" s="8" t="s">
-        <v>99</v>
+        <v>116</v>
       </c>
       <c r="D58" s="5">
         <v>1</v>
@@ -2013,7 +2145,7 @@
         <v>6</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2022,16 +2154,16 @@
       </c>
       <c r="B59" s="4"/>
       <c r="C59" s="8" t="s">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="D59" s="5">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="E59" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="60" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2040,16 +2172,16 @@
       </c>
       <c r="B60" s="4"/>
       <c r="C60" s="8" t="s">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="D60" s="5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="61" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2058,16 +2190,16 @@
       </c>
       <c r="B61" s="4"/>
       <c r="C61" s="8" t="s">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="D61" s="5">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E61" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="62" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2076,16 +2208,16 @@
       </c>
       <c r="B62" s="4"/>
       <c r="C62" s="8" t="s">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="D62" s="5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="63" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2094,16 +2226,16 @@
       </c>
       <c r="B63" s="4"/>
       <c r="C63" s="8" t="s">
-        <v>104</v>
+        <v>45</v>
       </c>
       <c r="D63" s="5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E63" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="64" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2112,16 +2244,16 @@
       </c>
       <c r="B64" s="4"/>
       <c r="C64" s="8" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="D64" s="5">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="65" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2130,16 +2262,16 @@
       </c>
       <c r="B65" s="4"/>
       <c r="C65" s="8" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="D65" s="5">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="66" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2148,16 +2280,16 @@
       </c>
       <c r="B66" s="4"/>
       <c r="C66" s="8" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="D66" s="5">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="67" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2166,16 +2298,16 @@
       </c>
       <c r="B67" s="4"/>
       <c r="C67" s="8" t="s">
-        <v>108</v>
+        <v>46</v>
       </c>
       <c r="D67" s="5">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="68" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2184,16 +2316,16 @@
       </c>
       <c r="B68" s="4"/>
       <c r="C68" s="8" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="D68" s="5">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="69" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2202,16 +2334,16 @@
       </c>
       <c r="B69" s="4"/>
       <c r="C69" s="8" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="D69" s="5">
-        <v>2.1</v>
+        <v>130</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="70" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2220,16 +2352,16 @@
       </c>
       <c r="B70" s="4"/>
       <c r="C70" s="8" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="D70" s="5">
-        <v>112</v>
+        <v>8</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="71" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2238,16 +2370,16 @@
       </c>
       <c r="B71" s="4"/>
       <c r="C71" s="8" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="D71" s="5">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="E71" s="6" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="72" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2256,16 +2388,16 @@
       </c>
       <c r="B72" s="4"/>
       <c r="C72" s="8" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="D72" s="5">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="73" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2274,16 +2406,16 @@
       </c>
       <c r="B73" s="4"/>
       <c r="C73" s="8" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
       <c r="D73" s="5">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E73" s="6" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="74" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2292,16 +2424,16 @@
       </c>
       <c r="B74" s="4"/>
       <c r="C74" s="8" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="D74" s="5">
-        <v>1</v>
+        <v>2.1</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="75" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2310,16 +2442,16 @@
       </c>
       <c r="B75" s="4"/>
       <c r="C75" s="8" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="D75" s="5">
-        <v>2</v>
+        <v>112</v>
       </c>
       <c r="E75" s="6" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="76" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2328,16 +2460,16 @@
       </c>
       <c r="B76" s="4"/>
       <c r="C76" s="8" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="D76" s="5">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="77" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2346,16 +2478,16 @@
       </c>
       <c r="B77" s="4"/>
       <c r="C77" s="8" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
       <c r="D77" s="5">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="E77" s="6" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="78" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2364,16 +2496,16 @@
       </c>
       <c r="B78" s="4"/>
       <c r="C78" s="8" t="s">
-        <v>48</v>
+        <v>134</v>
       </c>
       <c r="D78" s="5">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="F78" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="79" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2382,16 +2514,16 @@
       </c>
       <c r="B79" s="4"/>
       <c r="C79" s="8" t="s">
-        <v>119</v>
+        <v>135</v>
       </c>
       <c r="D79" s="5">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E79" s="6" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="F79" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="80" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2400,16 +2532,16 @@
       </c>
       <c r="B80" s="4"/>
       <c r="C80" s="8" t="s">
-        <v>120</v>
+        <v>136</v>
       </c>
       <c r="D80" s="5">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="81" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2418,16 +2550,16 @@
       </c>
       <c r="B81" s="4"/>
       <c r="C81" s="8" t="s">
-        <v>121</v>
+        <v>137</v>
       </c>
       <c r="D81" s="5">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E81" s="6" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="82" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2436,16 +2568,16 @@
       </c>
       <c r="B82" s="4"/>
       <c r="C82" s="8" t="s">
-        <v>122</v>
+        <v>138</v>
       </c>
       <c r="D82" s="5">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="83" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2454,16 +2586,16 @@
       </c>
       <c r="B83" s="4"/>
       <c r="C83" s="8" t="s">
-        <v>123</v>
+        <v>139</v>
       </c>
       <c r="D83" s="5">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="E83" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F83" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="84" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2472,16 +2604,16 @@
       </c>
       <c r="B84" s="4"/>
       <c r="C84" s="8" t="s">
-        <v>124</v>
+        <v>140</v>
       </c>
       <c r="D84" s="5">
-        <v>39</v>
+        <v>8</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="85" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2490,16 +2622,16 @@
       </c>
       <c r="B85" s="4"/>
       <c r="C85" s="8" t="s">
-        <v>125</v>
+        <v>141</v>
       </c>
       <c r="D85" s="5">
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="E85" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F85" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="86" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2508,16 +2640,16 @@
       </c>
       <c r="B86" s="4"/>
       <c r="C86" s="8" t="s">
-        <v>126</v>
+        <v>142</v>
       </c>
       <c r="D86" s="5">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="87" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2526,16 +2658,16 @@
       </c>
       <c r="B87" s="4"/>
       <c r="C87" s="8" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
       <c r="D87" s="5">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="E87" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="88" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2544,16 +2676,16 @@
       </c>
       <c r="B88" s="4"/>
       <c r="C88" s="8" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="D88" s="5">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="89" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2562,16 +2694,16 @@
       </c>
       <c r="B89" s="4"/>
       <c r="C89" s="8" t="s">
-        <v>129</v>
+        <v>145</v>
       </c>
       <c r="D89" s="5">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="E89" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="90" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2580,16 +2712,16 @@
       </c>
       <c r="B90" s="4"/>
       <c r="C90" s="8" t="s">
-        <v>130</v>
+        <v>146</v>
       </c>
       <c r="D90" s="5">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="91" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2598,16 +2730,16 @@
       </c>
       <c r="B91" s="4"/>
       <c r="C91" s="8" t="s">
-        <v>131</v>
+        <v>147</v>
       </c>
       <c r="D91" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E91" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="92" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2616,16 +2748,16 @@
       </c>
       <c r="B92" s="4"/>
       <c r="C92" s="8" t="s">
-        <v>132</v>
+        <v>148</v>
       </c>
       <c r="D92" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="93" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2634,16 +2766,16 @@
       </c>
       <c r="B93" s="4"/>
       <c r="C93" s="8" t="s">
-        <v>49</v>
+        <v>149</v>
       </c>
       <c r="D93" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E93" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="94" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2652,16 +2784,16 @@
       </c>
       <c r="B94" s="4"/>
       <c r="C94" s="8" t="s">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="D94" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="95" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2670,16 +2802,16 @@
       </c>
       <c r="B95" s="4"/>
       <c r="C95" s="8" t="s">
-        <v>133</v>
+        <v>151</v>
       </c>
       <c r="D95" s="5">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E95" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F95" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="96" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2688,16 +2820,16 @@
       </c>
       <c r="B96" s="4"/>
       <c r="C96" s="8" t="s">
-        <v>134</v>
+        <v>152</v>
       </c>
       <c r="D96" s="5">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F96" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="97" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2706,16 +2838,16 @@
       </c>
       <c r="B97" s="4"/>
       <c r="C97" s="8" t="s">
-        <v>135</v>
+        <v>153</v>
       </c>
       <c r="D97" s="5">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E97" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="98" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2724,7 +2856,7 @@
       </c>
       <c r="B98" s="4"/>
       <c r="C98" s="8" t="s">
-        <v>136</v>
+        <v>154</v>
       </c>
       <c r="D98" s="5">
         <v>1</v>
@@ -2733,7 +2865,7 @@
         <v>6</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="99" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2742,16 +2874,16 @@
       </c>
       <c r="B99" s="4"/>
       <c r="C99" s="8" t="s">
-        <v>137</v>
+        <v>155</v>
       </c>
       <c r="D99" s="5">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E99" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="100" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2760,16 +2892,16 @@
       </c>
       <c r="B100" s="4"/>
       <c r="C100" s="8" t="s">
-        <v>138</v>
+        <v>156</v>
       </c>
       <c r="D100" s="5">
-        <v>8</v>
+        <v>50</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F100" s="4" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="101" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2778,16 +2910,16 @@
       </c>
       <c r="B101" s="4"/>
       <c r="C101" s="8" t="s">
-        <v>139</v>
+        <v>157</v>
       </c>
       <c r="D101" s="5">
-        <v>8</v>
+        <v>80</v>
       </c>
       <c r="E101" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F101" s="4" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="102" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2796,16 +2928,16 @@
       </c>
       <c r="B102" s="4"/>
       <c r="C102" s="8" t="s">
-        <v>140</v>
+        <v>158</v>
       </c>
       <c r="D102" s="5">
-        <v>8</v>
+        <v>50</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F102" s="4" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="103" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2814,7 +2946,7 @@
       </c>
       <c r="B103" s="4"/>
       <c r="C103" s="8" t="s">
-        <v>141</v>
+        <v>159</v>
       </c>
       <c r="D103" s="5">
         <v>25</v>
@@ -2823,7 +2955,7 @@
         <v>6</v>
       </c>
       <c r="F103" s="4" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="104" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2832,16 +2964,16 @@
       </c>
       <c r="B104" s="4"/>
       <c r="C104" s="8" t="s">
-        <v>142</v>
+        <v>160</v>
       </c>
       <c r="D104" s="5">
-        <v>170</v>
+        <v>25</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F104" s="4" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="105" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2850,16 +2982,16 @@
       </c>
       <c r="B105" s="4"/>
       <c r="C105" s="8" t="s">
-        <v>143</v>
+        <v>161</v>
       </c>
       <c r="D105" s="5">
-        <v>25</v>
+        <v>170</v>
       </c>
       <c r="E105" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F105" s="4" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="106" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2868,16 +3000,16 @@
       </c>
       <c r="B106" s="4"/>
       <c r="C106" s="8" t="s">
-        <v>144</v>
+        <v>162</v>
       </c>
       <c r="D106" s="5">
         <v>25</v>
       </c>
       <c r="E106" s="6" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F106" s="4" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="107" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2886,67 +3018,67 @@
       </c>
       <c r="B107" s="4"/>
       <c r="C107" s="8" t="s">
-        <v>145</v>
+        <v>163</v>
       </c>
       <c r="D107" s="5">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="E107" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F107" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="3">
         <v>107</v>
       </c>
       <c r="B108" s="4"/>
       <c r="C108" s="8" t="s">
-        <v>146</v>
+        <v>49</v>
       </c>
       <c r="D108" s="5">
-        <v>80</v>
+        <v>1</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F108" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="3">
         <v>108</v>
       </c>
       <c r="B109" s="4"/>
       <c r="C109" s="8" t="s">
-        <v>147</v>
+        <v>164</v>
       </c>
       <c r="D109" s="5">
-        <v>50</v>
+        <v>291</v>
       </c>
       <c r="E109" s="6" t="s">
-        <v>6</v>
+        <v>37</v>
       </c>
       <c r="F109" s="4" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="110" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="3">
         <v>109</v>
       </c>
       <c r="B110" s="4"/>
       <c r="C110" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="D110" s="5">
-        <v>25</v>
+        <v>165</v>
+      </c>
+      <c r="D110" s="7">
+        <v>1415.25</v>
       </c>
       <c r="E110" s="6" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="F110" s="4" t="s">
         <v>51</v>
@@ -2958,16 +3090,16 @@
       </c>
       <c r="B111" s="4"/>
       <c r="C111" s="8" t="s">
-        <v>52</v>
+        <v>166</v>
       </c>
       <c r="D111" s="5">
-        <v>1</v>
+        <v>26.5</v>
       </c>
       <c r="E111" s="6" t="s">
-        <v>6</v>
+        <v>37</v>
       </c>
       <c r="F111" s="4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="112" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2976,16 +3108,16 @@
       </c>
       <c r="B112" s="4"/>
       <c r="C112" s="8" t="s">
-        <v>149</v>
+        <v>167</v>
       </c>
       <c r="D112" s="5">
-        <v>291</v>
+        <v>131</v>
       </c>
       <c r="E112" s="6" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="F112" s="4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="113" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2994,16 +3126,16 @@
       </c>
       <c r="B113" s="4"/>
       <c r="C113" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="D113" s="7">
-        <v>1415.25</v>
+        <v>168</v>
+      </c>
+      <c r="D113" s="5">
+        <v>950</v>
       </c>
       <c r="E113" s="6" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="F113" s="4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="114" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3012,16 +3144,16 @@
       </c>
       <c r="B114" s="4"/>
       <c r="C114" s="8" t="s">
-        <v>151</v>
+        <v>169</v>
       </c>
       <c r="D114" s="5">
-        <v>26.5</v>
+        <v>2.5</v>
       </c>
       <c r="E114" s="6" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="F114" s="4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="115" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3030,70 +3162,70 @@
       </c>
       <c r="B115" s="4"/>
       <c r="C115" s="8" t="s">
-        <v>152</v>
+        <v>170</v>
       </c>
       <c r="D115" s="5">
-        <v>131</v>
+        <v>1.5</v>
       </c>
       <c r="E115" s="6" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="F115" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="116" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="3">
         <v>115</v>
       </c>
       <c r="B116" s="4"/>
       <c r="C116" s="8" t="s">
-        <v>153</v>
+        <v>171</v>
       </c>
       <c r="D116" s="5">
-        <v>950</v>
+        <v>25</v>
       </c>
       <c r="E116" s="6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F116" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="117" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="3">
         <v>116</v>
       </c>
       <c r="B117" s="4"/>
       <c r="C117" s="8" t="s">
-        <v>154</v>
+        <v>172</v>
       </c>
       <c r="D117" s="5">
-        <v>2.5</v>
+        <v>100</v>
       </c>
       <c r="E117" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F117" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="118" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="3">
         <v>117</v>
       </c>
       <c r="B118" s="4"/>
       <c r="C118" s="8" t="s">
-        <v>155</v>
+        <v>173</v>
       </c>
       <c r="D118" s="5">
-        <v>1.5</v>
+        <v>50</v>
       </c>
       <c r="E118" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F118" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="119" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3102,16 +3234,16 @@
       </c>
       <c r="B119" s="4"/>
       <c r="C119" s="8" t="s">
-        <v>156</v>
+        <v>174</v>
       </c>
       <c r="D119" s="5">
-        <v>25</v>
+        <v>500</v>
       </c>
       <c r="E119" s="6" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="F119" s="4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="120" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3120,16 +3252,16 @@
       </c>
       <c r="B120" s="4"/>
       <c r="C120" s="8" t="s">
-        <v>157</v>
+        <v>53</v>
       </c>
       <c r="D120" s="5">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="E120" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F120" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="121" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3138,16 +3270,16 @@
       </c>
       <c r="B121" s="4"/>
       <c r="C121" s="8" t="s">
-        <v>158</v>
+        <v>55</v>
       </c>
       <c r="D121" s="5">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="E121" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F121" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="122" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3156,16 +3288,16 @@
       </c>
       <c r="B122" s="4"/>
       <c r="C122" s="8" t="s">
-        <v>159</v>
+        <v>57</v>
       </c>
       <c r="D122" s="5">
-        <v>500</v>
+        <v>20</v>
       </c>
       <c r="E122" s="6" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="F122" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="123" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3174,16 +3306,16 @@
       </c>
       <c r="B123" s="4"/>
       <c r="C123" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="D123" s="5">
+        <v>6</v>
+      </c>
+      <c r="E123" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F123" s="4" t="s">
         <v>56</v>
-      </c>
-      <c r="D123" s="5">
-        <v>1</v>
-      </c>
-      <c r="E123" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="F123" s="4" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="124" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3192,16 +3324,16 @@
       </c>
       <c r="B124" s="4"/>
       <c r="C124" s="8" t="s">
-        <v>58</v>
+        <v>176</v>
       </c>
       <c r="D124" s="5">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="E124" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F124" s="4" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="125" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3210,7 +3342,7 @@
       </c>
       <c r="B125" s="4"/>
       <c r="C125" s="8" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
       <c r="D125" s="5">
         <v>3</v>
@@ -3219,7 +3351,7 @@
         <v>6</v>
       </c>
       <c r="F125" s="4" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="126" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3228,7 +3360,7 @@
       </c>
       <c r="B126" s="4"/>
       <c r="C126" s="8" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
       <c r="D126" s="5">
         <v>3</v>
@@ -3237,7 +3369,7 @@
         <v>6</v>
       </c>
       <c r="F126" s="4" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="127" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3246,16 +3378,16 @@
       </c>
       <c r="B127" s="4"/>
       <c r="C127" s="8" t="s">
-        <v>162</v>
+        <v>57</v>
       </c>
       <c r="D127" s="5">
-        <v>16</v>
+        <v>60</v>
       </c>
       <c r="E127" s="6" t="s">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="F127" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="128" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3264,16 +3396,16 @@
       </c>
       <c r="B128" s="4"/>
       <c r="C128" s="8" t="s">
-        <v>163</v>
+        <v>55</v>
       </c>
       <c r="D128" s="5">
-        <v>6</v>
+        <v>120</v>
       </c>
       <c r="E128" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F128" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="129" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3282,16 +3414,16 @@
       </c>
       <c r="B129" s="4"/>
       <c r="C129" s="8" t="s">
-        <v>60</v>
+        <v>175</v>
       </c>
       <c r="D129" s="5">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E129" s="6" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="F129" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="130" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3300,16 +3432,16 @@
       </c>
       <c r="B130" s="4"/>
       <c r="C130" s="8" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
       <c r="D130" s="5">
-        <v>9</v>
+        <v>48</v>
       </c>
       <c r="E130" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F130" s="4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="131" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3318,7 +3450,7 @@
       </c>
       <c r="B131" s="4"/>
       <c r="C131" s="8" t="s">
-        <v>161</v>
+        <v>177</v>
       </c>
       <c r="D131" s="5">
         <v>9</v>
@@ -3327,7 +3459,7 @@
         <v>6</v>
       </c>
       <c r="F131" s="4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="132" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3336,16 +3468,16 @@
       </c>
       <c r="B132" s="4"/>
       <c r="C132" s="8" t="s">
-        <v>162</v>
+        <v>178</v>
       </c>
       <c r="D132" s="5">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="E132" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F132" s="4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="133" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3354,16 +3486,16 @@
       </c>
       <c r="B133" s="4"/>
       <c r="C133" s="8" t="s">
-        <v>60</v>
+        <v>179</v>
       </c>
       <c r="D133" s="5">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="E133" s="6" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="F133" s="4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="134" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3372,16 +3504,16 @@
       </c>
       <c r="B134" s="4"/>
       <c r="C134" s="8" t="s">
-        <v>58</v>
+        <v>180</v>
       </c>
       <c r="D134" s="5">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="E134" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F134" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="135" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3390,16 +3522,16 @@
       </c>
       <c r="B135" s="4"/>
       <c r="C135" s="8" t="s">
-        <v>163</v>
+        <v>61</v>
       </c>
       <c r="D135" s="5">
-        <v>18</v>
+        <v>250</v>
       </c>
       <c r="E135" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F135" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="136" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3408,28 +3540,28 @@
       </c>
       <c r="B136" s="4"/>
       <c r="C136" s="8" t="s">
-        <v>164</v>
+        <v>62</v>
       </c>
       <c r="D136" s="5">
-        <v>15</v>
+        <v>300</v>
       </c>
       <c r="E136" s="6" t="s">
         <v>6</v>
       </c>
       <c r="F136" s="4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="137" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="3">
         <v>136</v>
       </c>
       <c r="B137" s="4"/>
       <c r="C137" s="8" t="s">
-        <v>58</v>
+        <v>181</v>
       </c>
       <c r="D137" s="5">
-        <v>160</v>
+        <v>9</v>
       </c>
       <c r="E137" s="6" t="s">
         <v>6</v>
@@ -3438,16 +3570,16 @@
         <v>63</v>
       </c>
     </row>
-    <row r="138" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="3">
         <v>137</v>
       </c>
       <c r="B138" s="4"/>
       <c r="C138" s="8" t="s">
-        <v>160</v>
+        <v>182</v>
       </c>
       <c r="D138" s="5">
-        <v>12</v>
+        <v>72</v>
       </c>
       <c r="E138" s="6" t="s">
         <v>6</v>
@@ -3456,16 +3588,16 @@
         <v>63</v>
       </c>
     </row>
-    <row r="139" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="3">
         <v>138</v>
       </c>
       <c r="B139" s="4"/>
       <c r="C139" s="8" t="s">
-        <v>161</v>
+        <v>183</v>
       </c>
       <c r="D139" s="5">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="E139" s="6" t="s">
         <v>6</v>
@@ -3474,16 +3606,16 @@
         <v>63</v>
       </c>
     </row>
-    <row r="140" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" s="3">
         <v>139</v>
       </c>
       <c r="B140" s="4"/>
       <c r="C140" s="8" t="s">
-        <v>162</v>
+        <v>184</v>
       </c>
       <c r="D140" s="5">
-        <v>64</v>
+        <v>126</v>
       </c>
       <c r="E140" s="6" t="s">
         <v>6</v>
@@ -3492,16 +3624,16 @@
         <v>63</v>
       </c>
     </row>
-    <row r="141" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="3">
         <v>140</v>
       </c>
       <c r="B141" s="4"/>
       <c r="C141" s="8" t="s">
-        <v>163</v>
+        <v>185</v>
       </c>
       <c r="D141" s="5">
-        <v>24</v>
+        <v>126</v>
       </c>
       <c r="E141" s="6" t="s">
         <v>6</v>
@@ -3510,94 +3642,616 @@
         <v>63</v>
       </c>
     </row>
-    <row r="142" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" s="3">
         <v>141</v>
       </c>
       <c r="B142" s="4"/>
       <c r="C142" s="8" t="s">
-        <v>60</v>
+        <v>186</v>
       </c>
       <c r="D142" s="5">
-        <v>80</v>
+        <v>18</v>
       </c>
       <c r="E142" s="6" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="F142" s="4" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="143" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" s="3">
         <v>142</v>
       </c>
       <c r="B143" s="4"/>
       <c r="C143" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="D143" s="5">
+        <v>5.76</v>
+      </c>
+      <c r="E143" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F143" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D143" s="5">
-        <v>250</v>
-      </c>
-      <c r="E143" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="F143" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="144" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="144" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144" s="3">
         <v>143</v>
       </c>
       <c r="B144" s="4"/>
       <c r="C144" s="8" t="s">
-        <v>165</v>
+        <v>188</v>
       </c>
       <c r="D144" s="5">
-        <v>150</v>
+        <v>40.14</v>
       </c>
       <c r="E144" s="6" t="s">
-        <v>6</v>
+        <v>37</v>
       </c>
       <c r="F144" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="145" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="3">
         <v>144</v>
       </c>
       <c r="B145" s="4"/>
       <c r="C145" s="8" t="s">
-        <v>66</v>
+        <v>189</v>
       </c>
       <c r="D145" s="5">
-        <v>300</v>
+        <v>4.41</v>
       </c>
       <c r="E145" s="6" t="s">
-        <v>6</v>
+        <v>37</v>
       </c>
       <c r="F145" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="146" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" s="3">
         <v>145</v>
       </c>
       <c r="B146" s="4"/>
       <c r="C146" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="D146" s="5">
+        <v>1</v>
+      </c>
+      <c r="E146" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F146" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A147" s="3">
+        <v>146</v>
+      </c>
+      <c r="B147" s="4"/>
+      <c r="C147" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="D146" s="5">
-        <v>5</v>
-      </c>
-      <c r="E146" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="F146" s="4" t="s">
+      <c r="D147" s="5">
+        <v>1</v>
+      </c>
+      <c r="E147" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F147" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A148" s="3">
+        <v>147</v>
+      </c>
+      <c r="B148" s="4"/>
+      <c r="C148" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="D148" s="5">
+        <v>28.44</v>
+      </c>
+      <c r="E148" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F148" s="4" t="s">
         <v>68</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A149" s="3">
+        <v>148</v>
+      </c>
+      <c r="B149" s="4"/>
+      <c r="C149" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="D149" s="5">
+        <v>99</v>
+      </c>
+      <c r="E149" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F149" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A150" s="3">
+        <v>149</v>
+      </c>
+      <c r="B150" s="4"/>
+      <c r="C150" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="D150" s="5">
+        <v>1.71</v>
+      </c>
+      <c r="E150" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F150" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A151" s="3">
+        <v>150</v>
+      </c>
+      <c r="B151" s="4"/>
+      <c r="C151" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="D151" s="5">
+        <v>0.09</v>
+      </c>
+      <c r="E151" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F151" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A152" s="3">
+        <v>151</v>
+      </c>
+      <c r="B152" s="4"/>
+      <c r="C152" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="D152" s="5">
+        <v>0.36</v>
+      </c>
+      <c r="E152" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F152" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A153" s="3">
+        <v>152</v>
+      </c>
+      <c r="B153" s="4"/>
+      <c r="C153" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="D153" s="5">
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="E153" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F153" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A154" s="3">
+        <v>153</v>
+      </c>
+      <c r="B154" s="4"/>
+      <c r="C154" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="D154" s="5">
+        <v>9</v>
+      </c>
+      <c r="E154" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F154" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A155" s="3">
+        <v>154</v>
+      </c>
+      <c r="B155" s="4"/>
+      <c r="C155" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="D155" s="5">
+        <v>9</v>
+      </c>
+      <c r="E155" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F155" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A156" s="3">
+        <v>155</v>
+      </c>
+      <c r="B156" s="4"/>
+      <c r="C156" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="D156" s="5">
+        <v>9</v>
+      </c>
+      <c r="E156" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F156" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A157" s="3">
+        <v>156</v>
+      </c>
+      <c r="B157" s="4"/>
+      <c r="C157" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="D157" s="5">
+        <v>9</v>
+      </c>
+      <c r="E157" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F157" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A158" s="3">
+        <v>157</v>
+      </c>
+      <c r="B158" s="4"/>
+      <c r="C158" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="D158" s="5">
+        <v>1</v>
+      </c>
+      <c r="E158" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F158" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="159" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A159" s="3">
+        <v>158</v>
+      </c>
+      <c r="B159" s="4"/>
+      <c r="C159" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="D159" s="5">
+        <v>9</v>
+      </c>
+      <c r="E159" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F159" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A160" s="3">
+        <v>159</v>
+      </c>
+      <c r="B160" s="4"/>
+      <c r="C160" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="D160" s="5">
+        <v>29.72</v>
+      </c>
+      <c r="E160" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F160" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A161" s="3">
+        <v>160</v>
+      </c>
+      <c r="B161" s="4"/>
+      <c r="C161" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="D161" s="5">
+        <v>8</v>
+      </c>
+      <c r="E161" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F161" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A162" s="3">
+        <v>161</v>
+      </c>
+      <c r="B162" s="4"/>
+      <c r="C162" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="D162" s="5">
+        <v>3</v>
+      </c>
+      <c r="E162" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F162" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A163" s="3">
+        <v>162</v>
+      </c>
+      <c r="B163" s="4"/>
+      <c r="C163" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="D163" s="5">
+        <v>10</v>
+      </c>
+      <c r="E163" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F163" s="4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A164" s="3">
+        <v>163</v>
+      </c>
+      <c r="B164" s="4"/>
+      <c r="C164" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="D164" s="5">
+        <v>18</v>
+      </c>
+      <c r="E164" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F164" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A165" s="3">
+        <v>164</v>
+      </c>
+      <c r="B165" s="4"/>
+      <c r="C165" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="D165" s="5">
+        <v>80</v>
+      </c>
+      <c r="E165" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F165" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A166" s="3">
+        <v>165</v>
+      </c>
+      <c r="B166" s="4"/>
+      <c r="C166" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="D166" s="5">
+        <v>160</v>
+      </c>
+      <c r="E166" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F166" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="167" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A167" s="3">
+        <v>166</v>
+      </c>
+      <c r="B167" s="4"/>
+      <c r="C167" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="D167" s="5">
+        <v>10</v>
+      </c>
+      <c r="E167" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F167" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A168" s="3">
+        <v>167</v>
+      </c>
+      <c r="B168" s="4"/>
+      <c r="C168" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="D168" s="5">
+        <v>10</v>
+      </c>
+      <c r="E168" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F168" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="169" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A169" s="3">
+        <v>168</v>
+      </c>
+      <c r="B169" s="4"/>
+      <c r="C169" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D169" s="5">
+        <v>10</v>
+      </c>
+      <c r="E169" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F169" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="170" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A170" s="3">
+        <v>169</v>
+      </c>
+      <c r="B170" s="4"/>
+      <c r="C170" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="D170" s="5">
+        <v>10</v>
+      </c>
+      <c r="E170" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F170" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="171" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A171" s="3">
+        <v>170</v>
+      </c>
+      <c r="B171" s="4"/>
+      <c r="C171" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="D171" s="5">
+        <v>932</v>
+      </c>
+      <c r="E171" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F171" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="172" spans="1:6" ht="23.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A172" s="3">
+        <v>171</v>
+      </c>
+      <c r="B172" s="4"/>
+      <c r="C172" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="D172" s="7">
+        <v>1192</v>
+      </c>
+      <c r="E172" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F172" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A173" s="3">
+        <v>172</v>
+      </c>
+      <c r="B173" s="4"/>
+      <c r="C173" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="D173" s="5">
+        <v>0.18</v>
+      </c>
+      <c r="E173" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F173" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="174" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A174" s="3">
+        <v>173</v>
+      </c>
+      <c r="B174" s="4"/>
+      <c r="C174" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="D174" s="5">
+        <v>27</v>
+      </c>
+      <c r="E174" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F174" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="175" spans="1:6" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A175" s="3">
+        <v>174</v>
+      </c>
+      <c r="B175" s="4"/>
+      <c r="C175" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="D175" s="5">
+        <v>30</v>
+      </c>
+      <c r="E175" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F175" s="4" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>